<commit_message>
Rewrite ingredient book lines around concrete moments
- All 83 Mind/Gentle lines rewritten so ingredients in the most
  crowded cell read differently
- 45 other lines rewritten that named a hidden keyword outright
- Medium twins (red thread/ink/paint etc.) get their own lines
- Spellbook: book-line writing rule

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -85,7 +85,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Draft text for the books. It hints at target and strength in prose, never as a tag.</t>
+          <t xml:space="preserve">Draft text for the books. It hints at target and strength through a situation, never as a tag, and never names a hidden keyword (the words the player fills into the blanks).</t>
         </r>
       </text>
     </comment>
@@ -164,7 +164,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9842" uniqueCount="2330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9842" uniqueCount="2335">
   <si>
     <t xml:space="preserve">Image Asset Tracker</t>
   </si>
@@ -4177,7 +4177,7 @@
     <t xml:space="preserve">Gentle</t>
   </si>
   <si>
-    <t xml:space="preserve">Draws the mind inward, soft as moonlight. For dreams and for letting go.</t>
+    <t xml:space="preserve">Drink it by the window before bed. It loosens what the day left behind and carries you somewhere far.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,dreams,intuition,release</t>
@@ -4189,7 +4189,7 @@
     <t xml:space="preserve">Strong</t>
   </si>
   <si>
-    <t xml:space="preserve">Bright and bold. Pours courage straight into the heart.</t>
+    <t xml:space="preserve">Bright and bold. Pours nerve straight into the heart.</t>
   </si>
   <si>
     <t xml:space="preserve">confidence,courage,energy,joy,success</t>
@@ -4234,7 +4234,7 @@
     <t xml:space="preserve">love, beauty, self-love, confidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Softens the heart, toward others and toward yourself.</t>
+    <t xml:space="preserve">A splash on the face before the mirror, to be kinder to whoever looks back.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,confidence,love,self-love</t>
@@ -4243,7 +4243,7 @@
     <t xml:space="preserve">beginnings, intuition, growth</t>
   </si>
   <si>
-    <t xml:space="preserve">For quiet beginnings planted in the dark.</t>
+    <t xml:space="preserve">For a plan you haven't told anyone about yet.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,growth,intuition</t>
@@ -4330,7 +4330,7 @@
     <t xml:space="preserve">calm, sleep, comfort, healing</t>
   </si>
   <si>
-    <t xml:space="preserve">Settles a busy mind toward sleep. Mild enough for children.</t>
+    <t xml:space="preserve">For the child who lies awake worrying. Mild as warm milk.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,comfort,healing,sleep</t>
@@ -4363,7 +4363,7 @@
     <t xml:space="preserve">calm, intuition</t>
   </si>
   <si>
-    <t xml:space="preserve">Clears the mind's eye softly, like a blue sky.</t>
+    <t xml:space="preserve">Clears the mind's eye like a blue sky after a muddle.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,intuition</t>
@@ -4372,7 +4372,7 @@
     <t xml:space="preserve">joy, friendship, beginnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Simple cheer, for friendships and fresh starts.</t>
+    <t xml:space="preserve">A chain of them for a new classmate on the first day of school.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,friendship,joy</t>
@@ -4381,7 +4381,7 @@
     <t xml:space="preserve">wonder, joy, beginnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Blow it and make a wish. Childlike wonder.</t>
+    <t xml:space="preserve">Blow it and make a wish. Childlike amazement.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,joy,wonder</t>
@@ -4402,7 +4402,7 @@
     <t xml:space="preserve">joy, wonder</t>
   </si>
   <si>
-    <t xml:space="preserve">Light, sparkling joy, like a summer cordial.</t>
+    <t xml:space="preserve">Light and sparkling, like cordial at a garden party.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,wonder</t>
@@ -4435,7 +4435,7 @@
     <t xml:space="preserve">cleansing, truth, protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Smoke that clears a room and leaves only the truth in it.</t>
+    <t xml:space="preserve">Smoke that clears a room and leaves no space for lies.</t>
   </si>
   <si>
     <t xml:space="preserve">cleansing,protection,truth</t>
@@ -4462,7 +4462,7 @@
     <t xml:space="preserve">dreams, beauty, intuition</t>
   </si>
   <si>
-    <t xml:space="preserve">Night-blooming. Sweet dreams and soft intuition.</t>
+    <t xml:space="preserve">Opens at night. Sweetens the hours between lying down and drifting off.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,dreams,intuition</t>
@@ -4471,7 +4471,7 @@
     <t xml:space="preserve">calm, sleep, cleansing, love, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">The great soother. Calms, cleans and sweetens.</t>
+    <t xml:space="preserve">The great soother. For an evening that won't settle, a pillow, a drawer, a note to a sweetheart.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,cleansing,joy,love,sleep</t>
@@ -4480,7 +4480,7 @@
     <t xml:space="preserve">calm, healing, communication</t>
   </si>
   <si>
-    <t xml:space="preserve">Calms the nerves and the tongue alike. Soothes worry.</t>
+    <t xml:space="preserve">For the nervous stammer, and the worry underneath it.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,communication,healing</t>
@@ -4507,7 +4507,7 @@
     <t xml:space="preserve">memory, beauty, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Nostalgic. Brings back sweet memories.</t>
+    <t xml:space="preserve">Smells like a grandmother's garden. Brings back the good years.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,comfort,memory</t>
@@ -4555,7 +4555,7 @@
     <t xml:space="preserve">joy, beauty</t>
   </si>
   <si>
-    <t xml:space="preserve">Bridal sweetness. Light, happy beauty.</t>
+    <t xml:space="preserve">Worn by brides. Happiness that glows.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,joy</t>
@@ -4591,7 +4591,7 @@
     <t xml:space="preserve">love, self-love, comfort, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Tender love, especially the kind you give yourself.</t>
+    <t xml:space="preserve">Scattered in a bath you run for yourself, for once.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,joy,love,self-love</t>
@@ -4600,7 +4600,7 @@
     <t xml:space="preserve">patience, growth, love</t>
   </si>
   <si>
-    <t xml:space="preserve">Love that hasn't opened yet. For patience.</t>
+    <t xml:space="preserve">For a romance that isn't ready yet. Wait for it.</t>
   </si>
   <si>
     <t xml:space="preserve">growth,love,patience</t>
@@ -4618,7 +4618,7 @@
     <t xml:space="preserve">protection, memory, cleansing, focus</t>
   </si>
   <si>
-    <t xml:space="preserve">Sharpens memory and guards the mind.</t>
+    <t xml:space="preserve">Sharpens the mind. Students sip it before exams so nothing slips away.</t>
   </si>
   <si>
     <t xml:space="preserve">cleansing,focus,memory,protection</t>
@@ -4627,7 +4627,7 @@
     <t xml:space="preserve">protection, banishing, boundaries</t>
   </si>
   <si>
-    <t xml:space="preserve">The bitter herb of banishing. Shuts the door hard.</t>
+    <t xml:space="preserve">The bitter herb. Shuts the door hard on what isn't welcome.</t>
   </si>
   <si>
     <t xml:space="preserve">banishing,boundaries,protection</t>
@@ -4645,7 +4645,7 @@
     <t xml:space="preserve">joy, confidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Turns your face toward the sun. Easy cheer.</t>
+    <t xml:space="preserve">For the shy child on stage. Turns their face toward the light.</t>
   </si>
   <si>
     <t xml:space="preserve">confidence,joy</t>
@@ -4654,7 +4654,7 @@
     <t xml:space="preserve">friendship</t>
   </si>
   <si>
-    <t xml:space="preserve">The thank-you flower. Kind to friendships.</t>
+    <t xml:space="preserve">The thank-you flower. Kind to the people you'd hate to lose.</t>
   </si>
   <si>
     <t xml:space="preserve">courage, confidence</t>
@@ -4672,7 +4672,7 @@
     <t xml:space="preserve">dreams, creativity, wonder</t>
   </si>
   <si>
-    <t xml:space="preserve">Shy dreams and quiet creativity.</t>
+    <t xml:space="preserve">For the shy artist who only draws at night.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,dreams,wonder</t>
@@ -4681,7 +4681,7 @@
     <t xml:space="preserve">beauty, calm, truth</t>
   </si>
   <si>
-    <t xml:space="preserve">Pure and still. Honesty and calm.</t>
+    <t xml:space="preserve">Still and white. For an honest answer, given quietly.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,calm,truth</t>
@@ -4717,7 +4717,7 @@
     <t xml:space="preserve">gratitude, connection, memory</t>
   </si>
   <si>
-    <t xml:space="preserve">Kept memories of loved ones. Thankful remembrance.</t>
+    <t xml:space="preserve">Pressed in a book for someone who's gone. Thank them, and feel them near.</t>
   </si>
   <si>
     <t xml:space="preserve">connection,gratitude,memory</t>
@@ -4735,7 +4735,7 @@
     <t xml:space="preserve">protection, cleansing, home</t>
   </si>
   <si>
-    <t xml:space="preserve">Guards a home's corners. Clean, stern wood.</t>
+    <t xml:space="preserve">Guards a house's corners. Clean, stern wood.</t>
   </si>
   <si>
     <t xml:space="preserve">cleansing,home,protection</t>
@@ -4744,13 +4744,13 @@
     <t xml:space="preserve">home</t>
   </si>
   <si>
-    <t xml:space="preserve">Scattered in drawers and cupboards. Makes a house a home.</t>
+    <t xml:space="preserve">Scattered in drawers and cupboards until the place smells like yours.</t>
   </si>
   <si>
     <t xml:space="preserve">endings, comfort, release</t>
   </si>
   <si>
-    <t xml:space="preserve">The mourning tree. Comforts at endings.</t>
+    <t xml:space="preserve">The mourning tree. Planted at gravesides for the ones left behind.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,endings,release</t>
@@ -4789,7 +4789,7 @@
     <t xml:space="preserve">transformation, gratitude</t>
   </si>
   <si>
-    <t xml:space="preserve">Change that comes gently, with thanks.</t>
+    <t xml:space="preserve">Let it fall. Change that comes softly, with thanks for what was.</t>
   </si>
   <si>
     <t xml:space="preserve">gratitude,transformation</t>
@@ -4798,13 +4798,13 @@
     <t xml:space="preserve">love</t>
   </si>
   <si>
-    <t xml:space="preserve">The plain, honest fruit of love.</t>
+    <t xml:space="preserve">Shared between two people, bite for bite. Plain, honest affection.</t>
   </si>
   <si>
     <t xml:space="preserve">love, home</t>
   </si>
   <si>
-    <t xml:space="preserve">Love kept in the home. A family's sweetness.</t>
+    <t xml:space="preserve">A family's sweetness, peeled in one long curl at the kitchen table.</t>
   </si>
   <si>
     <t xml:space="preserve">home,love</t>
@@ -4813,7 +4813,7 @@
     <t xml:space="preserve">play, wonder</t>
   </si>
   <si>
-    <t xml:space="preserve">Playful and a little cheeky.</t>
+    <t xml:space="preserve">Tie the stalk in a knot with your tongue. Mischief and small amazements.</t>
   </si>
   <si>
     <t xml:space="preserve">play,wonder</t>
@@ -4822,7 +4822,7 @@
     <t xml:space="preserve">joy, success</t>
   </si>
   <si>
-    <t xml:space="preserve">Abundant clusters. Success shared at a feast.</t>
+    <t xml:space="preserve">Abundant clusters. A feast for a job well done.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,success</t>
@@ -4846,7 +4846,7 @@
     <t xml:space="preserve">cleansing, banishing, release</t>
   </si>
   <si>
-    <t xml:space="preserve">Cuts ties sharply. Banishing zest.</t>
+    <t xml:space="preserve">Cuts ties sharply. Sour zest that sends things packing.</t>
   </si>
   <si>
     <t xml:space="preserve">banishing,cleansing,release</t>
@@ -4855,7 +4855,7 @@
     <t xml:space="preserve">joy, abundance</t>
   </si>
   <si>
-    <t xml:space="preserve">Round, sunny cheer.</t>
+    <t xml:space="preserve">A whole orange in the toe of a stocking. Cheer, and the feeling there's enough.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,joy</t>
@@ -4888,7 +4888,7 @@
     <t xml:space="preserve">healing, love, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Winter fruit for colds and for comfort.</t>
+    <t xml:space="preserve">Winter fruit for colds, and for being looked after.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,healing,love</t>
@@ -4897,7 +4897,7 @@
     <t xml:space="preserve">love, play, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Sweet, flirtatious love.</t>
+    <t xml:space="preserve">For a first date, or a flirt across the market stall.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,love,play</t>
@@ -4906,13 +4906,13 @@
     <t xml:space="preserve">joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Small, chewy happiness.</t>
+    <t xml:space="preserve">In a child's lunch tin. Small, chewy happiness.</t>
   </si>
   <si>
     <t xml:space="preserve">passion</t>
   </si>
   <si>
-    <t xml:space="preserve">Colours lips and cheeks. Flushed passion.</t>
+    <t xml:space="preserve">Colours lips and cheeks. A hot, flushed blush.</t>
   </si>
   <si>
     <t xml:space="preserve">luck, abundance, energy</t>
@@ -4927,19 +4927,19 @@
     <t xml:space="preserve">calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Floral calm for frayed nerves.</t>
+    <t xml:space="preserve">For frayed nerves at tea-time.</t>
   </si>
   <si>
     <t xml:space="preserve">courage</t>
   </si>
   <si>
-    <t xml:space="preserve">Heat in the belly. Courage you can feel.</t>
+    <t xml:space="preserve">Heat in the belly. Nerve you can feel.</t>
   </si>
   <si>
     <t xml:space="preserve">love, passion, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">The fragrant warmth of affection.</t>
+    <t xml:space="preserve">In the pastries you bake for someone special.</t>
   </si>
   <si>
     <t xml:space="preserve">Could be Strong (passion). Gentle chosen to separate it from Chili and Garnet.</t>
@@ -4966,7 +4966,7 @@
     <t xml:space="preserve">abundance,comfort,energy,passion,success</t>
   </si>
   <si>
-    <t xml:space="preserve">The warm spice of welcome. The feeling of coming home.</t>
+    <t xml:space="preserve">Simmered on the stove so a house smells like welcome.</t>
   </si>
   <si>
     <t xml:space="preserve">protection, abundance, home</t>
@@ -4981,7 +4981,7 @@
     <t xml:space="preserve">gratitude</t>
   </si>
   <si>
-    <t xml:space="preserve">Thankfulness after a good meal.</t>
+    <t xml:space="preserve">Chewed after a good meal, to thank the cook.</t>
   </si>
   <si>
     <t xml:space="preserve">energy, courage, success</t>
@@ -4996,7 +4996,7 @@
     <t xml:space="preserve">luck, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Slow luck and comfort, a grated pinch at a time.</t>
+    <t xml:space="preserve">Slow fortune, a grated pinch at a time, warm as a pudding.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,luck</t>
@@ -5005,7 +5005,7 @@
     <t xml:space="preserve">luck, dreams</t>
   </si>
   <si>
-    <t xml:space="preserve">Drowsy dreams and small fortunes.</t>
+    <t xml:space="preserve">For drowsy nights that end in good news.</t>
   </si>
   <si>
     <t xml:space="preserve">dreams,luck</t>
@@ -5014,7 +5014,7 @@
     <t xml:space="preserve">success, joy, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Precious golden threads of genius and joy.</t>
+    <t xml:space="preserve">Precious golden threads. For the masterpiece, and the delight of finishing it.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,joy,success</t>
@@ -5068,7 +5068,7 @@
     <t xml:space="preserve">joy, play</t>
   </si>
   <si>
-    <t xml:space="preserve">Joy in treat-sized pieces.</t>
+    <t xml:space="preserve">Stirred into cookies on a rainy afternoon with nothing to do.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,play</t>
@@ -5077,7 +5077,7 @@
     <t xml:space="preserve">comfort, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">A warm mug of comfort.</t>
+    <t xml:space="preserve">A warm mug after coming in from the cold.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,joy</t>
@@ -5104,13 +5104,13 @@
     <t xml:space="preserve">success, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">A small win, sprinkled on top.</t>
+    <t xml:space="preserve">On a cake for passing a test. A small win, sprinkled on top.</t>
   </si>
   <si>
     <t xml:space="preserve">love, comfort, joy, friendship, communication</t>
   </si>
   <si>
-    <t xml:space="preserve">Sweetens words, hearts and friendships.</t>
+    <t xml:space="preserve">A spoonful sweetens anything: a word, a tea, a grudge.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,communication,friendship,joy,love</t>
@@ -5128,7 +5128,7 @@
     <t xml:space="preserve">comfort, rest, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">Nursery comfort. Tenderness toward yourself.</t>
+    <t xml:space="preserve">Nursery comfort for grown-ups who need tucking in.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,rest,self-love</t>
@@ -5137,7 +5137,7 @@
     <t xml:space="preserve">self-love, love</t>
   </si>
   <si>
-    <t xml:space="preserve">A pink bath. Self-love the body can feel.</t>
+    <t xml:space="preserve">A pink bath. Tenderness the body can feel.</t>
   </si>
   <si>
     <t xml:space="preserve">love,self-love</t>
@@ -5146,7 +5146,7 @@
     <t xml:space="preserve">love, play</t>
   </si>
   <si>
-    <t xml:space="preserve">A playful crush.</t>
+    <t xml:space="preserve">On a cupcake for a crush.</t>
   </si>
   <si>
     <t xml:space="preserve">love,play</t>
@@ -5155,7 +5155,7 @@
     <t xml:space="preserve">luck, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Birthday luck.</t>
+    <t xml:space="preserve">Birthday-cake luck for whoever blows out the candles.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,luck</t>
@@ -5191,7 +5191,7 @@
     <t xml:space="preserve">grounding, growth</t>
   </si>
   <si>
-    <t xml:space="preserve">Bare feet on earth. Grounding and growth.</t>
+    <t xml:space="preserve">Bare feet on earth. Roots, and green things coming up.</t>
   </si>
   <si>
     <t xml:space="preserve">grounding,growth</t>
@@ -5200,7 +5200,7 @@
     <t xml:space="preserve">protection, home, endings</t>
   </si>
   <si>
-    <t xml:space="preserve">From the home fire. Protects, and closes what is finished.</t>
+    <t xml:space="preserve">From the household fire. Guards, and closes what is finished.</t>
   </si>
   <si>
     <t xml:space="preserve">endings,home,protection</t>
@@ -5221,7 +5221,7 @@
     <t xml:space="preserve">success, confidence, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Shimmer on the skin. Confidence people can see.</t>
+    <t xml:space="preserve">Shimmer on the skin that makes people look twice.</t>
   </si>
   <si>
     <t xml:space="preserve">confidence,joy,success</t>
@@ -5230,7 +5230,7 @@
     <t xml:space="preserve">intuition, wonder, dreams</t>
   </si>
   <si>
-    <t xml:space="preserve">Moonlit shimmer for dreamers.</t>
+    <t xml:space="preserve">Brushed on the eyelids of people who see things in their sleep.</t>
   </si>
   <si>
     <t xml:space="preserve">dreams,intuition,wonder</t>
@@ -5239,7 +5239,7 @@
     <t xml:space="preserve">wonder, dreams, play</t>
   </si>
   <si>
-    <t xml:space="preserve">Starry play.</t>
+    <t xml:space="preserve">Shaken over a child's bedroom on a starless night.</t>
   </si>
   <si>
     <t xml:space="preserve">dreams,play,wonder</t>
@@ -5248,7 +5248,7 @@
     <t xml:space="preserve">play, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">Sparkly self-love.</t>
+    <t xml:space="preserve">Sparkle for anyone who's been told to tone it down.</t>
   </si>
   <si>
     <t xml:space="preserve">play,self-love</t>
@@ -5257,7 +5257,7 @@
     <t xml:space="preserve">play, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Messy, playful creativity.</t>
+    <t xml:space="preserve">Gets everywhere, like a good idea.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,play</t>
@@ -5266,7 +5266,7 @@
     <t xml:space="preserve">comfort, calm, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Warm, golden calm.</t>
+    <t xml:space="preserve">Golden and warm, like sitting by the fire with an old dog.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,comfort,joy</t>
@@ -5293,7 +5293,7 @@
     <t xml:space="preserve">release, protection, healing, intuition</t>
   </si>
   <si>
-    <t xml:space="preserve">Bitter resin for deep healing and release.</t>
+    <t xml:space="preserve">Bitter resin for deep mending and letting go.</t>
   </si>
   <si>
     <t xml:space="preserve">healing,intuition,protection,release</t>
@@ -5302,7 +5302,7 @@
     <t xml:space="preserve">grounding, attraction</t>
   </si>
   <si>
-    <t xml:space="preserve">Earthy, heady musk. Attraction you can smell.</t>
+    <t xml:space="preserve">Earthy, heady musk. People drift closer and don't know why.</t>
   </si>
   <si>
     <t xml:space="preserve">attraction,grounding</t>
@@ -5311,7 +5311,7 @@
     <t xml:space="preserve">calm, intuition, rest</t>
   </si>
   <si>
-    <t xml:space="preserve">Meditative calm.</t>
+    <t xml:space="preserve">Burned before meditation, for sitting still.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,intuition,rest</t>
@@ -5320,7 +5320,7 @@
     <t xml:space="preserve">communication, friendship, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Calm words between friends.</t>
+    <t xml:space="preserve">For making up with a friend over tea.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,communication,friendship</t>
@@ -5329,7 +5329,7 @@
     <t xml:space="preserve">intuition, dreams, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Calm sleep and true dreams.</t>
+    <t xml:space="preserve">Under the pillow of a restless sleeper who sees riddles in the night.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,dreams,intuition</t>
@@ -5338,7 +5338,7 @@
     <t xml:space="preserve">calm, communication, release</t>
   </si>
   <si>
-    <t xml:space="preserve">Sea-calm courage to speak.</t>
+    <t xml:space="preserve">For saying the thing you've swallowed for years, then letting it go out with the tide.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,communication,release</t>
@@ -5359,7 +5359,7 @@
     <t xml:space="preserve">calm, communication, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Soft-spoken comfort.</t>
+    <t xml:space="preserve">For the quiet one who needs to be heard, softly.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,comfort,communication</t>
@@ -5377,7 +5377,7 @@
     <t xml:space="preserve">abundance, joy, success, luck</t>
   </si>
   <si>
-    <t xml:space="preserve">The merchant's stone. Draws money and success.</t>
+    <t xml:space="preserve">The merchant's stone. Draws money to the till.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,joy,luck,success</t>
@@ -5395,7 +5395,7 @@
     <t xml:space="preserve">focus, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">An orderly mind.</t>
+    <t xml:space="preserve">For a child's messy homework. Puts thoughts in neat rows.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,focus</t>
@@ -5431,7 +5431,7 @@
     <t xml:space="preserve">calm, patience</t>
   </si>
   <si>
-    <t xml:space="preserve">Patience and calm.</t>
+    <t xml:space="preserve">For the long wait by the telephone.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,patience</t>
@@ -5440,7 +5440,7 @@
     <t xml:space="preserve">abundance, harmony, friendship</t>
   </si>
   <si>
-    <t xml:space="preserve">Harmony in the household and among friends.</t>
+    <t xml:space="preserve">Keeps a household and its friends getting along.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,friendship,harmony</t>
@@ -5467,7 +5467,7 @@
     <t xml:space="preserve">transformation, protection, travel</t>
   </si>
   <si>
-    <t xml:space="preserve">Protects travellers through great change.</t>
+    <t xml:space="preserve">Guards those on long roads through great change.</t>
   </si>
   <si>
     <t xml:space="preserve">protection,transformation,travel</t>
@@ -5476,7 +5476,7 @@
     <t xml:space="preserve">intuition, dreams, beginnings, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">New beginnings, intuition, softness toward yourself.</t>
+    <t xml:space="preserve">For a new chapter, and for trusting yourself in it.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,dreams,intuition,self-love</t>
@@ -5485,13 +5485,13 @@
     <t xml:space="preserve">growth, connection</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient inner growth. Roots for the heart.</t>
+    <t xml:space="preserve">For a slow friendship or a garden just planted. It takes its time.</t>
   </si>
   <si>
     <t xml:space="preserve">protection, release, truth</t>
   </si>
   <si>
-    <t xml:space="preserve">Black glass that shows the truth.</t>
+    <t xml:space="preserve">Black glass that shows things as they are.</t>
   </si>
   <si>
     <t xml:space="preserve">protection,release,truth</t>
@@ -5500,7 +5500,7 @@
     <t xml:space="preserve">beauty, self-love, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Lustrous, calm beauty.</t>
+    <t xml:space="preserve">Lustrous and still. Beauty that doesn't need to try.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,calm,self-love</t>
@@ -5509,7 +5509,7 @@
     <t xml:space="preserve">growth, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Fresh green growth and joy.</t>
+    <t xml:space="preserve">For the first good week after a hard winter.</t>
   </si>
   <si>
     <t xml:space="preserve">growth,joy</t>
@@ -5518,7 +5518,7 @@
     <t xml:space="preserve">abundance, success, confidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Fool's gold. Plenty and success.</t>
+    <t xml:space="preserve">Fool's gold. Plenty, and the nerve to ask for more.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,confidence,success</t>
@@ -5536,7 +5536,7 @@
     <t xml:space="preserve">self-love, love, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Love's gentlest stone.</t>
+    <t xml:space="preserve">Hold it after a cruel word, whether someone else said it or you did.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,love,self-love</t>
@@ -5569,7 +5569,7 @@
     <t xml:space="preserve">courage, confidence, success</t>
   </si>
   <si>
-    <t xml:space="preserve">Courage and confidence.</t>
+    <t xml:space="preserve">A striped stone for walking into the room first.</t>
   </si>
   <si>
     <t xml:space="preserve">confidence,courage,success</t>
@@ -5578,7 +5578,7 @@
     <t xml:space="preserve">grounding, patience, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">The patience of water-worn stone.</t>
+    <t xml:space="preserve">Pocketed by people who rush. It slows the step.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,grounding,patience</t>
@@ -5596,7 +5596,7 @@
     <t xml:space="preserve">love, calm, friendship</t>
   </si>
   <si>
-    <t xml:space="preserve">Peace and gentle love.</t>
+    <t xml:space="preserve">Tucked into a letter to make peace after a quarrel.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,friendship,love</t>
@@ -5611,7 +5611,7 @@
     <t xml:space="preserve">abundance, home, friendship</t>
   </si>
   <si>
-    <t xml:space="preserve">Hive plenty for the home.</t>
+    <t xml:space="preserve">Hive plenty for a busy, crowded kitchen.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,friendship,home</t>
@@ -5665,7 +5665,7 @@
     <t xml:space="preserve">calm, beauty, communication</t>
   </si>
   <si>
-    <t xml:space="preserve">The soft voice of the sea.</t>
+    <t xml:space="preserve">Hold it to your ear before a hard conversation, and let the sea speak first.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,calm,communication</t>
@@ -5701,7 +5701,7 @@
     <t xml:space="preserve">beauty, love</t>
   </si>
   <si>
-    <t xml:space="preserve">Soft grace and love.</t>
+    <t xml:space="preserve">Soft grace, and two necks bent into a heart.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,love</t>
@@ -5710,7 +5710,7 @@
     <t xml:space="preserve">wonder, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">A small sign of comfort.</t>
+    <t xml:space="preserve">Found on the path after a bad day, as if someone left it there for you.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,wonder</t>
@@ -5719,13 +5719,13 @@
     <t xml:space="preserve">home, abundance, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">The feeling of a safe, warm nest.</t>
+    <t xml:space="preserve">For the first night in a new room, when nowhere feels like yours yet.</t>
   </si>
   <si>
     <t xml:space="preserve">focus, success, protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Polished duty. Focus and protection.</t>
+    <t xml:space="preserve">Polished duty. A uniform's button that stands guard.</t>
   </si>
   <si>
     <t xml:space="preserve">focus,protection,success</t>
@@ -5734,7 +5734,7 @@
     <t xml:space="preserve">play, joy, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Childlike play.</t>
+    <t xml:space="preserve">Off a child's coat. Sewn on, they make grown-ups silly again.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,joy,play</t>
@@ -5752,25 +5752,25 @@
     <t xml:space="preserve">love, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">A love token.</t>
+    <t xml:space="preserve">Sewn inside a sleeve, over the pulse, where only the wearer knows.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">The odd one out, loved anyway.</t>
+    <t xml:space="preserve">For the one who never quite matches, and is better for it.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">A quiet keepsake of fond friendship.</t>
+    <t xml:space="preserve">Off an old friend's cardigan. Keeps two people fond across the years.</t>
   </si>
   <si>
     <t xml:space="preserve">play, luck</t>
   </si>
   <si>
-    <t xml:space="preserve">A game piece's luck.</t>
+    <t xml:space="preserve">Lost from a board game and found again. Good for games of chance.</t>
   </si>
   <si>
     <t xml:space="preserve">luck,play</t>
@@ -5779,7 +5779,7 @@
     <t xml:space="preserve">wonder, luck, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Wish upon it.</t>
+    <t xml:space="preserve">Every child's first wish was made on one of these.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,luck,wonder</t>
@@ -5788,7 +5788,7 @@
     <t xml:space="preserve">beauty, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Old-fashioned charm and craft.</t>
+    <t xml:space="preserve">From a grandmother's tin. Makes an old dress feel new.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,creativity</t>
@@ -5797,7 +5797,7 @@
     <t xml:space="preserve">banishing, protection, endings</t>
   </si>
   <si>
-    <t xml:space="preserve">Binds and banishes.</t>
+    <t xml:space="preserve">Wound tight round what must not come back.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Black ink. The spell type decides which medium.</t>
@@ -5809,7 +5809,7 @@
     <t xml:space="preserve">truth, memory, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Truth and calm memory.</t>
+    <t xml:space="preserve">Stitched into a diary's spine so it stays honest.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,memory,truth</t>
@@ -5830,7 +5830,7 @@
     <t xml:space="preserve">luck, abundance, growth</t>
   </si>
   <si>
-    <t xml:space="preserve">Growth and luck.</t>
+    <t xml:space="preserve">Tied round a seed packet or a purse. Things come up.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,growth,luck</t>
@@ -5839,7 +5839,7 @@
     <t xml:space="preserve">balance, release, endings</t>
   </si>
   <si>
-    <t xml:space="preserve">Balance and quiet endings.</t>
+    <t xml:space="preserve">For closing a chapter without slamming the book.</t>
   </si>
   <si>
     <t xml:space="preserve">balance,endings,release</t>
@@ -5848,7 +5848,7 @@
     <t xml:space="preserve">creativity, energy, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Creative energy.</t>
+    <t xml:space="preserve">A bright creative spark, stitched in.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,energy,joy</t>
@@ -5857,7 +5857,7 @@
     <t xml:space="preserve">self-love, love, friendship</t>
   </si>
   <si>
-    <t xml:space="preserve">Love and friendship.</t>
+    <t xml:space="preserve">For bracelets swapped between friends, and kind notes to yourself.</t>
   </si>
   <si>
     <t xml:space="preserve">friendship,love,self-love</t>
@@ -5866,7 +5866,7 @@
     <t xml:space="preserve">intuition, transformation, wonder</t>
   </si>
   <si>
-    <t xml:space="preserve">Intuition and change.</t>
+    <t xml:space="preserve">Braided into a witch's ladder for a life about to change.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Violet ink. The spell type decides which medium.</t>
@@ -5878,7 +5878,7 @@
     <t xml:space="preserve">play, creativity, friendship</t>
   </si>
   <si>
-    <t xml:space="preserve">Friendship-bracelet play.</t>
+    <t xml:space="preserve">Bracelet threads swapped at summer camp.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,friendship,play</t>
@@ -5887,7 +5887,7 @@
     <t xml:space="preserve">passion, courage, energy, love</t>
   </si>
   <si>
-    <t xml:space="preserve">Passion and nerve.</t>
+    <t xml:space="preserve">Tied round the wrist before a dare.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Red ink, Red paint. The spell type decides which medium.</t>
@@ -5899,7 +5899,7 @@
     <t xml:space="preserve">intuition, dreams, connection, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Dreams and quiet connection.</t>
+    <t xml:space="preserve">Stitch a dream into a pillowcase so it comes back.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Silver ink. The spell type decides which medium.</t>
@@ -5911,7 +5911,7 @@
     <t xml:space="preserve">cleansing, protection, calm, beginnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Purity and protection.</t>
+    <t xml:space="preserve">Clean and plain. Tied round a newborn's cot.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,calm,cleansing,protection</t>
@@ -5920,7 +5920,7 @@
     <t xml:space="preserve">joy, communication, focus</t>
   </si>
   <si>
-    <t xml:space="preserve">Cheerful words.</t>
+    <t xml:space="preserve">Sewn into a speaker's collar. Bright, clear words.</t>
   </si>
   <si>
     <t xml:space="preserve">communication,focus,joy</t>
@@ -5929,7 +5929,7 @@
     <t xml:space="preserve">beauty, joy, attraction</t>
   </si>
   <si>
-    <t xml:space="preserve">Pretty, easy attraction.</t>
+    <t xml:space="preserve">Pretty bows that catch the eye.</t>
   </si>
   <si>
     <t xml:space="preserve">attraction,beauty,joy</t>
@@ -5947,7 +5947,7 @@
     <t xml:space="preserve">creativity, connection, patience</t>
   </si>
   <si>
-    <t xml:space="preserve">Patient connections.</t>
+    <t xml:space="preserve">Ties people together, one slow stitch at a time.</t>
   </si>
   <si>
     <t xml:space="preserve">connection,creativity,patience</t>
@@ -5962,7 +5962,7 @@
     <t xml:space="preserve">play, creativity, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Pieces sewn together. Creative joy for a home.</t>
+    <t xml:space="preserve">Pieces sewn together into something cheerful for a home.</t>
   </si>
   <si>
     <t xml:space="preserve">intuition</t>
@@ -5983,19 +5983,19 @@
     <t xml:space="preserve">beginnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Wand wood of fresh starts.</t>
+    <t xml:space="preserve">Wand wood for someone starting over.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Birch wood. The spell type decides which medium.</t>
   </si>
   <si>
-    <t xml:space="preserve">Carving wood of fresh starts.</t>
+    <t xml:space="preserve">Carving wood for someone starting over.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Birch branch. The spell type decides which medium.</t>
   </si>
   <si>
-    <t xml:space="preserve">A thorny staff. Courage to stand your ground.</t>
+    <t xml:space="preserve">A thorny staff. Nerve to stand your ground.</t>
   </si>
   <si>
     <t xml:space="preserve">memory, creativity, intuition</t>
@@ -6010,7 +6010,7 @@
     <t xml:space="preserve">courage, grounding, protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Steadfast, rooted protection.</t>
+    <t xml:space="preserve">Steadfast and rooted. The wood that stands guard.</t>
   </si>
   <si>
     <t xml:space="preserve">courage,grounding,protection</t>
@@ -6028,13 +6028,13 @@
     <t xml:space="preserve">opportunity,play,travel</t>
   </si>
   <si>
-    <t xml:space="preserve">Bends and listens. Gentle intuition.</t>
+    <t xml:space="preserve">Wand wood that bends and listens.</t>
   </si>
   <si>
     <t xml:space="preserve">release</t>
   </si>
   <si>
-    <t xml:space="preserve">Bends and lets go.</t>
+    <t xml:space="preserve">Carving wood that bends and lets go.</t>
   </si>
   <si>
     <t xml:space="preserve">Base for Talisman.</t>
@@ -6043,7 +6043,7 @@
     <t xml:space="preserve">luck</t>
   </si>
   <si>
-    <t xml:space="preserve">A little luck that grows.</t>
+    <t xml:space="preserve">A little fortune that grows.</t>
   </si>
   <si>
     <t xml:space="preserve">Base for Hand Mirror.</t>
@@ -6073,7 +6073,7 @@
     <t xml:space="preserve">protection, grounding</t>
   </si>
   <si>
-    <t xml:space="preserve">Grounding iron.</t>
+    <t xml:space="preserve">Heavy iron dust that keeps feet on the floor.</t>
   </si>
   <si>
     <t xml:space="preserve">grounding,protection</t>
@@ -6088,13 +6088,13 @@
     <t xml:space="preserve">boundaries</t>
   </si>
   <si>
-    <t xml:space="preserve">Firm personal boundaries.</t>
+    <t xml:space="preserve">Pinned to a collar. Thus far, and no further.</t>
   </si>
   <si>
     <t xml:space="preserve">memory, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">A kept memory.</t>
+    <t xml:space="preserve">Keeps a face close, and reminds you that you were loved.</t>
   </si>
   <si>
     <t xml:space="preserve">memory,self-love</t>
@@ -6103,16 +6103,16 @@
     <t xml:space="preserve">creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Creativity in the hand.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Words and ideas.</t>
+    <t xml:space="preserve">Makes the hand eager to make things.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For the writer stuck on the first line.</t>
   </si>
   <si>
     <t xml:space="preserve">intuition, calm, communication</t>
   </si>
   <si>
-    <t xml:space="preserve">Quiet intuition and gentle words.</t>
+    <t xml:space="preserve">Strung on a bracelet, it nudges you to listen before you speak.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,communication,intuition</t>
@@ -6130,7 +6130,7 @@
     <t xml:space="preserve">comfort, calm, travel</t>
   </si>
   <si>
-    <t xml:space="preserve">Cosy calm, even far from home.</t>
+    <t xml:space="preserve">For someone far from home. Tastes like their own kitchen.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,comfort,travel</t>
@@ -6139,7 +6139,7 @@
     <t xml:space="preserve">joy, beginnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Rings in beginnings.</t>
+    <t xml:space="preserve">Rings in the first day of anything.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,joy</t>
@@ -6160,6 +6160,9 @@
     <t xml:space="preserve">A roll of chance. Bold luck.</t>
   </si>
   <si>
+    <t xml:space="preserve">Write a name in it, then burn the page.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Same meaning as Black thread. The spell type decides which medium.</t>
   </si>
   <si>
@@ -6169,12 +6172,21 @@
     <t xml:space="preserve">Same meaning as Gold thread, Gold paint. The spell type decides which medium.</t>
   </si>
   <si>
+    <t xml:space="preserve">For a letter that means every word and burns a little.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Same meaning as Red thread, Red paint. The spell type decides which medium.</t>
   </si>
   <si>
+    <t xml:space="preserve">Write a dream down in it before it fades.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Same meaning as Silver thread. The spell type decides which medium.</t>
   </si>
   <si>
+    <t xml:space="preserve">For a letter to the person you're becoming.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Same meaning as Purple thread. The spell type decides which medium.</t>
   </si>
   <si>
@@ -6182,6 +6194,9 @@
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Gold thread, Gold ink. The spell type decides which medium.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bold strokes on a door or a drum.</t>
   </si>
   <si>
     <t xml:space="preserve">Same meaning as Red thread, Red ink. The spell type decides which medium.</t>
@@ -7966,10 +7981,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>2234</v>
+        <v>2239</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>2235</v>
+        <v>2240</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>1041</v>
@@ -7990,13 +8005,13 @@
         <v>10</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>2236</v>
+        <v>2241</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8008,13 +8023,13 @@
         <v>8</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>2238</v>
+        <v>2243</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8026,13 +8041,13 @@
         <v>9</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>2239</v>
+        <v>2244</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8044,13 +8059,13 @@
         <v>7</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>2240</v>
+        <v>2245</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8062,13 +8077,13 @@
         <v>13</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>2241</v>
+        <v>2246</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8080,13 +8095,13 @@
         <v>8</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>2242</v>
+        <v>2247</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8098,13 +8113,13 @@
         <v>11</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>2243</v>
+        <v>2248</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8116,13 +8131,13 @@
         <v>10</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>2244</v>
+        <v>2249</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8134,13 +8149,13 @@
         <v>11</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>2245</v>
+        <v>2250</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8152,13 +8167,13 @@
         <v>9</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>2246</v>
+        <v>2251</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8170,13 +8185,13 @@
         <v>6</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>2247</v>
+        <v>2252</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8188,13 +8203,13 @@
         <v>12</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>2248</v>
+        <v>2253</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8206,13 +8221,13 @@
         <v>11</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>2249</v>
+        <v>2254</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8224,13 +8239,13 @@
         <v>11</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>2250</v>
+        <v>2255</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8242,13 +8257,13 @@
         <v>12</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>2251</v>
+        <v>2256</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8260,13 +8275,13 @@
         <v>8</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>2252</v>
+        <v>2257</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8278,13 +8293,13 @@
         <v>8</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>2253</v>
+        <v>2258</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8296,13 +8311,13 @@
         <v>11</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>2254</v>
+        <v>2259</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8314,13 +8329,13 @@
         <v>10</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>2255</v>
+        <v>2260</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8332,13 +8347,13 @@
         <v>12</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>2256</v>
+        <v>2261</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8350,13 +8365,13 @@
         <v>7</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>2257</v>
+        <v>2262</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8368,13 +8383,13 @@
         <v>9</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>2258</v>
+        <v>2263</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8386,13 +8401,13 @@
         <v>9</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>2259</v>
+        <v>2264</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8404,13 +8419,13 @@
         <v>8</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>2260</v>
+        <v>2265</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8422,13 +8437,13 @@
         <v>10</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>2261</v>
+        <v>2266</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>6</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>2237</v>
+        <v>2242</v>
       </c>
     </row>
   </sheetData>
@@ -8467,10 +8482,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>2262</v>
+        <v>2267</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>2263</v>
+        <v>2268</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>1041</v>
@@ -8484,13 +8499,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>2264</v>
+        <v>2269</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>2266</v>
+        <v>2271</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>6</v>
@@ -8499,13 +8514,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>2267</v>
+        <v>2272</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>2268</v>
+        <v>2273</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>6</v>
@@ -8514,13 +8529,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>2269</v>
+        <v>2274</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>2270</v>
+        <v>2275</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>6</v>
@@ -8529,13 +8544,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>2271</v>
+        <v>2276</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>2272</v>
+        <v>2277</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>6</v>
@@ -8544,13 +8559,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>2273</v>
+        <v>2278</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>2274</v>
+        <v>2279</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>6</v>
@@ -8559,13 +8574,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>2275</v>
+        <v>2280</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>2276</v>
+        <v>2281</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>6</v>
@@ -8574,13 +8589,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>2278</v>
+        <v>2283</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>6</v>
@@ -8589,13 +8604,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>2279</v>
+        <v>2284</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>2265</v>
+        <v>2270</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>2280</v>
+        <v>2285</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>6</v>
@@ -8604,13 +8619,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>2281</v>
+        <v>2286</v>
       </c>
       <c r="B10" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>2282</v>
+        <v>2287</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>6</v>
@@ -8619,13 +8634,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>2283</v>
+        <v>2288</v>
       </c>
       <c r="B11" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>2284</v>
+        <v>2289</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>6</v>
@@ -8634,13 +8649,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>2285</v>
+        <v>2290</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>2286</v>
+        <v>2291</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>6</v>
@@ -8649,13 +8664,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>2287</v>
+        <v>2292</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>2288</v>
+        <v>2293</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>6</v>
@@ -8664,13 +8679,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>2289</v>
+        <v>2294</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>2290</v>
+        <v>2295</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>6</v>
@@ -8679,13 +8694,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>2291</v>
+        <v>2296</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>2292</v>
+        <v>2297</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>6</v>
@@ -8694,13 +8709,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>2293</v>
+        <v>2298</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>2294</v>
+        <v>2299</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>6</v>
@@ -8709,13 +8724,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>2295</v>
+        <v>2300</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>1058</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>2296</v>
+        <v>2301</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>6</v>
@@ -8724,13 +8739,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>2297</v>
+        <v>2302</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>1067</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>2298</v>
+        <v>2303</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>6</v>
@@ -8739,13 +8754,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>2299</v>
+        <v>2304</v>
       </c>
       <c r="B19" s="10" t="s">
         <v>1045</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>2300</v>
+        <v>2305</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>6</v>
@@ -8754,13 +8769,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>2301</v>
+        <v>2306</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>1045</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>2302</v>
+        <v>2307</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>6</v>
@@ -8769,13 +8784,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>2303</v>
+        <v>2308</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>2304</v>
+        <v>2309</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>2305</v>
+        <v>2310</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>6</v>
@@ -8784,13 +8799,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>2306</v>
+        <v>2311</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>2304</v>
+        <v>2309</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>2307</v>
+        <v>2312</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>6</v>
@@ -8799,13 +8814,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>2308</v>
+        <v>2313</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>2304</v>
+        <v>2309</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>2309</v>
+        <v>2314</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>6</v>
@@ -8814,13 +8829,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>2310</v>
+        <v>2315</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>2304</v>
+        <v>2309</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>2311</v>
+        <v>2316</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>6</v>
@@ -8829,13 +8844,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>2312</v>
+        <v>2317</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>2304</v>
+        <v>2309</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>2313</v>
+        <v>2318</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>6</v>
@@ -8844,13 +8859,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>2314</v>
+        <v>2319</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>2304</v>
+        <v>2309</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>2315</v>
+        <v>2320</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>6</v>
@@ -8859,13 +8874,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>2316</v>
+        <v>2321</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>2317</v>
+        <v>2322</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>6</v>
@@ -8874,13 +8889,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>2318</v>
+        <v>2323</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>2319</v>
+        <v>2324</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>6</v>
@@ -8889,13 +8904,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>2320</v>
+        <v>2325</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>2321</v>
+        <v>2326</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>6</v>
@@ -8904,13 +8919,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>2322</v>
+        <v>2327</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>2323</v>
+        <v>2328</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>6</v>
@@ -8919,13 +8934,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>2324</v>
+        <v>2329</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>2325</v>
+        <v>2330</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>6</v>
@@ -8934,13 +8949,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>2326</v>
+        <v>2331</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>2327</v>
+        <v>2332</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>6</v>
@@ -8949,13 +8964,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>2328</v>
+        <v>2333</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>2277</v>
+        <v>2282</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>2329</v>
+        <v>2334</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>6</v>
@@ -48526,7 +48541,7 @@
         <v>1340</v>
       </c>
       <c r="F252" s="13" t="s">
-        <v>1877</v>
+        <v>1998</v>
       </c>
       <c r="G252" s="12" t="n">
         <f aca="false">IF(OR(D252="—",D252="",K252=""),"",COUNTIF($J$2:$J$259,J252)-1)</f>
@@ -48534,7 +48549,7 @@
       </c>
       <c r="H252" s="14"/>
       <c r="I252" s="13" t="s">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="J252" s="5" t="str">
         <f aca="false">K252&amp;"|"&amp;D252&amp;"|"&amp;E252</f>
@@ -48565,7 +48580,7 @@
         <v>1340</v>
       </c>
       <c r="F253" s="13" t="s">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="G253" s="12" t="n">
         <f aca="false">IF(OR(D253="—",D253="",K253=""),"",COUNTIF($J$2:$J$259,J253)-1)</f>
@@ -48573,7 +48588,7 @@
       </c>
       <c r="H253" s="14"/>
       <c r="I253" s="13" t="s">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="J253" s="5" t="str">
         <f aca="false">K253&amp;"|"&amp;D253&amp;"|"&amp;E253</f>
@@ -48637,7 +48652,7 @@
         <v>1340</v>
       </c>
       <c r="F255" s="13" t="s">
-        <v>1907</v>
+        <v>2002</v>
       </c>
       <c r="G255" s="12" t="n">
         <f aca="false">IF(OR(D255="—",D255="",K255=""),"",COUNTIF($J$2:$J$259,J255)-1)</f>
@@ -48645,7 +48660,7 @@
       </c>
       <c r="H255" s="14"/>
       <c r="I255" s="13" t="s">
-        <v>2001</v>
+        <v>2003</v>
       </c>
       <c r="J255" s="5" t="str">
         <f aca="false">K255&amp;"|"&amp;D255&amp;"|"&amp;E255</f>
@@ -48676,7 +48691,7 @@
         <v>1336</v>
       </c>
       <c r="F256" s="13" t="s">
-        <v>1911</v>
+        <v>2004</v>
       </c>
       <c r="G256" s="12" t="n">
         <f aca="false">IF(OR(D256="—",D256="",K256=""),"",COUNTIF($J$2:$J$259,J256)-1)</f>
@@ -48684,7 +48699,7 @@
       </c>
       <c r="H256" s="14"/>
       <c r="I256" s="13" t="s">
-        <v>2002</v>
+        <v>2005</v>
       </c>
       <c r="J256" s="5" t="str">
         <f aca="false">K256&amp;"|"&amp;D256&amp;"|"&amp;E256</f>
@@ -48715,7 +48730,7 @@
         <v>1340</v>
       </c>
       <c r="F257" s="13" t="s">
-        <v>1900</v>
+        <v>2006</v>
       </c>
       <c r="G257" s="12" t="n">
         <f aca="false">IF(OR(D257="—",D257="",K257=""),"",COUNTIF($J$2:$J$259,J257)-1)</f>
@@ -48723,7 +48738,7 @@
       </c>
       <c r="H257" s="14"/>
       <c r="I257" s="13" t="s">
-        <v>2003</v>
+        <v>2007</v>
       </c>
       <c r="J257" s="5" t="str">
         <f aca="false">K257&amp;"|"&amp;D257&amp;"|"&amp;E257</f>
@@ -48754,7 +48769,7 @@
         <v>1340</v>
       </c>
       <c r="F258" s="13" t="s">
-        <v>2004</v>
+        <v>2008</v>
       </c>
       <c r="G258" s="12" t="n">
         <f aca="false">IF(OR(D258="—",D258="",K258=""),"",COUNTIF($J$2:$J$259,J258)-1)</f>
@@ -48762,7 +48777,7 @@
       </c>
       <c r="H258" s="14"/>
       <c r="I258" s="13" t="s">
-        <v>2005</v>
+        <v>2009</v>
       </c>
       <c r="J258" s="5" t="str">
         <f aca="false">K258&amp;"|"&amp;D258&amp;"|"&amp;E258</f>
@@ -48793,7 +48808,7 @@
         <v>1340</v>
       </c>
       <c r="F259" s="13" t="s">
-        <v>1907</v>
+        <v>2010</v>
       </c>
       <c r="G259" s="12" t="n">
         <f aca="false">IF(OR(D259="—",D259="",K259=""),"",COUNTIF($J$2:$J$259,J259)-1)</f>
@@ -48801,7 +48816,7 @@
       </c>
       <c r="H259" s="14"/>
       <c r="I259" s="13" t="s">
-        <v>2006</v>
+        <v>2011</v>
       </c>
       <c r="J259" s="5" t="str">
         <f aca="false">K259&amp;"|"&amp;D259&amp;"|"&amp;E259</f>
@@ -48870,19 +48885,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>2007</v>
+        <v>2012</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>2008</v>
+        <v>2013</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2009</v>
+        <v>2014</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2010</v>
+        <v>2015</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>2011</v>
+        <v>2016</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>1326</v>
@@ -48891,22 +48906,22 @@
         <v>939</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>2012</v>
+        <v>2017</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>2013</v>
+        <v>2018</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>2014</v>
+        <v>2019</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>2017</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -48914,10 +48929,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>2018</v>
+        <v>2023</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>2019</v>
+        <v>2024</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>1066</v>
@@ -48935,7 +48950,7 @@
         <v>129</v>
       </c>
       <c r="I2" s="15" t="s">
-        <v>2020</v>
+        <v>2025</v>
       </c>
       <c r="J2" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E2&amp;", *",'Ingredient Feel'!$B$2:$B$259,D2,'Ingredient Feel'!$D$2:$D$259,F2,'Ingredient Feel'!$E$2:$E$259,G2)</f>
@@ -48950,7 +48965,7 @@
         <v>8</v>
       </c>
       <c r="M2" s="13" t="s">
-        <v>2021</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -48958,16 +48973,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>2023</v>
+        <v>2028</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>2024</v>
+        <v>2029</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>1344</v>
@@ -48979,7 +48994,7 @@
         <v>604</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>2025</v>
+        <v>2030</v>
       </c>
       <c r="J3" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E3&amp;", *",'Ingredient Feel'!$B$2:$B$259,D3,'Ingredient Feel'!$D$2:$D$259,F3,'Ingredient Feel'!$E$2:$E$259,G3)</f>
@@ -48994,7 +49009,7 @@
         <v>3</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>2026</v>
+        <v>2031</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49002,16 +49017,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>2028</v>
+        <v>2033</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>2029</v>
+        <v>2034</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>1344</v>
@@ -49023,7 +49038,7 @@
         <v>718</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>2030</v>
+        <v>2035</v>
       </c>
       <c r="J4" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E4&amp;", *",'Ingredient Feel'!$B$2:$B$259,D4,'Ingredient Feel'!$D$2:$D$259,F4,'Ingredient Feel'!$E$2:$E$259,G4)</f>
@@ -49038,7 +49053,7 @@
         <v>3</v>
       </c>
       <c r="M4" s="13" t="s">
-        <v>2031</v>
+        <v>2036</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49046,16 +49061,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>2032</v>
+        <v>2037</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>2033</v>
+        <v>2038</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>2029</v>
+        <v>2034</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>1335</v>
@@ -49067,7 +49082,7 @@
         <v>467</v>
       </c>
       <c r="I5" s="15" t="s">
-        <v>2034</v>
+        <v>2039</v>
       </c>
       <c r="J5" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E5&amp;", *",'Ingredient Feel'!$B$2:$B$259,D5,'Ingredient Feel'!$D$2:$D$259,F5,'Ingredient Feel'!$E$2:$E$259,G5)</f>
@@ -49082,7 +49097,7 @@
         <v>3</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>2035</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49090,10 +49105,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>2036</v>
+        <v>2041</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>1066</v>
@@ -49111,7 +49126,7 @@
         <v>624</v>
       </c>
       <c r="I6" s="15" t="s">
-        <v>2037</v>
+        <v>2042</v>
       </c>
       <c r="J6" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E6&amp;", *",'Ingredient Feel'!$B$2:$B$259,D6,'Ingredient Feel'!$D$2:$D$259,F6,'Ingredient Feel'!$E$2:$E$259,G6)</f>
@@ -49126,7 +49141,7 @@
         <v>8</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>2038</v>
+        <v>2043</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49134,10 +49149,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>2039</v>
+        <v>2044</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>1066</v>
@@ -49155,7 +49170,7 @@
         <v>115</v>
       </c>
       <c r="I7" s="15" t="s">
-        <v>2040</v>
+        <v>2045</v>
       </c>
       <c r="J7" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E7&amp;", *",'Ingredient Feel'!$B$2:$B$259,D7,'Ingredient Feel'!$D$2:$D$259,F7,'Ingredient Feel'!$E$2:$E$259,G7)</f>
@@ -49170,7 +49185,7 @@
         <v>7</v>
       </c>
       <c r="M7" s="13" t="s">
-        <v>2041</v>
+        <v>2046</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49178,10 +49193,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>2042</v>
+        <v>2047</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>1066</v>
@@ -49199,7 +49214,7 @@
         <v>596</v>
       </c>
       <c r="I8" s="15" t="s">
-        <v>2043</v>
+        <v>2048</v>
       </c>
       <c r="J8" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E8&amp;", *",'Ingredient Feel'!$B$2:$B$259,D8,'Ingredient Feel'!$D$2:$D$259,F8,'Ingredient Feel'!$E$2:$E$259,G8)</f>
@@ -49214,7 +49229,7 @@
         <v>7</v>
       </c>
       <c r="M8" s="13" t="s">
-        <v>2044</v>
+        <v>2049</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49222,16 +49237,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>2045</v>
+        <v>2050</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>2046</v>
+        <v>2051</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>2047</v>
+        <v>2052</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>1335</v>
@@ -49243,7 +49258,7 @@
         <v>184</v>
       </c>
       <c r="I9" s="15" t="s">
-        <v>2048</v>
+        <v>2053</v>
       </c>
       <c r="J9" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E9&amp;", *",'Ingredient Feel'!$B$2:$B$259,D9,'Ingredient Feel'!$D$2:$D$259,F9,'Ingredient Feel'!$E$2:$E$259,G9)</f>
@@ -49258,7 +49273,7 @@
         <v>2</v>
       </c>
       <c r="M9" s="13" t="s">
-        <v>2049</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49266,10 +49281,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>2050</v>
+        <v>2055</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>2051</v>
+        <v>2056</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>1066</v>
@@ -49287,7 +49302,7 @@
         <v>99</v>
       </c>
       <c r="I10" s="15" t="s">
-        <v>2052</v>
+        <v>2057</v>
       </c>
       <c r="J10" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E10&amp;", *",'Ingredient Feel'!$B$2:$B$259,D10,'Ingredient Feel'!$D$2:$D$259,F10,'Ingredient Feel'!$E$2:$E$259,G10)</f>
@@ -49302,7 +49317,7 @@
         <v>4</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>2053</v>
+        <v>2058</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49310,10 +49325,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>2050</v>
+        <v>2055</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>2054</v>
+        <v>2059</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>1066</v>
@@ -49331,7 +49346,7 @@
         <v>71</v>
       </c>
       <c r="I11" s="15" t="s">
-        <v>2055</v>
+        <v>2060</v>
       </c>
       <c r="J11" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E11&amp;", *",'Ingredient Feel'!$B$2:$B$259,D11,'Ingredient Feel'!$D$2:$D$259,F11,'Ingredient Feel'!$E$2:$E$259,G11)</f>
@@ -49346,7 +49361,7 @@
         <v>4</v>
       </c>
       <c r="M11" s="13" t="s">
-        <v>2056</v>
+        <v>2061</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49354,10 +49369,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>2057</v>
+        <v>2062</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>1066</v>
@@ -49375,7 +49390,7 @@
         <v>227</v>
       </c>
       <c r="I12" s="15" t="s">
-        <v>2058</v>
+        <v>2063</v>
       </c>
       <c r="J12" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E12&amp;", *",'Ingredient Feel'!$B$2:$B$259,D12,'Ingredient Feel'!$D$2:$D$259,F12,'Ingredient Feel'!$E$2:$E$259,G12)</f>
@@ -49390,7 +49405,7 @@
         <v>8</v>
       </c>
       <c r="M12" s="13" t="s">
-        <v>2059</v>
+        <v>2064</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49398,10 +49413,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>2060</v>
+        <v>2065</v>
       </c>
       <c r="D13" s="14" t="s">
         <v>1066</v>
@@ -49419,7 +49434,7 @@
         <v>500</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>2061</v>
+        <v>2066</v>
       </c>
       <c r="J13" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E13&amp;", *",'Ingredient Feel'!$B$2:$B$259,D13,'Ingredient Feel'!$D$2:$D$259,F13,'Ingredient Feel'!$E$2:$E$259,G13)</f>
@@ -49434,7 +49449,7 @@
         <v>8</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>2062</v>
+        <v>2067</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49442,10 +49457,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>2063</v>
+        <v>2068</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>1066</v>
@@ -49463,7 +49478,7 @@
         <v>480</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>2064</v>
+        <v>2069</v>
       </c>
       <c r="J14" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E14&amp;", *",'Ingredient Feel'!$B$2:$B$259,D14,'Ingredient Feel'!$D$2:$D$259,F14,'Ingredient Feel'!$E$2:$E$259,G14)</f>
@@ -49478,7 +49493,7 @@
         <v>2</v>
       </c>
       <c r="M14" s="13" t="s">
-        <v>2065</v>
+        <v>2070</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49486,10 +49501,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>2066</v>
+        <v>2071</v>
       </c>
       <c r="D15" s="14" t="s">
         <v>1066</v>
@@ -49507,7 +49522,7 @@
         <v>355</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>2067</v>
+        <v>2072</v>
       </c>
       <c r="J15" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E15&amp;", *",'Ingredient Feel'!$B$2:$B$259,D15,'Ingredient Feel'!$D$2:$D$259,F15,'Ingredient Feel'!$E$2:$E$259,G15)</f>
@@ -49522,7 +49537,7 @@
         <v>2</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>2068</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49530,10 +49545,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>2069</v>
+        <v>2074</v>
       </c>
       <c r="D16" s="14" t="s">
         <v>1066</v>
@@ -49551,7 +49566,7 @@
         <v>243</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>2070</v>
+        <v>2075</v>
       </c>
       <c r="J16" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E16&amp;", *",'Ingredient Feel'!$B$2:$B$259,D16,'Ingredient Feel'!$D$2:$D$259,F16,'Ingredient Feel'!$E$2:$E$259,G16)</f>
@@ -49566,7 +49581,7 @@
         <v>2</v>
       </c>
       <c r="M16" s="13" t="s">
-        <v>2071</v>
+        <v>2076</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49574,16 +49589,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>2072</v>
+        <v>2077</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>2073</v>
+        <v>2078</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>2074</v>
+        <v>2079</v>
       </c>
       <c r="F17" s="14" t="s">
         <v>1335</v>
@@ -49595,7 +49610,7 @@
         <v>229</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>2075</v>
+        <v>2080</v>
       </c>
       <c r="J17" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E17&amp;", *",'Ingredient Feel'!$B$2:$B$259,D17,'Ingredient Feel'!$D$2:$D$259,F17,'Ingredient Feel'!$E$2:$E$259,G17)</f>
@@ -49610,7 +49625,7 @@
         <v>2</v>
       </c>
       <c r="M17" s="13" t="s">
-        <v>2076</v>
+        <v>2081</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49618,16 +49633,16 @@
         <v>17</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>2077</v>
+        <v>2082</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>2078</v>
+        <v>2083</v>
       </c>
       <c r="F18" s="14" t="s">
         <v>1335</v>
@@ -49639,7 +49654,7 @@
         <v>459</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>2079</v>
+        <v>2084</v>
       </c>
       <c r="J18" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E18&amp;", *",'Ingredient Feel'!$B$2:$B$259,D18,'Ingredient Feel'!$D$2:$D$259,F18,'Ingredient Feel'!$E$2:$E$259,G18)</f>
@@ -49654,7 +49669,7 @@
         <v>3</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>2080</v>
+        <v>2085</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49662,16 +49677,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>2081</v>
+        <v>2086</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>1066</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>2082</v>
+        <v>2087</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>1335</v>
@@ -49683,7 +49698,7 @@
         <v>468</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>2083</v>
+        <v>2088</v>
       </c>
       <c r="J19" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E19&amp;", *",'Ingredient Feel'!$B$2:$B$259,D19,'Ingredient Feel'!$D$2:$D$259,F19,'Ingredient Feel'!$E$2:$E$259,G19)</f>
@@ -49698,7 +49713,7 @@
         <v>3</v>
       </c>
       <c r="M19" s="13" t="s">
-        <v>2084</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49706,10 +49721,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>2085</v>
+        <v>2090</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>2086</v>
+        <v>2091</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>1196</v>
@@ -49727,7 +49742,7 @@
         <v>337</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>2087</v>
+        <v>2092</v>
       </c>
       <c r="J20" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E20&amp;", *",'Ingredient Feel'!$B$2:$B$259,D20,'Ingredient Feel'!$D$2:$D$259,F20,'Ingredient Feel'!$E$2:$E$259,G20)</f>
@@ -49742,7 +49757,7 @@
         <v>2</v>
       </c>
       <c r="M20" s="13" t="s">
-        <v>2088</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49750,16 +49765,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>2089</v>
+        <v>2094</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>1196</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>2090</v>
+        <v>2095</v>
       </c>
       <c r="F21" s="14" t="s">
         <v>1344</v>
@@ -49771,7 +49786,7 @@
         <v>213</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>2091</v>
+        <v>2096</v>
       </c>
       <c r="J21" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E21&amp;", *",'Ingredient Feel'!$B$2:$B$259,D21,'Ingredient Feel'!$D$2:$D$259,F21,'Ingredient Feel'!$E$2:$E$259,G21)</f>
@@ -49786,7 +49801,7 @@
         <v>2</v>
       </c>
       <c r="M21" s="13" t="s">
-        <v>2092</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49794,16 +49809,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>2093</v>
+        <v>2098</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>1196</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>2090</v>
+        <v>2095</v>
       </c>
       <c r="F22" s="14" t="s">
         <v>1335</v>
@@ -49815,7 +49830,7 @@
         <v>614</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>2094</v>
+        <v>2099</v>
       </c>
       <c r="J22" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E22&amp;", *",'Ingredient Feel'!$B$2:$B$259,D22,'Ingredient Feel'!$D$2:$D$259,F22,'Ingredient Feel'!$E$2:$E$259,G22)</f>
@@ -49830,7 +49845,7 @@
         <v>2</v>
       </c>
       <c r="M22" s="13" t="s">
-        <v>2095</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49838,16 +49853,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>2096</v>
+        <v>2101</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>2097</v>
+        <v>2102</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>1196</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>2098</v>
+        <v>2103</v>
       </c>
       <c r="F23" s="14" t="s">
         <v>1344</v>
@@ -49859,7 +49874,7 @@
         <v>88</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>2099</v>
+        <v>2104</v>
       </c>
       <c r="J23" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E23&amp;", *",'Ingredient Feel'!$B$2:$B$259,D23,'Ingredient Feel'!$D$2:$D$259,F23,'Ingredient Feel'!$E$2:$E$259,G23)</f>
@@ -49874,7 +49889,7 @@
         <v>3</v>
       </c>
       <c r="M23" s="13" t="s">
-        <v>2100</v>
+        <v>2105</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49882,16 +49897,16 @@
         <v>23</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>2101</v>
+        <v>2106</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>1196</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>2098</v>
+        <v>2103</v>
       </c>
       <c r="F24" s="14" t="s">
         <v>1335</v>
@@ -49903,7 +49918,7 @@
         <v>131</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>2102</v>
+        <v>2107</v>
       </c>
       <c r="J24" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E24&amp;", *",'Ingredient Feel'!$B$2:$B$259,D24,'Ingredient Feel'!$D$2:$D$259,F24,'Ingredient Feel'!$E$2:$E$259,G24)</f>
@@ -49918,7 +49933,7 @@
         <v>3</v>
       </c>
       <c r="M24" s="13" t="s">
-        <v>2103</v>
+        <v>2108</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49926,16 +49941,16 @@
         <v>24</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>2104</v>
+        <v>2109</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>1196</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>2082</v>
+        <v>2087</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>1335</v>
@@ -49947,7 +49962,7 @@
         <v>586</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>2105</v>
+        <v>2110</v>
       </c>
       <c r="J25" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E25&amp;", *",'Ingredient Feel'!$B$2:$B$259,D25,'Ingredient Feel'!$D$2:$D$259,F25,'Ingredient Feel'!$E$2:$E$259,G25)</f>
@@ -49962,7 +49977,7 @@
         <v>3</v>
       </c>
       <c r="M25" s="13" t="s">
-        <v>2106</v>
+        <v>2111</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -49970,10 +49985,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>2107</v>
+        <v>2112</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>1196</v>
@@ -49991,7 +50006,7 @@
         <v>290</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>2108</v>
+        <v>2113</v>
       </c>
       <c r="J26" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E26&amp;", *",'Ingredient Feel'!$B$2:$B$259,D26,'Ingredient Feel'!$D$2:$D$259,F26,'Ingredient Feel'!$E$2:$E$259,G26)</f>
@@ -50006,7 +50021,7 @@
         <v>7</v>
       </c>
       <c r="M26" s="13" t="s">
-        <v>2109</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -50014,10 +50029,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>2027</v>
+        <v>2032</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>2110</v>
+        <v>2115</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>1196</v>
@@ -50035,7 +50050,7 @@
         <v>262</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>2111</v>
+        <v>2116</v>
       </c>
       <c r="J27" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E27&amp;", *",'Ingredient Feel'!$B$2:$B$259,D27,'Ingredient Feel'!$D$2:$D$259,F27,'Ingredient Feel'!$E$2:$E$259,G27)</f>
@@ -50050,7 +50065,7 @@
         <v>3</v>
       </c>
       <c r="M27" s="13" t="s">
-        <v>2112</v>
+        <v>2117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -50058,16 +50073,16 @@
         <v>27</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>2022</v>
+        <v>2027</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>2113</v>
+        <v>2118</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>1196</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>2114</v>
+        <v>2119</v>
       </c>
       <c r="F28" s="14" t="s">
         <v>1335</v>
@@ -50079,7 +50094,7 @@
         <v>446</v>
       </c>
       <c r="I28" s="15" t="s">
-        <v>2115</v>
+        <v>2120</v>
       </c>
       <c r="J28" s="16" t="n">
         <f aca="false">COUNTIFS('Ingredient Feel'!$L$2:$L$259,"*, "&amp;E28&amp;", *",'Ingredient Feel'!$B$2:$B$259,D28,'Ingredient Feel'!$D$2:$D$259,F28,'Ingredient Feel'!$E$2:$E$259,G28)</f>
@@ -50094,7 +50109,7 @@
         <v>2</v>
       </c>
       <c r="M28" s="13" t="s">
-        <v>2116</v>
+        <v>2121</v>
       </c>
     </row>
   </sheetData>
@@ -50152,7 +50167,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>2117</v>
+        <v>2122</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1040</v>
@@ -50176,7 +50191,7 @@
         <v>15</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>2118</v>
+        <v>2123</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>6</v>
@@ -50192,7 +50207,7 @@
         <v>10</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>2119</v>
+        <v>2124</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>6</v>
@@ -50208,7 +50223,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>2120</v>
+        <v>2125</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>6</v>
@@ -50224,7 +50239,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>2121</v>
+        <v>2126</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>6</v>
@@ -50240,7 +50255,7 @@
         <v>9</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>2122</v>
+        <v>2127</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>6</v>
@@ -50256,7 +50271,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>2123</v>
+        <v>2128</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>6</v>
@@ -50272,7 +50287,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>2124</v>
+        <v>2129</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>6</v>
@@ -50288,7 +50303,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>2125</v>
+        <v>2130</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>6</v>
@@ -50304,7 +50319,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>2126</v>
+        <v>2131</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>6</v>
@@ -50320,7 +50335,7 @@
         <v>13</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>2127</v>
+        <v>2132</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>6</v>
@@ -50336,7 +50351,7 @@
         <v>17</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>2128</v>
+        <v>2133</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>6</v>
@@ -50352,7 +50367,7 @@
         <v>9</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>2129</v>
+        <v>2134</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>6</v>
@@ -50368,7 +50383,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>2130</v>
+        <v>2135</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>6</v>
@@ -50384,7 +50399,7 @@
         <v>9</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>2131</v>
+        <v>2136</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>6</v>
@@ -50400,7 +50415,7 @@
         <v>10</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>2132</v>
+        <v>2137</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>6</v>
@@ -50443,7 +50458,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>2133</v>
+        <v>2138</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>1040</v>
@@ -50467,7 +50482,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>2134</v>
+        <v>2139</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>6</v>
@@ -50483,7 +50498,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>2135</v>
+        <v>2140</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>6</v>
@@ -50499,7 +50514,7 @@
         <v>7</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>2136</v>
+        <v>2141</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>6</v>
@@ -50515,7 +50530,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>2137</v>
+        <v>2142</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>6</v>
@@ -50531,7 +50546,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>2138</v>
+        <v>2143</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>6</v>
@@ -50547,7 +50562,7 @@
         <v>7</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>2139</v>
+        <v>2144</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>6</v>
@@ -50563,7 +50578,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>2140</v>
+        <v>2145</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>6</v>
@@ -50579,7 +50594,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>2141</v>
+        <v>2146</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>6</v>
@@ -50595,7 +50610,7 @@
         <v>10</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>2142</v>
+        <v>2147</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>6</v>
@@ -50611,7 +50626,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>2143</v>
+        <v>2148</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>6</v>
@@ -50627,7 +50642,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>2144</v>
+        <v>2149</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>6</v>
@@ -50643,7 +50658,7 @@
         <v>5</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>2145</v>
+        <v>2150</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>6</v>
@@ -50659,7 +50674,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>2146</v>
+        <v>2151</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>6</v>
@@ -50675,7 +50690,7 @@
         <v>6</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>2147</v>
+        <v>2152</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>6</v>
@@ -50691,7 +50706,7 @@
         <v>7</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>2148</v>
+        <v>2153</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>6</v>
@@ -50707,7 +50722,7 @@
         <v>6</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>2149</v>
+        <v>2154</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>6</v>
@@ -50723,7 +50738,7 @@
         <v>5</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>2150</v>
+        <v>2155</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>6</v>
@@ -50739,7 +50754,7 @@
         <v>9</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>2151</v>
+        <v>2156</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>6</v>
@@ -50755,7 +50770,7 @@
         <v>6</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>2152</v>
+        <v>2157</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>6</v>
@@ -50771,7 +50786,7 @@
         <v>11</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>2153</v>
+        <v>2158</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>6</v>
@@ -50787,7 +50802,7 @@
         <v>8</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>2154</v>
+        <v>2159</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>6</v>
@@ -50803,7 +50818,7 @@
         <v>6</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>2155</v>
+        <v>2160</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>6</v>
@@ -50846,10 +50861,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>2156</v>
+        <v>2161</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>2157</v>
+        <v>2162</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>1041</v>
@@ -50863,13 +50878,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>2158</v>
+        <v>2163</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>2160</v>
+        <v>2165</v>
       </c>
       <c r="D2" s="11" t="s">
         <v>6</v>
@@ -50881,10 +50896,10 @@
         <v>994</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>2161</v>
+        <v>2166</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>6</v>
@@ -50896,10 +50911,10 @@
         <v>970</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>2162</v>
+        <v>2167</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>6</v>
@@ -50908,13 +50923,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>2163</v>
+        <v>2168</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>2164</v>
+        <v>2169</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>6</v>
@@ -50926,10 +50941,10 @@
         <v>999</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>2165</v>
+        <v>2170</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>6</v>
@@ -50941,10 +50956,10 @@
         <v>884</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>2166</v>
+        <v>2171</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>6</v>
@@ -50956,10 +50971,10 @@
         <v>996</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>2167</v>
+        <v>2172</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>6</v>
@@ -50968,13 +50983,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>2168</v>
+        <v>2173</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>2169</v>
+        <v>2174</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>6</v>
@@ -50986,10 +51001,10 @@
         <v>1000</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>2159</v>
+        <v>2164</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>2170</v>
+        <v>2175</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>6</v>
@@ -50998,13 +51013,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>2171</v>
+        <v>2176</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>2173</v>
+        <v>2178</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>6</v>
@@ -51013,13 +51028,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>2174</v>
+        <v>2179</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>2175</v>
+        <v>2180</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>6</v>
@@ -51028,13 +51043,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>2176</v>
+        <v>2181</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>2177</v>
+        <v>2182</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>6</v>
@@ -51043,13 +51058,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>2178</v>
+        <v>2183</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>2179</v>
+        <v>2184</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>6</v>
@@ -51058,13 +51073,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>2180</v>
+        <v>2185</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>2181</v>
+        <v>2186</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>6</v>
@@ -51076,10 +51091,10 @@
         <v>133</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>2182</v>
+        <v>2187</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>6</v>
@@ -51088,13 +51103,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>2183</v>
+        <v>2188</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>2184</v>
+        <v>2189</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>6</v>
@@ -51103,13 +51118,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>2185</v>
+        <v>2190</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>2186</v>
+        <v>2191</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>6</v>
@@ -51118,13 +51133,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>2187</v>
+        <v>2192</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>2188</v>
+        <v>2193</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>6</v>
@@ -51133,13 +51148,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>2189</v>
+        <v>2194</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>2190</v>
+        <v>2195</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>6</v>
@@ -51148,13 +51163,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>2191</v>
+        <v>2196</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>2192</v>
+        <v>2197</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>6</v>
@@ -51163,13 +51178,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>2193</v>
+        <v>2198</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>2194</v>
+        <v>2199</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>6</v>
@@ -51178,13 +51193,13 @@
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>2195</v>
+        <v>2200</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>2196</v>
+        <v>2201</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>6</v>
@@ -51193,13 +51208,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>2197</v>
+        <v>2202</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>2172</v>
+        <v>2177</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>2198</v>
+        <v>2203</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>6</v>
@@ -51211,10 +51226,10 @@
         <v>977</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>2200</v>
+        <v>2205</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>6</v>
@@ -51226,10 +51241,10 @@
         <v>903</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>2201</v>
+        <v>2206</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>6</v>
@@ -51241,10 +51256,10 @@
         <v>957</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>2202</v>
+        <v>2207</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>6</v>
@@ -51256,10 +51271,10 @@
         <v>922</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>2203</v>
+        <v>2208</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>6</v>
@@ -51271,10 +51286,10 @@
         <v>878</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>2204</v>
+        <v>2209</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>6</v>
@@ -51286,10 +51301,10 @@
         <v>933</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>2205</v>
+        <v>2210</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>6</v>
@@ -51301,10 +51316,10 @@
         <v>986</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>2199</v>
+        <v>2204</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>2206</v>
+        <v>2211</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>6</v>
@@ -51316,10 +51331,10 @@
         <v>1001</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>2207</v>
+        <v>2212</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>2208</v>
+        <v>2213</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>6</v>
@@ -51328,13 +51343,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>2209</v>
+        <v>2214</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>2207</v>
+        <v>2212</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>2210</v>
+        <v>2215</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>6</v>
@@ -51346,10 +51361,10 @@
         <v>978</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>2207</v>
+        <v>2212</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>2211</v>
+        <v>2216</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>6</v>
@@ -51361,10 +51376,10 @@
         <v>983</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>2207</v>
+        <v>2212</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>2212</v>
+        <v>2217</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>6</v>
@@ -51376,10 +51391,10 @@
         <v>1015</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>2214</v>
+        <v>2219</v>
       </c>
       <c r="D36" s="11" t="s">
         <v>6</v>
@@ -51388,13 +51403,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>2215</v>
+        <v>2220</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>2216</v>
+        <v>2221</v>
       </c>
       <c r="D37" s="11" t="s">
         <v>6</v>
@@ -51406,10 +51421,10 @@
         <v>1017</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>2217</v>
+        <v>2222</v>
       </c>
       <c r="D38" s="11" t="s">
         <v>6</v>
@@ -51421,10 +51436,10 @@
         <v>971</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>2218</v>
+        <v>2223</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>6</v>
@@ -51436,10 +51451,10 @@
         <v>1028</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>2219</v>
+        <v>2224</v>
       </c>
       <c r="D40" s="11" t="s">
         <v>6</v>
@@ -51451,10 +51466,10 @@
         <v>930</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>2220</v>
+        <v>2225</v>
       </c>
       <c r="D41" s="11" t="s">
         <v>6</v>
@@ -51466,10 +51481,10 @@
         <v>1023</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>2221</v>
+        <v>2226</v>
       </c>
       <c r="D42" s="11" t="s">
         <v>6</v>
@@ -51481,10 +51496,10 @@
         <v>998</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>2222</v>
+        <v>2227</v>
       </c>
       <c r="D43" s="11" t="s">
         <v>6</v>
@@ -51496,10 +51511,10 @@
         <v>1021</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>2223</v>
+        <v>2228</v>
       </c>
       <c r="D44" s="11" t="s">
         <v>6</v>
@@ -51511,10 +51526,10 @@
         <v>1037</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>2213</v>
+        <v>2218</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>2224</v>
+        <v>2229</v>
       </c>
       <c r="D45" s="11" t="s">
         <v>6</v>
@@ -51526,10 +51541,10 @@
         <v>991</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>2226</v>
+        <v>2231</v>
       </c>
       <c r="D46" s="11" t="s">
         <v>6</v>
@@ -51541,10 +51556,10 @@
         <v>960</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>2227</v>
+        <v>2232</v>
       </c>
       <c r="D47" s="11" t="s">
         <v>6</v>
@@ -51556,10 +51571,10 @@
         <v>918</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>2228</v>
+        <v>2233</v>
       </c>
       <c r="D48" s="11" t="s">
         <v>6</v>
@@ -51571,10 +51586,10 @@
         <v>955</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C49" s="10" t="s">
-        <v>2229</v>
+        <v>2234</v>
       </c>
       <c r="D49" s="11" t="s">
         <v>6</v>
@@ -51586,10 +51601,10 @@
         <v>892</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C50" s="10" t="s">
-        <v>2230</v>
+        <v>2235</v>
       </c>
       <c r="D50" s="11" t="s">
         <v>6</v>
@@ -51601,10 +51616,10 @@
         <v>967</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C51" s="10" t="s">
-        <v>2231</v>
+        <v>2236</v>
       </c>
       <c r="D51" s="11" t="s">
         <v>6</v>
@@ -51616,10 +51631,10 @@
         <v>937</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C52" s="10" t="s">
-        <v>2232</v>
+        <v>2237</v>
       </c>
       <c r="D52" s="11" t="s">
         <v>6</v>
@@ -51631,10 +51646,10 @@
         <v>964</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>2225</v>
+        <v>2230</v>
       </c>
       <c r="C53" s="10" t="s">
-        <v>2233</v>
+        <v>2238</v>
       </c>
       <c r="D53" s="11" t="s">
         <v>6</v>

</xml_diff>

<commit_message>
Blue shows calm first, so the first puzzle's thread is findable
Blue (colour and thread) now reads calm · truth · memory instead of
truth first. It is the only thread whose visible keyword is calm,
which points straight at #179's thread.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -5892,7 +5892,7 @@
     <t xml:space="preserve">banishing,endings,protection</t>
   </si>
   <si>
-    <t xml:space="preserve">truth, memory, calm</t>
+    <t xml:space="preserve">calm, truth, memory</t>
   </si>
   <si>
     <t xml:space="preserve">Stitched into a diary's spine so it stays honest.</t>
@@ -8095,7 +8095,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -8162,18 +8162,6 @@
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -48707,7 +48695,7 @@
       </c>
       <c r="L200" s="5" t="str">
         <f aca="false">", "&amp;C200&amp;", "</f>
-        <v>, truth, memory, calm, </v>
+        <v>, calm, truth, memory, </v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -52207,74 +52195,74 @@
   <dimension ref="A1:P150"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="22"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>2123</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="4" t="s">
         <v>2124</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="4" t="s">
         <v>2125</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="4" t="s">
         <v>2126</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="4" t="s">
         <v>2127</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="4" t="s">
         <v>2128</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="4" t="s">
         <v>2129</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="4" t="s">
         <v>2013</v>
       </c>
-      <c r="I1" s="17" t="s">
+      <c r="I1" s="4" t="s">
         <v>2130</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="4" t="s">
         <v>2131</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="K1" s="4" t="s">
         <v>868</v>
       </c>
-      <c r="L1" s="17" t="s">
+      <c r="L1" s="4" t="s">
         <v>2132</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="4" t="s">
         <v>2133</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="N1" s="4" t="s">
         <v>2134</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="O1" s="4" t="s">
         <v>2135</v>
       </c>
-      <c r="P1" s="17" t="s">
+      <c r="P1" s="4" t="s">
         <v>2136</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
@@ -52321,7 +52309,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="n">
         <v>1</v>
       </c>
@@ -52368,7 +52356,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="n">
         <v>2</v>
       </c>
@@ -52415,7 +52403,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="n">
         <v>3</v>
       </c>
@@ -52462,7 +52450,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
         <v>4</v>
       </c>
@@ -52509,7 +52497,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
         <v>5</v>
       </c>
@@ -52556,7 +52544,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
         <v>6</v>
       </c>
@@ -52603,7 +52591,7 @@
         <v>2142</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
         <v>7</v>
       </c>
@@ -52650,7 +52638,7 @@
         <v>2152</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="n">
         <v>8</v>
       </c>
@@ -52697,7 +52685,7 @@
       </c>
       <c r="P10" s="13"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
@@ -52744,7 +52732,7 @@
       </c>
       <c r="P11" s="13"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="n">
         <v>9</v>
       </c>
@@ -52793,7 +52781,7 @@
       </c>
       <c r="P12" s="13"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="n">
         <v>9</v>
       </c>
@@ -52840,7 +52828,7 @@
       </c>
       <c r="P13" s="13"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="n">
         <v>10</v>
       </c>
@@ -52887,7 +52875,7 @@
       </c>
       <c r="P14" s="13"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="n">
         <v>10</v>
       </c>
@@ -52934,7 +52922,7 @@
       </c>
       <c r="P15" s="13"/>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="n">
         <v>11</v>
       </c>
@@ -52981,7 +52969,7 @@
       </c>
       <c r="P16" s="13"/>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="n">
         <v>11</v>
       </c>
@@ -53028,7 +53016,7 @@
       </c>
       <c r="P17" s="13"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="n">
         <v>12</v>
       </c>
@@ -53075,7 +53063,7 @@
       </c>
       <c r="P18" s="13"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="n">
         <v>12</v>
       </c>
@@ -53122,7 +53110,7 @@
       </c>
       <c r="P19" s="13"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="n">
         <v>13</v>
       </c>
@@ -53169,7 +53157,7 @@
       </c>
       <c r="P20" s="13"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="n">
         <v>13</v>
       </c>
@@ -53214,7 +53202,7 @@
       <c r="O21" s="13"/>
       <c r="P21" s="13"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="n">
         <v>14</v>
       </c>
@@ -53261,7 +53249,7 @@
       </c>
       <c r="P22" s="13"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="n">
         <v>14</v>
       </c>
@@ -53308,7 +53296,7 @@
       </c>
       <c r="P23" s="13"/>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="n">
         <v>15</v>
       </c>
@@ -53357,7 +53345,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="n">
         <v>15</v>
       </c>
@@ -53402,7 +53390,7 @@
       <c r="O25" s="13"/>
       <c r="P25" s="13"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="n">
         <v>16</v>
       </c>
@@ -53447,7 +53435,7 @@
       <c r="O26" s="13"/>
       <c r="P26" s="13"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="n">
         <v>16</v>
       </c>
@@ -53492,7 +53480,7 @@
       <c r="O27" s="13"/>
       <c r="P27" s="13"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="n">
         <v>17</v>
       </c>
@@ -53539,7 +53527,7 @@
       </c>
       <c r="P28" s="13"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="n">
         <v>17</v>
       </c>
@@ -53584,7 +53572,7 @@
       <c r="O29" s="13"/>
       <c r="P29" s="13"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="n">
         <v>18</v>
       </c>
@@ -53631,7 +53619,7 @@
       <c r="O30" s="13"/>
       <c r="P30" s="13"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="n">
         <v>18</v>
       </c>
@@ -53678,7 +53666,7 @@
       <c r="O31" s="13"/>
       <c r="P31" s="13"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="n">
         <v>19</v>
       </c>
@@ -53725,7 +53713,7 @@
       <c r="O32" s="13"/>
       <c r="P32" s="13"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="n">
         <v>19</v>
       </c>
@@ -53770,7 +53758,7 @@
       <c r="O33" s="13"/>
       <c r="P33" s="13"/>
     </row>
-    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="n">
         <v>20</v>
       </c>
@@ -53817,7 +53805,7 @@
       </c>
       <c r="P34" s="13"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="n">
         <v>20</v>
       </c>
@@ -53862,7 +53850,7 @@
       <c r="O35" s="13"/>
       <c r="P35" s="13"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="n">
         <v>21</v>
       </c>
@@ -53907,7 +53895,7 @@
       <c r="O36" s="13"/>
       <c r="P36" s="13"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="n">
         <v>21</v>
       </c>
@@ -53952,7 +53940,7 @@
       <c r="O37" s="13"/>
       <c r="P37" s="13"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="n">
         <v>22</v>
       </c>
@@ -53999,7 +53987,7 @@
       </c>
       <c r="P38" s="13"/>
     </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="n">
         <v>22</v>
       </c>
@@ -54044,7 +54032,7 @@
       <c r="O39" s="13"/>
       <c r="P39" s="13"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="n">
         <v>23</v>
       </c>
@@ -54091,7 +54079,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="n">
         <v>23</v>
       </c>
@@ -54136,7 +54124,7 @@
       <c r="O41" s="13"/>
       <c r="P41" s="13"/>
     </row>
-    <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="n">
         <v>24</v>
       </c>
@@ -54183,7 +54171,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="n">
         <v>24</v>
       </c>
@@ -54228,7 +54216,7 @@
       <c r="O43" s="13"/>
       <c r="P43" s="13"/>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="n">
         <v>25</v>
       </c>
@@ -54275,7 +54263,7 @@
       </c>
       <c r="P44" s="13"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="n">
         <v>25</v>
       </c>
@@ -54320,7 +54308,7 @@
       <c r="O45" s="13"/>
       <c r="P45" s="13"/>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="n">
         <v>26</v>
       </c>
@@ -54367,7 +54355,7 @@
       </c>
       <c r="P46" s="13"/>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="n">
         <v>26</v>
       </c>
@@ -54414,7 +54402,7 @@
       </c>
       <c r="P47" s="13"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="n">
         <v>27</v>
       </c>
@@ -54459,7 +54447,7 @@
       <c r="O48" s="13"/>
       <c r="P48" s="13"/>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="n">
         <v>27</v>
       </c>
@@ -54504,7 +54492,7 @@
       <c r="O49" s="13"/>
       <c r="P49" s="13"/>
     </row>
-    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="n">
         <v>28</v>
       </c>
@@ -54551,7 +54539,7 @@
       </c>
       <c r="P50" s="13"/>
     </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="n">
         <v>28</v>
       </c>
@@ -54598,7 +54586,7 @@
       </c>
       <c r="P51" s="13"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="n">
         <v>29</v>
       </c>
@@ -54643,7 +54631,7 @@
       <c r="O52" s="13"/>
       <c r="P52" s="13"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="n">
         <v>29</v>
       </c>
@@ -54688,7 +54676,7 @@
       <c r="O53" s="13"/>
       <c r="P53" s="13"/>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="n">
         <v>30</v>
       </c>
@@ -54733,7 +54721,7 @@
       <c r="O54" s="13"/>
       <c r="P54" s="13"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="n">
         <v>30</v>
       </c>
@@ -54778,7 +54766,7 @@
       <c r="O55" s="13"/>
       <c r="P55" s="13"/>
     </row>
-    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="n">
         <v>31</v>
       </c>
@@ -54825,7 +54813,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="n">
         <v>31</v>
       </c>
@@ -54870,7 +54858,7 @@
       <c r="O57" s="13"/>
       <c r="P57" s="13"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="n">
         <v>32</v>
       </c>
@@ -54917,7 +54905,7 @@
       </c>
       <c r="P58" s="13"/>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="n">
         <v>32</v>
       </c>
@@ -54962,7 +54950,7 @@
       <c r="O59" s="13"/>
       <c r="P59" s="13"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="n">
         <v>33</v>
       </c>
@@ -55009,7 +54997,7 @@
       </c>
       <c r="P60" s="13"/>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="n">
         <v>33</v>
       </c>
@@ -55054,7 +55042,7 @@
       <c r="O61" s="13"/>
       <c r="P61" s="13"/>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="n">
         <v>34</v>
       </c>
@@ -55101,7 +55089,7 @@
       </c>
       <c r="P62" s="13"/>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="n">
         <v>34</v>
       </c>
@@ -55148,7 +55136,7 @@
       </c>
       <c r="P63" s="13"/>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="n">
         <v>35</v>
       </c>
@@ -55195,7 +55183,7 @@
       </c>
       <c r="P64" s="13"/>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="n">
         <v>35</v>
       </c>
@@ -55242,7 +55230,7 @@
       <c r="O65" s="13"/>
       <c r="P65" s="13"/>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="12" t="n">
         <v>36</v>
       </c>
@@ -55287,7 +55275,7 @@
       <c r="O66" s="13"/>
       <c r="P66" s="13"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="12" t="n">
         <v>36</v>
       </c>
@@ -55332,7 +55320,7 @@
       <c r="O67" s="13"/>
       <c r="P67" s="13"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="12" t="n">
         <v>37</v>
       </c>
@@ -55379,7 +55367,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="12" t="n">
         <v>37</v>
       </c>
@@ -55422,7 +55410,7 @@
       <c r="O69" s="13"/>
       <c r="P69" s="13"/>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="12" t="n">
         <v>38</v>
       </c>
@@ -55467,7 +55455,7 @@
       <c r="O70" s="13"/>
       <c r="P70" s="13"/>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="n">
         <v>38</v>
       </c>
@@ -55512,7 +55500,7 @@
       <c r="O71" s="13"/>
       <c r="P71" s="13"/>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="n">
         <v>39</v>
       </c>
@@ -55559,7 +55547,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="n">
         <v>39</v>
       </c>
@@ -55604,7 +55592,7 @@
       <c r="O73" s="13"/>
       <c r="P73" s="13"/>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="n">
         <v>40</v>
       </c>
@@ -55647,7 +55635,7 @@
       <c r="O74" s="13"/>
       <c r="P74" s="13"/>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="n">
         <v>40</v>
       </c>
@@ -55692,7 +55680,7 @@
       <c r="O75" s="13"/>
       <c r="P75" s="13"/>
     </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="n">
         <v>41</v>
       </c>
@@ -55737,7 +55725,7 @@
       <c r="O76" s="13"/>
       <c r="P76" s="13"/>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="n">
         <v>41</v>
       </c>
@@ -55780,7 +55768,7 @@
       <c r="O77" s="13"/>
       <c r="P77" s="13"/>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="n">
         <v>42</v>
       </c>
@@ -55825,7 +55813,7 @@
       <c r="O78" s="13"/>
       <c r="P78" s="13"/>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="n">
         <v>42</v>
       </c>
@@ -55868,7 +55856,7 @@
       <c r="O79" s="13"/>
       <c r="P79" s="13"/>
     </row>
-    <row r="80" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="n">
         <v>43</v>
       </c>
@@ -55913,7 +55901,7 @@
       <c r="O80" s="13"/>
       <c r="P80" s="13"/>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="n">
         <v>44</v>
       </c>
@@ -55960,7 +55948,7 @@
       </c>
       <c r="P81" s="13"/>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="n">
         <v>45</v>
       </c>
@@ -56009,7 +55997,7 @@
       </c>
       <c r="P82" s="13"/>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="n">
         <v>45</v>
       </c>
@@ -56054,7 +56042,7 @@
       <c r="O83" s="13"/>
       <c r="P83" s="13"/>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="n">
         <v>46</v>
       </c>
@@ -56097,7 +56085,7 @@
       <c r="O84" s="13"/>
       <c r="P84" s="13"/>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="n">
         <v>47</v>
       </c>
@@ -56144,7 +56132,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="n">
         <v>48</v>
       </c>
@@ -56189,7 +56177,7 @@
       <c r="O86" s="13"/>
       <c r="P86" s="13"/>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="n">
         <v>49</v>
       </c>
@@ -56236,7 +56224,7 @@
       </c>
       <c r="P87" s="13"/>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="n">
         <v>49</v>
       </c>
@@ -56279,7 +56267,7 @@
       <c r="O88" s="13"/>
       <c r="P88" s="13"/>
     </row>
-    <row r="89" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="n">
         <v>50</v>
       </c>
@@ -56324,7 +56312,7 @@
       <c r="O89" s="13"/>
       <c r="P89" s="13"/>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="n">
         <v>51</v>
       </c>
@@ -56367,7 +56355,7 @@
       <c r="O90" s="13"/>
       <c r="P90" s="13"/>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="n">
         <v>52</v>
       </c>
@@ -56414,7 +56402,7 @@
       <c r="O91" s="13"/>
       <c r="P91" s="13"/>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="n">
         <v>53</v>
       </c>
@@ -56459,7 +56447,7 @@
       <c r="O92" s="13"/>
       <c r="P92" s="13"/>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="n">
         <v>53</v>
       </c>
@@ -56502,7 +56490,7 @@
       <c r="O93" s="13"/>
       <c r="P93" s="13"/>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="n">
         <v>54</v>
       </c>
@@ -56547,7 +56535,7 @@
       <c r="O94" s="13"/>
       <c r="P94" s="13"/>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="n">
         <v>55</v>
       </c>
@@ -56594,7 +56582,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="n">
         <v>56</v>
       </c>
@@ -56639,7 +56627,7 @@
       <c r="O96" s="13"/>
       <c r="P96" s="13"/>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="12" t="n">
         <v>57</v>
       </c>
@@ -56682,7 +56670,7 @@
       <c r="O97" s="13"/>
       <c r="P97" s="13"/>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="12" t="n">
         <v>57</v>
       </c>
@@ -56727,7 +56715,7 @@
       <c r="O98" s="13"/>
       <c r="P98" s="13"/>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="12" t="n">
         <v>58</v>
       </c>
@@ -56770,7 +56758,7 @@
       <c r="O99" s="13"/>
       <c r="P99" s="13"/>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="12" t="n">
         <v>59</v>
       </c>
@@ -56815,7 +56803,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="12" t="n">
         <v>60</v>
       </c>
@@ -56858,7 +56846,7 @@
       <c r="O101" s="13"/>
       <c r="P101" s="13"/>
     </row>
-    <row r="102" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="12" t="n">
         <v>61</v>
       </c>
@@ -56903,7 +56891,7 @@
       <c r="O102" s="13"/>
       <c r="P102" s="13"/>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="12" t="n">
         <v>61</v>
       </c>
@@ -56948,7 +56936,7 @@
       <c r="O103" s="13"/>
       <c r="P103" s="13"/>
     </row>
-    <row r="104" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="12" t="n">
         <v>62</v>
       </c>
@@ -56993,7 +56981,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="12" t="n">
         <v>62</v>
       </c>
@@ -57040,7 +57028,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="12" t="n">
         <v>63</v>
       </c>
@@ -57089,7 +57077,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="12" t="n">
         <v>63</v>
       </c>
@@ -57136,7 +57124,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="12" t="n">
         <v>63</v>
       </c>
@@ -57183,7 +57171,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="12" t="n">
         <v>64</v>
       </c>
@@ -57228,7 +57216,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="12" t="n">
         <v>64</v>
       </c>
@@ -57273,7 +57261,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="12" t="n">
         <v>64</v>
       </c>
@@ -57320,7 +57308,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="12" t="n">
         <v>65</v>
       </c>
@@ -57363,7 +57351,7 @@
       <c r="O112" s="13"/>
       <c r="P112" s="13"/>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="12" t="n">
         <v>66</v>
       </c>
@@ -57406,7 +57394,7 @@
       <c r="O113" s="13"/>
       <c r="P113" s="13"/>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="12" t="n">
         <v>67</v>
       </c>
@@ -57449,7 +57437,7 @@
       <c r="O114" s="13"/>
       <c r="P114" s="13"/>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="12" t="n">
         <v>68</v>
       </c>
@@ -57492,7 +57480,7 @@
       <c r="O115" s="13"/>
       <c r="P115" s="13"/>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="12" t="n">
         <v>69</v>
       </c>
@@ -57539,7 +57527,7 @@
       </c>
       <c r="P116" s="13"/>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="12" t="n">
         <v>70</v>
       </c>
@@ -57584,7 +57572,7 @@
       <c r="O117" s="13"/>
       <c r="P117" s="13"/>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="12" t="n">
         <v>71</v>
       </c>
@@ -57629,7 +57617,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="12" t="n">
         <v>71</v>
       </c>
@@ -57676,7 +57664,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="12" t="n">
         <v>72</v>
       </c>
@@ -57719,7 +57707,7 @@
       <c r="O120" s="13"/>
       <c r="P120" s="13"/>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="12" t="n">
         <v>73</v>
       </c>
@@ -57762,7 +57750,7 @@
       <c r="O121" s="13"/>
       <c r="P121" s="13"/>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="12" t="n">
         <v>74</v>
       </c>
@@ -57805,7 +57793,7 @@
       <c r="O122" s="13"/>
       <c r="P122" s="13"/>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="12" t="n">
         <v>75</v>
       </c>
@@ -57850,7 +57838,7 @@
       <c r="O123" s="13"/>
       <c r="P123" s="13"/>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="12" t="n">
         <v>76</v>
       </c>
@@ -57895,7 +57883,7 @@
       <c r="O124" s="13"/>
       <c r="P124" s="13"/>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="12" t="n">
         <v>77</v>
       </c>
@@ -57938,7 +57926,7 @@
       <c r="O125" s="13"/>
       <c r="P125" s="13"/>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="12" t="n">
         <v>78</v>
       </c>
@@ -57983,7 +57971,7 @@
       <c r="O126" s="13"/>
       <c r="P126" s="13"/>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="12" t="n">
         <v>79</v>
       </c>
@@ -58028,7 +58016,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="12" t="n">
         <v>79</v>
       </c>
@@ -58075,7 +58063,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="12" t="n">
         <v>80</v>
       </c>
@@ -58122,7 +58110,7 @@
       </c>
       <c r="P129" s="13"/>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="12" t="n">
         <v>81</v>
       </c>
@@ -58165,7 +58153,7 @@
       <c r="O130" s="13"/>
       <c r="P130" s="13"/>
     </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="12" t="n">
         <v>82</v>
       </c>
@@ -58210,7 +58198,7 @@
       <c r="O131" s="13"/>
       <c r="P131" s="13"/>
     </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="12" t="n">
         <v>83</v>
       </c>
@@ -58253,7 +58241,7 @@
       <c r="O132" s="13"/>
       <c r="P132" s="13"/>
     </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="12" t="n">
         <v>85</v>
       </c>
@@ -58300,7 +58288,7 @@
       </c>
       <c r="P133" s="13"/>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="12" t="n">
         <v>87</v>
       </c>
@@ -58347,7 +58335,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="12" t="n">
         <v>87</v>
       </c>
@@ -58394,7 +58382,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="12" t="n">
         <v>87</v>
       </c>
@@ -58441,7 +58429,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="12" t="n">
         <v>87</v>
       </c>
@@ -58488,7 +58476,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="12" t="n">
         <v>89</v>
       </c>
@@ -58531,7 +58519,7 @@
       <c r="O138" s="13"/>
       <c r="P138" s="13"/>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="12" t="n">
         <v>91</v>
       </c>
@@ -58576,7 +58564,7 @@
       <c r="O139" s="13"/>
       <c r="P139" s="13"/>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="12" t="n">
         <v>91</v>
       </c>
@@ -58619,7 +58607,7 @@
       <c r="O140" s="13"/>
       <c r="P140" s="13"/>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="12" t="n">
         <v>92</v>
       </c>
@@ -58666,7 +58654,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="12" t="n">
         <v>95</v>
       </c>
@@ -58713,7 +58701,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="12" t="n">
         <v>95</v>
       </c>
@@ -58758,7 +58746,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="12" t="n">
         <v>95</v>
       </c>
@@ -58805,7 +58793,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="12" t="n">
         <v>95</v>
       </c>
@@ -58852,7 +58840,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="12" t="n">
         <v>96</v>
       </c>
@@ -58897,7 +58885,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="12" t="n">
         <v>96</v>
       </c>
@@ -58942,7 +58930,7 @@
         <v>2181</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="12" t="n">
         <v>97</v>
       </c>
@@ -58985,7 +58973,7 @@
       <c r="O148" s="13"/>
       <c r="P148" s="13"/>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="12" t="n">
         <v>98</v>
       </c>
@@ -59028,7 +59016,7 @@
       <c r="O149" s="13"/>
       <c r="P149" s="13"/>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="12" t="n">
         <v>99</v>
       </c>
@@ -59100,2221 +59088,2221 @@
   <dimension ref="A1:G90"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="8"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>2267</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="4" t="s">
         <v>2268</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="4" t="s">
         <v>2130</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="4" t="s">
         <v>2269</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="4" t="s">
         <v>2270</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="4" t="s">
         <v>2271</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="4" t="s">
         <v>2272</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="n">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="5" t="s">
         <v>2274</v>
       </c>
-      <c r="D2" s="18" t="n">
+      <c r="D2" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E2" s="18" t="n">
+      <c r="E2" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="18" t="n">
+      <c r="F2" s="5" t="n">
         <f aca="false">D2-E2</f>
         <v>0</v>
       </c>
-      <c r="G2" s="18" t="str">
+      <c r="G2" s="5" t="str">
         <f aca="false">IF(E2&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="n">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="5" t="s">
         <v>2275</v>
       </c>
-      <c r="D3" s="18" t="n">
+      <c r="D3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="5" t="n">
         <f aca="false">D3-E3</f>
         <v>0</v>
       </c>
-      <c r="G3" s="18" t="str">
+      <c r="G3" s="5" t="str">
         <f aca="false">IF(E3&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="n">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="5" t="s">
         <v>2277</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="5" t="n">
         <f aca="false">D4-E4</f>
         <v>0</v>
       </c>
-      <c r="G4" s="18" t="str">
+      <c r="G4" s="5" t="str">
         <f aca="false">IF(E4&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="5" t="s">
         <v>2279</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="5" t="n">
         <f aca="false">D5-E5</f>
         <v>0</v>
       </c>
-      <c r="G5" s="18" t="str">
+      <c r="G5" s="5" t="str">
         <f aca="false">IF(E5&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="5" t="s">
         <v>2281</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="5" t="n">
         <f aca="false">D6-E6</f>
         <v>4</v>
       </c>
-      <c r="G6" s="18" t="str">
+      <c r="G6" s="5" t="str">
         <f aca="false">IF(E6&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="5" t="s">
         <v>2283</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="5" t="n">
         <f aca="false">D7-E7</f>
         <v>2</v>
       </c>
-      <c r="G7" s="18" t="str">
+      <c r="G7" s="5" t="str">
         <f aca="false">IF(E7&gt;=5,"Check","")</f>
         <v>Check</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="5" t="s">
         <v>2024</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="5" t="s">
         <v>2284</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="5" t="n">
         <f aca="false">D8-E8</f>
         <v>1</v>
       </c>
-      <c r="G8" s="18" t="str">
+      <c r="G8" s="5" t="str">
         <f aca="false">IF(E8&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="5" t="s">
         <v>2285</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="5" t="n">
         <f aca="false">D9-E9</f>
         <v>2</v>
       </c>
-      <c r="G9" s="18" t="str">
+      <c r="G9" s="5" t="str">
         <f aca="false">IF(E9&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="5" t="s">
         <v>2286</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="5" t="n">
         <f aca="false">D10-E10</f>
         <v>0</v>
       </c>
-      <c r="G10" s="18" t="str">
+      <c r="G10" s="5" t="str">
         <f aca="false">IF(E10&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="5" t="s">
         <v>2287</v>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="5" t="n">
         <f aca="false">D11-E11</f>
         <v>3</v>
       </c>
-      <c r="G11" s="18" t="str">
+      <c r="G11" s="5" t="str">
         <f aca="false">IF(E11&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="5" t="s">
         <v>2288</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="5" t="n">
         <f aca="false">D12-E12</f>
         <v>2</v>
       </c>
-      <c r="G12" s="18" t="str">
+      <c r="G12" s="5" t="str">
         <f aca="false">IF(E12&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="18" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="5" t="s">
         <v>2289</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="5" t="n">
         <f aca="false">D13-E13</f>
         <v>3</v>
       </c>
-      <c r="G13" s="18" t="str">
+      <c r="G13" s="5" t="str">
         <f aca="false">IF(E13&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="18" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="5" t="s">
         <v>2290</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="5" t="n">
         <f aca="false">D14-E14</f>
         <v>3</v>
       </c>
-      <c r="G14" s="18" t="str">
+      <c r="G14" s="5" t="str">
         <f aca="false">IF(E14&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="18" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C15" s="5" t="s">
         <v>2291</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="5" t="n">
         <f aca="false">D15-E15</f>
         <v>2</v>
       </c>
-      <c r="G15" s="18" t="str">
+      <c r="G15" s="5" t="str">
         <f aca="false">IF(E15&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="5" t="s">
         <v>2292</v>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="5" t="n">
         <f aca="false">D16-E16</f>
         <v>4</v>
       </c>
-      <c r="G16" s="18" t="str">
+      <c r="G16" s="5" t="str">
         <f aca="false">IF(E16&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="5" t="s">
         <v>2024</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C17" s="5" t="s">
         <v>2293</v>
       </c>
-      <c r="D17" s="18" t="n">
+      <c r="D17" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F17" s="5" t="n">
         <f aca="false">D17-E17</f>
         <v>2</v>
       </c>
-      <c r="G17" s="18" t="str">
+      <c r="G17" s="5" t="str">
         <f aca="false">IF(E17&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C18" s="5" t="s">
         <v>2294</v>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="5" t="n">
         <f aca="false">D18-E18</f>
         <v>0</v>
       </c>
-      <c r="G18" s="18" t="str">
+      <c r="G18" s="5" t="str">
         <f aca="false">IF(E18&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="5" t="s">
         <v>2295</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E19" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="18" t="n">
+      <c r="F19" s="5" t="n">
         <f aca="false">D19-E19</f>
         <v>0</v>
       </c>
-      <c r="G19" s="18" t="str">
+      <c r="G19" s="5" t="str">
         <f aca="false">IF(E19&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="18" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="C20" s="5" t="s">
         <v>2296</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="5" t="n">
         <f aca="false">D20-E20</f>
         <v>0</v>
       </c>
-      <c r="G20" s="18" t="str">
+      <c r="G20" s="5" t="str">
         <f aca="false">IF(E20&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="18" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="5" t="s">
         <v>2078</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="5" t="s">
         <v>2297</v>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="18" t="n">
+      <c r="E21" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="18" t="n">
+      <c r="F21" s="5" t="n">
         <f aca="false">D21-E21</f>
         <v>1</v>
       </c>
-      <c r="G21" s="18" t="str">
+      <c r="G21" s="5" t="str">
         <f aca="false">IF(E21&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="5" t="s">
         <v>2298</v>
       </c>
-      <c r="D22" s="18" t="n">
+      <c r="D22" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E22" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="18" t="n">
+      <c r="F22" s="5" t="n">
         <f aca="false">D22-E22</f>
         <v>4</v>
       </c>
-      <c r="G22" s="18" t="str">
+      <c r="G22" s="5" t="str">
         <f aca="false">IF(E22&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="5" t="s">
         <v>2299</v>
       </c>
-      <c r="D23" s="18" t="n">
+      <c r="D23" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="18" t="n">
+      <c r="E23" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="18" t="n">
+      <c r="F23" s="5" t="n">
         <f aca="false">D23-E23</f>
         <v>1</v>
       </c>
-      <c r="G23" s="18" t="str">
+      <c r="G23" s="5" t="str">
         <f aca="false">IF(E23&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="5" t="s">
         <v>2300</v>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="18" t="n">
+      <c r="F24" s="5" t="n">
         <f aca="false">D24-E24</f>
         <v>3</v>
       </c>
-      <c r="G24" s="18" t="str">
+      <c r="G24" s="5" t="str">
         <f aca="false">IF(E24&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="5" t="s">
         <v>2301</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E25" s="18" t="n">
+      <c r="E25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="18" t="n">
+      <c r="F25" s="5" t="n">
         <f aca="false">D25-E25</f>
         <v>2</v>
       </c>
-      <c r="G25" s="18" t="str">
+      <c r="G25" s="5" t="str">
         <f aca="false">IF(E25&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="5" t="s">
         <v>2302</v>
       </c>
-      <c r="D26" s="18" t="n">
+      <c r="D26" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E26" s="18" t="n">
+      <c r="E26" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="18" t="n">
+      <c r="F26" s="5" t="n">
         <f aca="false">D26-E26</f>
         <v>2</v>
       </c>
-      <c r="G26" s="18" t="str">
+      <c r="G26" s="5" t="str">
         <f aca="false">IF(E26&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="18" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="5" t="s">
         <v>2303</v>
       </c>
-      <c r="D27" s="18" t="n">
+      <c r="D27" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E27" s="18" t="n">
+      <c r="E27" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F27" s="18" t="n">
+      <c r="F27" s="5" t="n">
         <f aca="false">D27-E27</f>
         <v>4</v>
       </c>
-      <c r="G27" s="18" t="str">
+      <c r="G27" s="5" t="str">
         <f aca="false">IF(E27&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="18" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="5" t="s">
         <v>2304</v>
       </c>
-      <c r="D28" s="18" t="n">
+      <c r="D28" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E28" s="18" t="n">
+      <c r="E28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="18" t="n">
+      <c r="F28" s="5" t="n">
         <f aca="false">D28-E28</f>
         <v>4</v>
       </c>
-      <c r="G28" s="18" t="str">
+      <c r="G28" s="5" t="str">
         <f aca="false">IF(E28&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="18" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="5" t="s">
         <v>2305</v>
       </c>
-      <c r="D29" s="18" t="n">
+      <c r="D29" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="18" t="n">
+      <c r="E29" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F29" s="18" t="n">
+      <c r="F29" s="5" t="n">
         <f aca="false">D29-E29</f>
         <v>0</v>
       </c>
-      <c r="G29" s="18" t="str">
+      <c r="G29" s="5" t="str">
         <f aca="false">IF(E29&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="18" t="n">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="5" t="s">
         <v>2306</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F30" s="18" t="n">
+      <c r="F30" s="5" t="n">
         <f aca="false">D30-E30</f>
         <v>0</v>
       </c>
-      <c r="G30" s="18" t="str">
+      <c r="G30" s="5" t="str">
         <f aca="false">IF(E30&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="18" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="B31" s="18" t="s">
+      <c r="B31" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="5" t="s">
         <v>2307</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E31" s="18" t="n">
+      <c r="E31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F31" s="18" t="n">
+      <c r="F31" s="5" t="n">
         <f aca="false">D31-E31</f>
         <v>5</v>
       </c>
-      <c r="G31" s="18" t="str">
+      <c r="G31" s="5" t="str">
         <f aca="false">IF(E31&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="18" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B32" s="18" t="s">
+      <c r="B32" s="5" t="s">
         <v>2078</v>
       </c>
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="5" t="s">
         <v>2308</v>
       </c>
-      <c r="D32" s="18" t="n">
+      <c r="D32" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E32" s="18" t="n">
+      <c r="E32" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F32" s="18" t="n">
+      <c r="F32" s="5" t="n">
         <f aca="false">D32-E32</f>
         <v>1</v>
       </c>
-      <c r="G32" s="18" t="str">
+      <c r="G32" s="5" t="str">
         <f aca="false">IF(E32&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="18" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="5" t="s">
         <v>2309</v>
       </c>
-      <c r="D33" s="18" t="n">
+      <c r="D33" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E33" s="18" t="n">
+      <c r="E33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="18" t="n">
+      <c r="F33" s="5" t="n">
         <f aca="false">D33-E33</f>
         <v>3</v>
       </c>
-      <c r="G33" s="18" t="str">
+      <c r="G33" s="5" t="str">
         <f aca="false">IF(E33&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="18" t="n">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B34" s="18" t="s">
+      <c r="B34" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="5" t="s">
         <v>2310</v>
       </c>
-      <c r="D34" s="18" t="n">
+      <c r="D34" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E34" s="18" t="n">
+      <c r="E34" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F34" s="18" t="n">
+      <c r="F34" s="5" t="n">
         <f aca="false">D34-E34</f>
         <v>1</v>
       </c>
-      <c r="G34" s="18" t="str">
+      <c r="G34" s="5" t="str">
         <f aca="false">IF(E34&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="n">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="5" t="s">
         <v>2024</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="5" t="s">
         <v>2311</v>
       </c>
-      <c r="D35" s="18" t="n">
+      <c r="D35" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E35" s="18" t="n">
+      <c r="E35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="18" t="n">
+      <c r="F35" s="5" t="n">
         <f aca="false">D35-E35</f>
         <v>2</v>
       </c>
-      <c r="G35" s="18" t="str">
+      <c r="G35" s="5" t="str">
         <f aca="false">IF(E35&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="n">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="5" t="s">
         <v>2312</v>
       </c>
-      <c r="D36" s="18" t="n">
+      <c r="D36" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="18" t="n">
+      <c r="E36" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F36" s="18" t="n">
+      <c r="F36" s="5" t="n">
         <f aca="false">D36-E36</f>
         <v>1</v>
       </c>
-      <c r="G36" s="18" t="str">
+      <c r="G36" s="5" t="str">
         <f aca="false">IF(E36&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="18" t="n">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C37" s="18" t="s">
+      <c r="C37" s="5" t="s">
         <v>2313</v>
       </c>
-      <c r="D37" s="18" t="n">
+      <c r="D37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E37" s="18" t="n">
+      <c r="E37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F37" s="18" t="n">
+      <c r="F37" s="5" t="n">
         <f aca="false">D37-E37</f>
         <v>0</v>
       </c>
-      <c r="G37" s="18" t="str">
+      <c r="G37" s="5" t="str">
         <f aca="false">IF(E37&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="n">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="C38" s="5" t="s">
         <v>2314</v>
       </c>
-      <c r="D38" s="18" t="n">
+      <c r="D38" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E38" s="18" t="n">
+      <c r="E38" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F38" s="18" t="n">
+      <c r="F38" s="5" t="n">
         <f aca="false">D38-E38</f>
         <v>2</v>
       </c>
-      <c r="G38" s="18" t="str">
+      <c r="G38" s="5" t="str">
         <f aca="false">IF(E38&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="n">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="B39" s="18" t="s">
+      <c r="B39" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C39" s="18" t="s">
+      <c r="C39" s="5" t="s">
         <v>2315</v>
       </c>
-      <c r="D39" s="18" t="n">
+      <c r="D39" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E39" s="18" t="n">
+      <c r="E39" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F39" s="18" t="n">
+      <c r="F39" s="5" t="n">
         <f aca="false">D39-E39</f>
         <v>1</v>
       </c>
-      <c r="G39" s="18" t="str">
+      <c r="G39" s="5" t="str">
         <f aca="false">IF(E39&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="18" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="B40" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="5" t="s">
         <v>2316</v>
       </c>
-      <c r="D40" s="18" t="n">
+      <c r="D40" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E40" s="18" t="n">
+      <c r="E40" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F40" s="18" t="n">
+      <c r="F40" s="5" t="n">
         <f aca="false">D40-E40</f>
         <v>0</v>
       </c>
-      <c r="G40" s="18" t="str">
+      <c r="G40" s="5" t="str">
         <f aca="false">IF(E40&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="18" t="n">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="n">
         <v>47</v>
       </c>
-      <c r="B41" s="18" t="s">
+      <c r="B41" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C41" s="18" t="s">
+      <c r="C41" s="5" t="s">
         <v>2317</v>
       </c>
-      <c r="D41" s="18" t="n">
+      <c r="D41" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E41" s="18" t="n">
+      <c r="E41" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F41" s="18" t="n">
+      <c r="F41" s="5" t="n">
         <f aca="false">D41-E41</f>
         <v>2</v>
       </c>
-      <c r="G41" s="18" t="str">
+      <c r="G41" s="5" t="str">
         <f aca="false">IF(E41&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="18" t="n">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="n">
         <v>49</v>
       </c>
-      <c r="B42" s="18" t="s">
+      <c r="B42" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="C42" s="5" t="s">
         <v>2318</v>
       </c>
-      <c r="D42" s="18" t="n">
+      <c r="D42" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E42" s="18" t="n">
+      <c r="E42" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F42" s="18" t="n">
+      <c r="F42" s="5" t="n">
         <f aca="false">D42-E42</f>
         <v>1</v>
       </c>
-      <c r="G42" s="18" t="str">
+      <c r="G42" s="5" t="str">
         <f aca="false">IF(E42&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="18" t="n">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C43" s="18" t="s">
+      <c r="C43" s="5" t="s">
         <v>2319</v>
       </c>
-      <c r="D43" s="18" t="n">
+      <c r="D43" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E43" s="18" t="n">
+      <c r="E43" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F43" s="18" t="n">
+      <c r="F43" s="5" t="n">
         <f aca="false">D43-E43</f>
         <v>4</v>
       </c>
-      <c r="G43" s="18" t="str">
+      <c r="G43" s="5" t="str">
         <f aca="false">IF(E43&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="18" t="n">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="B44" s="18" t="s">
+      <c r="B44" s="5" t="s">
         <v>2024</v>
       </c>
-      <c r="C44" s="18" t="s">
+      <c r="C44" s="5" t="s">
         <v>2320</v>
       </c>
-      <c r="D44" s="18" t="n">
+      <c r="D44" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E44" s="18" t="n">
+      <c r="E44" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F44" s="18" t="n">
+      <c r="F44" s="5" t="n">
         <f aca="false">D44-E44</f>
         <v>2</v>
       </c>
-      <c r="G44" s="18" t="str">
+      <c r="G44" s="5" t="str">
         <f aca="false">IF(E44&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="18" t="n">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="B45" s="18" t="s">
+      <c r="B45" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C45" s="18" t="s">
+      <c r="C45" s="5" t="s">
         <v>2321</v>
       </c>
-      <c r="D45" s="18" t="n">
+      <c r="D45" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E45" s="18" t="n">
+      <c r="E45" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F45" s="18" t="n">
+      <c r="F45" s="5" t="n">
         <f aca="false">D45-E45</f>
         <v>3</v>
       </c>
-      <c r="G45" s="18" t="str">
+      <c r="G45" s="5" t="str">
         <f aca="false">IF(E45&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="18" t="n">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="B46" s="18" t="s">
+      <c r="B46" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C46" s="18" t="s">
+      <c r="C46" s="5" t="s">
         <v>2322</v>
       </c>
-      <c r="D46" s="18" t="n">
+      <c r="D46" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="18" t="n">
+      <c r="E46" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F46" s="18" t="n">
+      <c r="F46" s="5" t="n">
         <f aca="false">D46-E46</f>
         <v>0</v>
       </c>
-      <c r="G46" s="18" t="str">
+      <c r="G46" s="5" t="str">
         <f aca="false">IF(E46&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="n">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="n">
         <v>61</v>
       </c>
-      <c r="B47" s="18" t="s">
+      <c r="B47" s="5" t="s">
         <v>2078</v>
       </c>
-      <c r="C47" s="18" t="s">
+      <c r="C47" s="5" t="s">
         <v>2323</v>
       </c>
-      <c r="D47" s="18" t="n">
+      <c r="D47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E47" s="18" t="n">
+      <c r="E47" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F47" s="18" t="n">
+      <c r="F47" s="5" t="n">
         <f aca="false">D47-E47</f>
         <v>0</v>
       </c>
-      <c r="G47" s="18" t="str">
+      <c r="G47" s="5" t="str">
         <f aca="false">IF(E47&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="18" t="n">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="B48" s="18" t="s">
+      <c r="B48" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C48" s="18" t="s">
+      <c r="C48" s="5" t="s">
         <v>2324</v>
       </c>
-      <c r="D48" s="18" t="n">
+      <c r="D48" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E48" s="18" t="n">
+      <c r="E48" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F48" s="18" t="n">
+      <c r="F48" s="5" t="n">
         <f aca="false">D48-E48</f>
         <v>0</v>
       </c>
-      <c r="G48" s="18" t="str">
+      <c r="G48" s="5" t="str">
         <f aca="false">IF(E48&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="18" t="n">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="B49" s="18" t="s">
+      <c r="B49" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C49" s="18" t="s">
+      <c r="C49" s="5" t="s">
         <v>2325</v>
       </c>
-      <c r="D49" s="18" t="n">
+      <c r="D49" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E49" s="18" t="n">
+      <c r="E49" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="18" t="n">
+      <c r="F49" s="5" t="n">
         <f aca="false">D49-E49</f>
         <v>2</v>
       </c>
-      <c r="G49" s="18" t="str">
+      <c r="G49" s="5" t="str">
         <f aca="false">IF(E49&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="18" t="n">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C50" s="18" t="s">
+      <c r="C50" s="5" t="s">
         <v>2326</v>
       </c>
-      <c r="D50" s="18" t="n">
+      <c r="D50" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E50" s="18" t="n">
+      <c r="E50" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F50" s="18" t="n">
+      <c r="F50" s="5" t="n">
         <f aca="false">D50-E50</f>
         <v>1</v>
       </c>
-      <c r="G50" s="18" t="str">
+      <c r="G50" s="5" t="str">
         <f aca="false">IF(E50&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="18" t="n">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="B51" s="18" t="s">
+      <c r="B51" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C51" s="18" t="s">
+      <c r="C51" s="5" t="s">
         <v>2327</v>
       </c>
-      <c r="D51" s="18" t="n">
+      <c r="D51" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E51" s="18" t="n">
+      <c r="E51" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F51" s="18" t="n">
+      <c r="F51" s="5" t="n">
         <f aca="false">D51-E51</f>
         <v>0</v>
       </c>
-      <c r="G51" s="18" t="str">
+      <c r="G51" s="5" t="str">
         <f aca="false">IF(E51&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="18" t="n">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B52" s="5" t="s">
         <v>2078</v>
       </c>
-      <c r="C52" s="18" t="s">
+      <c r="C52" s="5" t="s">
         <v>2328</v>
       </c>
-      <c r="D52" s="18" t="n">
+      <c r="D52" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E52" s="18" t="n">
+      <c r="E52" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F52" s="18" t="n">
+      <c r="F52" s="5" t="n">
         <f aca="false">D52-E52</f>
         <v>0</v>
       </c>
-      <c r="G52" s="18" t="str">
+      <c r="G52" s="5" t="str">
         <f aca="false">IF(E52&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="18" t="n">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="B53" s="18" t="s">
+      <c r="B53" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C53" s="18" t="s">
+      <c r="C53" s="5" t="s">
         <v>2329</v>
       </c>
-      <c r="D53" s="18" t="n">
+      <c r="D53" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E53" s="18" t="n">
+      <c r="E53" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F53" s="18" t="n">
+      <c r="F53" s="5" t="n">
         <f aca="false">D53-E53</f>
         <v>0</v>
       </c>
-      <c r="G53" s="18" t="str">
+      <c r="G53" s="5" t="str">
         <f aca="false">IF(E53&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="18" t="n">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="n">
         <v>61</v>
       </c>
-      <c r="B54" s="18" t="s">
+      <c r="B54" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C54" s="18" t="s">
+      <c r="C54" s="5" t="s">
         <v>2330</v>
       </c>
-      <c r="D54" s="18" t="n">
+      <c r="D54" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E54" s="18" t="n">
+      <c r="E54" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F54" s="18" t="n">
+      <c r="F54" s="5" t="n">
         <f aca="false">D54-E54</f>
         <v>0</v>
       </c>
-      <c r="G54" s="18" t="str">
+      <c r="G54" s="5" t="str">
         <f aca="false">IF(E54&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="18" t="n">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="B55" s="18" t="s">
+      <c r="B55" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C55" s="18" t="s">
+      <c r="C55" s="5" t="s">
         <v>2331</v>
       </c>
-      <c r="D55" s="18" t="n">
+      <c r="D55" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E55" s="18" t="n">
+      <c r="E55" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F55" s="18" t="n">
+      <c r="F55" s="5" t="n">
         <f aca="false">D55-E55</f>
         <v>3</v>
       </c>
-      <c r="G55" s="18" t="str">
+      <c r="G55" s="5" t="str">
         <f aca="false">IF(E55&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="18" t="n">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5" t="n">
         <v>63</v>
       </c>
-      <c r="B56" s="18" t="s">
+      <c r="B56" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C56" s="18" t="s">
+      <c r="C56" s="5" t="s">
         <v>2332</v>
       </c>
-      <c r="D56" s="18" t="n">
+      <c r="D56" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E56" s="18" t="n">
+      <c r="E56" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F56" s="18" t="n">
+      <c r="F56" s="5" t="n">
         <f aca="false">D56-E56</f>
         <v>5</v>
       </c>
-      <c r="G56" s="18" t="str">
+      <c r="G56" s="5" t="str">
         <f aca="false">IF(E56&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="18" t="n">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="5" t="n">
         <v>67</v>
       </c>
-      <c r="B57" s="18" t="s">
+      <c r="B57" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C57" s="18" t="s">
+      <c r="C57" s="5" t="s">
         <v>2333</v>
       </c>
-      <c r="D57" s="18" t="n">
+      <c r="D57" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E57" s="18" t="n">
+      <c r="E57" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F57" s="18" t="n">
+      <c r="F57" s="5" t="n">
         <f aca="false">D57-E57</f>
         <v>1</v>
       </c>
-      <c r="G57" s="18" t="str">
+      <c r="G57" s="5" t="str">
         <f aca="false">IF(E57&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="18" t="n">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5" t="n">
         <v>65</v>
       </c>
-      <c r="B58" s="18" t="s">
+      <c r="B58" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C58" s="18" t="s">
+      <c r="C58" s="5" t="s">
         <v>2334</v>
       </c>
-      <c r="D58" s="18" t="n">
+      <c r="D58" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E58" s="18" t="n">
+      <c r="E58" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F58" s="18" t="n">
+      <c r="F58" s="5" t="n">
         <f aca="false">D58-E58</f>
         <v>0</v>
       </c>
-      <c r="G58" s="18" t="str">
+      <c r="G58" s="5" t="str">
         <f aca="false">IF(E58&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="18" t="n">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="B59" s="18" t="s">
+      <c r="B59" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C59" s="18" t="s">
+      <c r="C59" s="5" t="s">
         <v>2335</v>
       </c>
-      <c r="D59" s="18" t="n">
+      <c r="D59" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E59" s="18" t="n">
+      <c r="E59" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F59" s="18" t="n">
+      <c r="F59" s="5" t="n">
         <f aca="false">D59-E59</f>
         <v>0</v>
       </c>
-      <c r="G59" s="18" t="str">
+      <c r="G59" s="5" t="str">
         <f aca="false">IF(E59&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="18" t="n">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="B60" s="18" t="s">
+      <c r="B60" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C60" s="18" t="s">
+      <c r="C60" s="5" t="s">
         <v>2336</v>
       </c>
-      <c r="D60" s="18" t="n">
+      <c r="D60" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E60" s="18" t="n">
+      <c r="E60" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F60" s="18" t="n">
+      <c r="F60" s="5" t="n">
         <f aca="false">D60-E60</f>
         <v>1</v>
       </c>
-      <c r="G60" s="18" t="str">
+      <c r="G60" s="5" t="str">
         <f aca="false">IF(E60&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="18" t="n">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="5" t="n">
         <v>68</v>
       </c>
-      <c r="B61" s="18" t="s">
+      <c r="B61" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C61" s="18" t="s">
+      <c r="C61" s="5" t="s">
         <v>2337</v>
       </c>
-      <c r="D61" s="18" t="n">
+      <c r="D61" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E61" s="18" t="n">
+      <c r="E61" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F61" s="18" t="n">
+      <c r="F61" s="5" t="n">
         <f aca="false">D61-E61</f>
         <v>2</v>
       </c>
-      <c r="G61" s="18" t="str">
+      <c r="G61" s="5" t="str">
         <f aca="false">IF(E61&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="18" t="n">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5" t="n">
         <v>78</v>
       </c>
-      <c r="B62" s="18" t="s">
+      <c r="B62" s="5" t="s">
         <v>2078</v>
       </c>
-      <c r="C62" s="18" t="s">
+      <c r="C62" s="5" t="s">
         <v>2338</v>
       </c>
-      <c r="D62" s="18" t="n">
+      <c r="D62" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E62" s="18" t="n">
+      <c r="E62" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F62" s="18" t="n">
+      <c r="F62" s="5" t="n">
         <f aca="false">D62-E62</f>
         <v>1</v>
       </c>
-      <c r="G62" s="18" t="str">
+      <c r="G62" s="5" t="str">
         <f aca="false">IF(E62&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="18" t="n">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5" t="n">
         <v>75</v>
       </c>
-      <c r="B63" s="18" t="s">
+      <c r="B63" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C63" s="18" t="s">
+      <c r="C63" s="5" t="s">
         <v>2339</v>
       </c>
-      <c r="D63" s="18" t="n">
+      <c r="D63" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E63" s="18" t="n">
+      <c r="E63" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F63" s="18" t="n">
+      <c r="F63" s="5" t="n">
         <f aca="false">D63-E63</f>
         <v>0</v>
       </c>
-      <c r="G63" s="18" t="str">
+      <c r="G63" s="5" t="str">
         <f aca="false">IF(E63&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="18" t="n">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5" t="n">
         <v>71</v>
       </c>
-      <c r="B64" s="18" t="s">
+      <c r="B64" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C64" s="18" t="s">
+      <c r="C64" s="5" t="s">
         <v>2340</v>
       </c>
-      <c r="D64" s="18" t="n">
+      <c r="D64" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E64" s="18" t="n">
+      <c r="E64" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F64" s="18" t="n">
+      <c r="F64" s="5" t="n">
         <f aca="false">D64-E64</f>
         <v>0</v>
       </c>
-      <c r="G64" s="18" t="str">
+      <c r="G64" s="5" t="str">
         <f aca="false">IF(E64&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="18" t="n">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5" t="n">
         <v>72</v>
       </c>
-      <c r="B65" s="18" t="s">
+      <c r="B65" s="5" t="s">
         <v>2024</v>
       </c>
-      <c r="C65" s="18" t="s">
+      <c r="C65" s="5" t="s">
         <v>2341</v>
       </c>
-      <c r="D65" s="18" t="n">
+      <c r="D65" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E65" s="18" t="n">
+      <c r="E65" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F65" s="18" t="n">
+      <c r="F65" s="5" t="n">
         <f aca="false">D65-E65</f>
         <v>1</v>
       </c>
-      <c r="G65" s="18" t="str">
+      <c r="G65" s="5" t="str">
         <f aca="false">IF(E65&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="18" t="n">
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="B66" s="18" t="s">
+      <c r="B66" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C66" s="18" t="s">
+      <c r="C66" s="5" t="s">
         <v>2342</v>
       </c>
-      <c r="D66" s="18" t="n">
+      <c r="D66" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="E66" s="18" t="n">
+      <c r="E66" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F66" s="18" t="n">
+      <c r="F66" s="5" t="n">
         <f aca="false">D66-E66</f>
         <v>4</v>
       </c>
-      <c r="G66" s="18" t="str">
+      <c r="G66" s="5" t="str">
         <f aca="false">IF(E66&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="18" t="n">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="n">
         <v>73</v>
       </c>
-      <c r="B67" s="18" t="s">
+      <c r="B67" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C67" s="18" t="s">
+      <c r="C67" s="5" t="s">
         <v>2343</v>
       </c>
-      <c r="D67" s="18" t="n">
+      <c r="D67" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E67" s="18" t="n">
+      <c r="E67" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F67" s="18" t="n">
+      <c r="F67" s="5" t="n">
         <f aca="false">D67-E67</f>
         <v>1</v>
       </c>
-      <c r="G67" s="18" t="str">
+      <c r="G67" s="5" t="str">
         <f aca="false">IF(E67&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="18" t="n">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5" t="n">
         <v>76</v>
       </c>
-      <c r="B68" s="18" t="s">
+      <c r="B68" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C68" s="18" t="s">
+      <c r="C68" s="5" t="s">
         <v>2344</v>
       </c>
-      <c r="D68" s="18" t="n">
+      <c r="D68" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E68" s="18" t="n">
+      <c r="E68" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F68" s="18" t="n">
+      <c r="F68" s="5" t="n">
         <f aca="false">D68-E68</f>
         <v>2</v>
       </c>
-      <c r="G68" s="18" t="str">
+      <c r="G68" s="5" t="str">
         <f aca="false">IF(E68&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="18" t="n">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="n">
         <v>84</v>
       </c>
-      <c r="B69" s="18" t="s">
+      <c r="B69" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C69" s="18" t="s">
+      <c r="C69" s="5" t="s">
         <v>2345</v>
       </c>
-      <c r="D69" s="18" t="n">
+      <c r="D69" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E69" s="18" t="n">
+      <c r="E69" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F69" s="18" t="n">
+      <c r="F69" s="5" t="n">
         <f aca="false">D69-E69</f>
         <v>2</v>
       </c>
-      <c r="G69" s="18" t="str">
+      <c r="G69" s="5" t="str">
         <f aca="false">IF(E69&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="18" t="n">
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="5" t="n">
         <v>79</v>
       </c>
-      <c r="B70" s="18" t="s">
+      <c r="B70" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C70" s="18" t="s">
+      <c r="C70" s="5" t="s">
         <v>2346</v>
       </c>
-      <c r="D70" s="18" t="n">
+      <c r="D70" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E70" s="18" t="n">
+      <c r="E70" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F70" s="18" t="n">
+      <c r="F70" s="5" t="n">
         <f aca="false">D70-E70</f>
         <v>3</v>
       </c>
-      <c r="G70" s="18" t="str">
+      <c r="G70" s="5" t="str">
         <f aca="false">IF(E70&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="18" t="n">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="B71" s="18" t="s">
+      <c r="B71" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C71" s="18" t="s">
+      <c r="C71" s="5" t="s">
         <v>2347</v>
       </c>
-      <c r="D71" s="18" t="n">
+      <c r="D71" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E71" s="18" t="n">
+      <c r="E71" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F71" s="18" t="n">
+      <c r="F71" s="5" t="n">
         <f aca="false">D71-E71</f>
         <v>3</v>
       </c>
-      <c r="G71" s="18" t="str">
+      <c r="G71" s="5" t="str">
         <f aca="false">IF(E71&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="18" t="n">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5" t="n">
         <v>79</v>
       </c>
-      <c r="B72" s="18" t="s">
+      <c r="B72" s="5" t="s">
         <v>2102</v>
       </c>
-      <c r="C72" s="18" t="s">
+      <c r="C72" s="5" t="s">
         <v>2348</v>
       </c>
-      <c r="D72" s="18" t="n">
+      <c r="D72" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="E72" s="18" t="n">
+      <c r="E72" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F72" s="18" t="n">
+      <c r="F72" s="5" t="n">
         <f aca="false">D72-E72</f>
         <v>2</v>
       </c>
-      <c r="G72" s="18" t="str">
+      <c r="G72" s="5" t="str">
         <f aca="false">IF(E72&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="18" t="n">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="B73" s="18" t="s">
+      <c r="B73" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C73" s="18" t="s">
+      <c r="C73" s="5" t="s">
         <v>2349</v>
       </c>
-      <c r="D73" s="18" t="n">
+      <c r="D73" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E73" s="18" t="n">
+      <c r="E73" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F73" s="18" t="n">
+      <c r="F73" s="5" t="n">
         <f aca="false">D73-E73</f>
         <v>1</v>
       </c>
-      <c r="G73" s="18" t="str">
+      <c r="G73" s="5" t="str">
         <f aca="false">IF(E73&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="18" t="n">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="5" t="n">
         <v>81</v>
       </c>
-      <c r="B74" s="18" t="s">
+      <c r="B74" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C74" s="18" t="s">
+      <c r="C74" s="5" t="s">
         <v>2350</v>
       </c>
-      <c r="D74" s="18" t="n">
+      <c r="D74" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E74" s="18" t="n">
+      <c r="E74" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F74" s="18" t="n">
+      <c r="F74" s="5" t="n">
         <f aca="false">D74-E74</f>
         <v>0</v>
       </c>
-      <c r="G74" s="18" t="str">
+      <c r="G74" s="5" t="str">
         <f aca="false">IF(E74&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="18" t="n">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5" t="n">
         <v>87</v>
       </c>
-      <c r="B75" s="18" t="s">
+      <c r="B75" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C75" s="18" t="s">
+      <c r="C75" s="5" t="s">
         <v>2351</v>
       </c>
-      <c r="D75" s="18" t="n">
+      <c r="D75" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="E75" s="18" t="n">
+      <c r="E75" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F75" s="18" t="n">
+      <c r="F75" s="5" t="n">
         <f aca="false">D75-E75</f>
         <v>3</v>
       </c>
-      <c r="G75" s="18" t="str">
+      <c r="G75" s="5" t="str">
         <f aca="false">IF(E75&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="18" t="n">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="B76" s="18" t="s">
+      <c r="B76" s="5" t="s">
         <v>2078</v>
       </c>
-      <c r="C76" s="18" t="s">
+      <c r="C76" s="5" t="s">
         <v>2352</v>
       </c>
-      <c r="D76" s="18" t="n">
+      <c r="D76" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E76" s="18" t="n">
+      <c r="E76" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F76" s="18" t="n">
+      <c r="F76" s="5" t="n">
         <f aca="false">D76-E76</f>
         <v>1</v>
       </c>
-      <c r="G76" s="18" t="str">
+      <c r="G76" s="5" t="str">
         <f aca="false">IF(E76&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="18" t="n">
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="B77" s="18" t="s">
+      <c r="B77" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C77" s="18" t="s">
+      <c r="C77" s="5" t="s">
         <v>2353</v>
       </c>
-      <c r="D77" s="18" t="n">
+      <c r="D77" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E77" s="18" t="n">
+      <c r="E77" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F77" s="18" t="n">
+      <c r="F77" s="5" t="n">
         <f aca="false">D77-E77</f>
         <v>1</v>
       </c>
-      <c r="G77" s="18" t="str">
+      <c r="G77" s="5" t="str">
         <f aca="false">IF(E77&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="18" t="n">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="B78" s="18" t="s">
+      <c r="B78" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C78" s="18" t="s">
+      <c r="C78" s="5" t="s">
         <v>2354</v>
       </c>
-      <c r="D78" s="18" t="n">
+      <c r="D78" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E78" s="18" t="n">
+      <c r="E78" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F78" s="18" t="n">
+      <c r="F78" s="5" t="n">
         <f aca="false">D78-E78</f>
         <v>2</v>
       </c>
-      <c r="G78" s="18" t="str">
+      <c r="G78" s="5" t="str">
         <f aca="false">IF(E78&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="18" t="n">
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="5" t="n">
         <v>87</v>
       </c>
-      <c r="B79" s="18" t="s">
+      <c r="B79" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C79" s="18" t="s">
+      <c r="C79" s="5" t="s">
         <v>2355</v>
       </c>
-      <c r="D79" s="18" t="n">
+      <c r="D79" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E79" s="18" t="n">
+      <c r="E79" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F79" s="18" t="n">
+      <c r="F79" s="5" t="n">
         <f aca="false">D79-E79</f>
         <v>1</v>
       </c>
-      <c r="G79" s="18" t="str">
+      <c r="G79" s="5" t="str">
         <f aca="false">IF(E79&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="18" t="n">
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="B80" s="18" t="s">
+      <c r="B80" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C80" s="18" t="s">
+      <c r="C80" s="5" t="s">
         <v>2356</v>
       </c>
-      <c r="D80" s="18" t="n">
+      <c r="D80" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E80" s="18" t="n">
+      <c r="E80" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F80" s="18" t="n">
+      <c r="F80" s="5" t="n">
         <f aca="false">D80-E80</f>
         <v>0</v>
       </c>
-      <c r="G80" s="18" t="str">
+      <c r="G80" s="5" t="str">
         <f aca="false">IF(E80&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="18" t="n">
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="B81" s="18" t="s">
+      <c r="B81" s="5" t="s">
         <v>2024</v>
       </c>
-      <c r="C81" s="18" t="s">
+      <c r="C81" s="5" t="s">
         <v>2357</v>
       </c>
-      <c r="D81" s="18" t="n">
+      <c r="D81" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E81" s="18" t="n">
+      <c r="E81" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F81" s="18" t="n">
+      <c r="F81" s="5" t="n">
         <f aca="false">D81-E81</f>
         <v>0</v>
       </c>
-      <c r="G81" s="18" t="str">
+      <c r="G81" s="5" t="str">
         <f aca="false">IF(E81&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="18" t="n">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5" t="n">
         <v>91</v>
       </c>
-      <c r="B82" s="18" t="s">
+      <c r="B82" s="5" t="s">
         <v>2038</v>
       </c>
-      <c r="C82" s="18" t="s">
+      <c r="C82" s="5" t="s">
         <v>2358</v>
       </c>
-      <c r="D82" s="18" t="n">
+      <c r="D82" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E82" s="18" t="n">
+      <c r="E82" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F82" s="18" t="n">
+      <c r="F82" s="5" t="n">
         <f aca="false">D82-E82</f>
         <v>0</v>
       </c>
-      <c r="G82" s="18" t="str">
+      <c r="G82" s="5" t="str">
         <f aca="false">IF(E82&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="18" t="n">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="5" t="n">
         <v>93</v>
       </c>
-      <c r="B83" s="18" t="s">
+      <c r="B83" s="5" t="s">
         <v>2051</v>
       </c>
-      <c r="C83" s="18" t="s">
+      <c r="C83" s="5" t="s">
         <v>2359</v>
       </c>
-      <c r="D83" s="18" t="n">
+      <c r="D83" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E83" s="18" t="n">
+      <c r="E83" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F83" s="18" t="n">
+      <c r="F83" s="5" t="n">
         <f aca="false">D83-E83</f>
         <v>0</v>
       </c>
-      <c r="G83" s="18" t="str">
+      <c r="G83" s="5" t="str">
         <f aca="false">IF(E83&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="18" t="n">
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="5" t="n">
         <v>94</v>
       </c>
-      <c r="B84" s="18" t="s">
+      <c r="B84" s="5" t="s">
         <v>2276</v>
       </c>
-      <c r="C84" s="18" t="s">
+      <c r="C84" s="5" t="s">
         <v>2360</v>
       </c>
-      <c r="D84" s="18" t="n">
+      <c r="D84" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E84" s="18" t="n">
+      <c r="E84" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F84" s="18" t="n">
+      <c r="F84" s="5" t="n">
         <f aca="false">D84-E84</f>
         <v>0</v>
       </c>
-      <c r="G84" s="18" t="str">
+      <c r="G84" s="5" t="str">
         <f aca="false">IF(E84&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="18" t="n">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="5" t="n">
         <v>95</v>
       </c>
-      <c r="B85" s="18" t="s">
+      <c r="B85" s="5" t="s">
         <v>2280</v>
       </c>
-      <c r="C85" s="18" t="s">
+      <c r="C85" s="5" t="s">
         <v>2361</v>
       </c>
-      <c r="D85" s="18" t="n">
+      <c r="D85" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E85" s="18" t="n">
+      <c r="E85" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F85" s="18" t="n">
+      <c r="F85" s="5" t="n">
         <f aca="false">D85-E85</f>
         <v>1</v>
       </c>
-      <c r="G85" s="18" t="str">
+      <c r="G85" s="5" t="str">
         <f aca="false">IF(E85&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="18" t="n">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="5" t="n">
         <v>98</v>
       </c>
-      <c r="B86" s="18" t="s">
+      <c r="B86" s="5" t="s">
         <v>2278</v>
       </c>
-      <c r="C86" s="18" t="s">
+      <c r="C86" s="5" t="s">
         <v>2362</v>
       </c>
-      <c r="D86" s="18" t="n">
+      <c r="D86" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E86" s="18" t="n">
+      <c r="E86" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F86" s="18" t="n">
+      <c r="F86" s="5" t="n">
         <f aca="false">D86-E86</f>
         <v>0</v>
       </c>
-      <c r="G86" s="18" t="str">
+      <c r="G86" s="5" t="str">
         <f aca="false">IF(E86&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="18" t="n">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="5" t="n">
         <v>97</v>
       </c>
-      <c r="B87" s="18" t="s">
+      <c r="B87" s="5" t="s">
         <v>2282</v>
       </c>
-      <c r="C87" s="18" t="s">
+      <c r="C87" s="5" t="s">
         <v>2363</v>
       </c>
-      <c r="D87" s="18" t="n">
+      <c r="D87" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E87" s="18" t="n">
+      <c r="E87" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F87" s="18" t="n">
+      <c r="F87" s="5" t="n">
         <f aca="false">D87-E87</f>
         <v>0</v>
       </c>
-      <c r="G87" s="18" t="str">
+      <c r="G87" s="5" t="str">
         <f aca="false">IF(E87&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="18" t="n">
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="5" t="n">
         <v>98</v>
       </c>
-      <c r="B88" s="18" t="s">
+      <c r="B88" s="5" t="s">
         <v>2273</v>
       </c>
-      <c r="C88" s="18" t="s">
+      <c r="C88" s="5" t="s">
         <v>2364</v>
       </c>
-      <c r="D88" s="18" t="n">
+      <c r="D88" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="E88" s="18" t="n">
+      <c r="E88" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F88" s="18" t="n">
+      <c r="F88" s="5" t="n">
         <f aca="false">D88-E88</f>
         <v>1</v>
       </c>
-      <c r="G88" s="18" t="str">
+      <c r="G88" s="5" t="str">
         <f aca="false">IF(E88&gt;=5,"Check","")</f>
         <v/>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B90" s="19" t="s">
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B90" s="7" t="s">
         <v>2365</v>
       </c>
-      <c r="D90" s="18" t="n">
+      <c r="D90" s="5" t="n">
         <f aca="false">COUNTIF(D2:D88,"&gt;=5")</f>
         <v>10</v>
       </c>
-      <c r="E90" s="18" t="n">
+      <c r="E90" s="5" t="n">
         <f aca="false">COUNTIF(E2:E88,"&gt;=5")</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Chamomile shows calm and comfort up front
Entries can now show more than one keyword. Chamomile, which the first
puzzle needs for its comfort theme, shows calm and comfort and hides
sleep and healing. Spellbook Herbiary row, blank rule and Ingredient
Feel order updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -4413,7 +4413,7 @@
     <t xml:space="preserve">confidence,healing,joy</t>
   </si>
   <si>
-    <t xml:space="preserve">calm, sleep, comfort, healing</t>
+    <t xml:space="preserve">calm, comfort, sleep, healing</t>
   </si>
   <si>
     <t xml:space="preserve">For the child who lies awake worrying. Mild as warm milk.</t>
@@ -42183,7 +42183,7 @@
       </c>
       <c r="L24" s="5" t="str">
         <f aca="false">", "&amp;C24&amp;", "</f>
-        <v>, calm, sleep, comfort, healing, </v>
+        <v>, calm, comfort, sleep, healing, </v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Fixed, slightly hard visible keywords; letter three adds #111's themes
- Visible keywords are now a fixed table, the same every playthrough:
  most entries show their second most-used keyword across the 240
  recipes so the obvious link stays hidden; week-one puzzle parts
  show the keyword their recipe needs; 5+ keyword entries show two
- Entries are keyed per book, so the Lavender herb and the Lavender
  colour no longer share keywords or filled blanks (save key bumped)
- 25 book lines that named a now-hidden keyword reworded
- Letter three also adds intuition, transformation and truth
- Spellbook book tables synced to the game's shown/hidden keywords

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -4347,7 +4347,7 @@
     <t xml:space="preserve">rest, calm, cleansing</t>
   </si>
   <si>
-    <t xml:space="preserve">Hushes the body toward rest.</t>
+    <t xml:space="preserve">Hushes the body, like a house after snowfall.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,cleansing,rest</t>
@@ -4425,7 +4425,7 @@
     <t xml:space="preserve">luck, friendship, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Small, everyday luck, shared between friends.</t>
+    <t xml:space="preserve">Small, everyday good fortune, shared between friends.</t>
   </si>
   <si>
     <t xml:space="preserve">friendship,joy,luck</t>
@@ -4512,7 +4512,7 @@
     <t xml:space="preserve">luck, opportunity, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Rare and potent luck. Opens doors that were shut.</t>
+    <t xml:space="preserve">Rare and potent fortune. Opens doors that were shut.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,luck,opportunity</t>
@@ -4530,7 +4530,7 @@
     <t xml:space="preserve">passion, love, beauty</t>
   </si>
   <si>
-    <t xml:space="preserve">Hot-blooded. Passion you can feel in your cheeks.</t>
+    <t xml:space="preserve">Hot-blooded. A fire you can feel in your cheeks.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,love,passion</t>
@@ -4539,7 +4539,7 @@
     <t xml:space="preserve">sleep, rest, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Heavy-lidded and gentle. Brings the body down to sleep.</t>
+    <t xml:space="preserve">Heavy-lidded and gentle. Brings the body down for the night.</t>
   </si>
   <si>
     <t xml:space="preserve">calm,rest,sleep</t>
@@ -4617,7 +4617,7 @@
     <t xml:space="preserve">dreams, intuition, protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Strong dreams, open sight, watchful sleep. Not for the faint-hearted.</t>
+    <t xml:space="preserve">Vivid nights, open sight, a watchful pillow. Not for the faint-hearted.</t>
   </si>
   <si>
     <t xml:space="preserve">dreams,intuition,protection</t>
@@ -4746,7 +4746,7 @@
     <t xml:space="preserve">courage, confidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Courage for a fearful heart.</t>
+    <t xml:space="preserve">Nerve for a fearful heart.</t>
   </si>
   <si>
     <t xml:space="preserve">confidence,courage</t>
@@ -5046,7 +5046,7 @@
     <t xml:space="preserve">success, passion, abundance, energy, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Quick success and warm plenty.</t>
+    <t xml:space="preserve">Quick wins and warm plenty.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,comfort,energy,passion,success</t>
@@ -5214,7 +5214,7 @@
     <t xml:space="preserve">comfort, rest, self-love</t>
   </si>
   <si>
-    <t xml:space="preserve">Nursery comfort for grown-ups who need tucking in.</t>
+    <t xml:space="preserve">Nursery softness for grown-ups who need tucking in.</t>
   </si>
   <si>
     <t xml:space="preserve">comfort,rest,self-love</t>
@@ -5241,7 +5241,7 @@
     <t xml:space="preserve">luck, joy</t>
   </si>
   <si>
-    <t xml:space="preserve">Birthday-cake luck for whoever blows out the candles.</t>
+    <t xml:space="preserve">Birthday-cake fortune for whoever blows out the candles.</t>
   </si>
   <si>
     <t xml:space="preserve">joy,luck</t>
@@ -5253,7 +5253,7 @@
     <t xml:space="preserve">beauty, self-love, comfort</t>
   </si>
   <si>
-    <t xml:space="preserve">Draws out and smooths the skin. A beauty mask.</t>
+    <t xml:space="preserve">Draws out and smooths the skin. A face mask for a glow.</t>
   </si>
   <si>
     <t xml:space="preserve">protection, cleansing, grounding, home</t>
@@ -5295,7 +5295,7 @@
     <t xml:space="preserve">protection, beginnings</t>
   </si>
   <si>
-    <t xml:space="preserve">Crushed shell for gentle protection of new things.</t>
+    <t xml:space="preserve">Crushed shell that gently guards new things.</t>
   </si>
   <si>
     <t xml:space="preserve">beginnings,protection</t>
@@ -5454,7 +5454,7 @@
     <t xml:space="preserve">courage, creativity, energy</t>
   </si>
   <si>
-    <t xml:space="preserve">Fire for action and courage.</t>
+    <t xml:space="preserve">Fire for action and nerve.</t>
   </si>
   <si>
     <t xml:space="preserve">courage,creativity,energy</t>
@@ -5499,7 +5499,7 @@
     <t xml:space="preserve">luck, opportunity, abundance</t>
   </si>
   <si>
-    <t xml:space="preserve">Gentle luck and new chances.</t>
+    <t xml:space="preserve">Gentle good fortune and new chances.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance,luck,opportunity</t>
@@ -5508,7 +5508,7 @@
     <t xml:space="preserve">grounding, protection, focus</t>
   </si>
   <si>
-    <t xml:space="preserve">Heavy grounding for the body.</t>
+    <t xml:space="preserve">Heavy iron weight that keeps the body steady.</t>
   </si>
   <si>
     <t xml:space="preserve">focus,grounding,protection</t>
@@ -5535,7 +5535,7 @@
     <t xml:space="preserve">transformation, intuition, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Shifting light of transformation.</t>
+    <t xml:space="preserve">Shifting light, for becoming someone new.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,intuition,transformation</t>
@@ -5544,7 +5544,7 @@
     <t xml:space="preserve">truth, communication</t>
   </si>
   <si>
-    <t xml:space="preserve">The stone of truth-telling.</t>
+    <t xml:space="preserve">The stone for saying what is real.</t>
   </si>
   <si>
     <t xml:space="preserve">communication,truth</t>
@@ -5586,7 +5586,7 @@
     <t xml:space="preserve">beauty, self-love, calm</t>
   </si>
   <si>
-    <t xml:space="preserve">Lustrous and still. Beauty that doesn't need to try.</t>
+    <t xml:space="preserve">Lustrous and still. Loveliness that doesn't need to try.</t>
   </si>
   <si>
     <t xml:space="preserve">beauty,calm,self-love</t>
@@ -5691,7 +5691,7 @@
     <t xml:space="preserve">boundaries, protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Prickly. Boundaries for someone too soft-hearted.</t>
+    <t xml:space="preserve">Prickly. A line drawn for someone too soft-hearted.</t>
   </si>
   <si>
     <t xml:space="preserve">abundance, home, friendship</t>
@@ -5706,7 +5706,7 @@
     <t xml:space="preserve">luck, opportunity, play</t>
   </si>
   <si>
-    <t xml:space="preserve">Snatches luck and chances.</t>
+    <t xml:space="preserve">Snatches fortune and chances.</t>
   </si>
   <si>
     <t xml:space="preserve">luck,opportunity,play</t>
@@ -5715,7 +5715,7 @@
     <t xml:space="preserve">dreams, transformation, intuition</t>
   </si>
   <si>
-    <t xml:space="preserve">Drawn to the moon. Uncanny dreams and change.</t>
+    <t xml:space="preserve">Drawn to the moon. Uncanny nights and change.</t>
   </si>
   <si>
     <t xml:space="preserve">dreams,intuition,transformation</t>
@@ -6024,7 +6024,7 @@
     <t xml:space="preserve">love, attraction</t>
   </si>
   <si>
-    <t xml:space="preserve">Deep, devoted love.</t>
+    <t xml:space="preserve">Deep, devoted affection.</t>
   </si>
   <si>
     <t xml:space="preserve">attraction,love</t>
@@ -6108,7 +6108,7 @@
     <t xml:space="preserve">play, opportunity, travel</t>
   </si>
   <si>
-    <t xml:space="preserve">Wandering play and small chances.</t>
+    <t xml:space="preserve">Wandering games and small chances.</t>
   </si>
   <si>
     <t xml:space="preserve">opportunity,play,travel</t>
@@ -6141,7 +6141,7 @@
     <t xml:space="preserve">luck, abundance</t>
   </si>
   <si>
-    <t xml:space="preserve">Hard luck you can hold.</t>
+    <t xml:space="preserve">Hard fortune you can hold.</t>
   </si>
   <si>
     <t xml:space="preserve">protection, play, wonder</t>
@@ -6243,7 +6243,7 @@
     <t xml:space="preserve">luck, play</t>
   </si>
   <si>
-    <t xml:space="preserve">A roll of chance. Bold luck.</t>
+    <t xml:space="preserve">A roll of chance. Bold fortune.</t>
   </si>
   <si>
     <t xml:space="preserve">Write a name in it, then burn the page.</t>

</xml_diff>

<commit_message>
Hide keywords where showing one barely matters; shuffle blank positions
- Two-keyword entries that only one or two recipes use now show no
  keyword (47 entries); others keep the slightly-hard choice, week-one
  parts stay pinned
- Shown keywords and blanks sit in a fixed shuffled order, so the
  shown one is no longer always first
- Colour entries no longer borrow a same-named herb's book line
- Two book lines reworded; spellbook tables and blank rule synced

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -4356,7 +4356,7 @@
     <t xml:space="preserve">energy, creativity</t>
   </si>
   <si>
-    <t xml:space="preserve">Raw, crackling energy for a stuck mind.</t>
+    <t xml:space="preserve">Raw, crackling force for a stuck mind.</t>
   </si>
   <si>
     <t xml:space="preserve">creativity,energy</t>
@@ -6102,7 +6102,7 @@
     <t xml:space="preserve">courage,grounding,protection</t>
   </si>
   <si>
-    <t xml:space="preserve">Hung over the door. Old, steady protection.</t>
+    <t xml:space="preserve">Hung over the door. Old, steady guard.</t>
   </si>
   <si>
     <t xml:space="preserve">play, opportunity, travel</t>

</xml_diff>

<commit_message>
Point letters only at dead ends: ingredients a keyword search can't find
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -972,7 +972,7 @@
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>Letters lists the 17 letters that arrive in the post: sender, the one or two ingredients each describes, the keyword it names, and the first order that needs it. Letters are a side help; every order can be solved without them.</t>
+          <t>Letters lists the 17 letters that arrive in the post. Each points at a dead end: an ingredient whose needed keyword is hidden, so searching collected words won't find it. Columns give the keyword it names, the first order that needs it, and why that spot is hard. Letters are a side help; every order can be solved without them.</t>
         </is>
       </c>
     </row>
@@ -74005,22 +74005,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="18" min="1" max="1"/>
     <col width="10" customWidth="1" style="18" min="2" max="2"/>
-    <col width="34" customWidth="1" style="18" min="3" max="3"/>
-    <col width="12" customWidth="1" style="18" min="4" max="4"/>
-    <col width="40" customWidth="1" style="18" min="5" max="5"/>
-    <col width="9" customWidth="1" style="18" min="6" max="6"/>
-    <col width="18" customWidth="1" style="18" min="7" max="7"/>
-    <col width="13" customWidth="1" style="18" min="8" max="8"/>
-    <col width="34" customWidth="1" style="18" min="9" max="9"/>
+    <col width="32" customWidth="1" style="18" min="3" max="3"/>
+    <col width="36" customWidth="1" style="18" min="4" max="4"/>
+    <col width="9" customWidth="1" style="18" min="5" max="5"/>
+    <col width="18" customWidth="1" style="18" min="6" max="6"/>
+    <col width="13" customWidth="1" style="18" min="7" max="7"/>
+    <col width="32" customWidth="1" style="18" min="8" max="8"/>
+    <col width="40" customWidth="1" style="18" min="9" max="9"/>
     <col width="18" customWidth="1" style="18" min="10" max="10"/>
     <col width="13" customWidth="1" style="18" min="11" max="11"/>
-    <col width="34" customWidth="1" style="18" min="12" max="12"/>
-    <col width="90" customWidth="1" style="18" min="13" max="13"/>
+    <col width="32" customWidth="1" style="18" min="12" max="12"/>
+    <col width="40" customWidth="1" style="18" min="13" max="13"/>
+    <col width="90" customWidth="1" style="18" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -74041,32 +74042,32 @@
       </c>
       <c r="D1" s="33" t="inlineStr">
         <is>
-          <t>Place type</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="E1" s="33" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Hints (#)</t>
         </is>
       </c>
       <c r="F1" s="33" t="inlineStr">
         <is>
-          <t>Hints (#)</t>
+          <t>Ingredient 1</t>
         </is>
       </c>
       <c r="G1" s="33" t="inlineStr">
         <is>
-          <t>Ingredient 1</t>
+          <t>Keyword 1</t>
         </is>
       </c>
       <c r="H1" s="33" t="inlineStr">
         <is>
-          <t>Keyword 1</t>
+          <t>First needed 1</t>
         </is>
       </c>
       <c r="I1" s="33" t="inlineStr">
         <is>
-          <t>First needed 1</t>
+          <t>Why it is hard 1</t>
         </is>
       </c>
       <c r="J1" s="33" t="inlineStr">
@@ -74085,6 +74086,11 @@
         </is>
       </c>
       <c r="M1" s="33" t="inlineStr">
+        <is>
+          <t>Why it is hard 2</t>
+        </is>
+      </c>
+      <c r="N1" s="33" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
@@ -74106,36 +74112,37 @@
       </c>
       <c r="D2" s="34" t="inlineStr">
         <is>
-          <t>Market town</t>
-        </is>
-      </c>
-      <c r="E2" s="34" t="inlineStr">
-        <is>
           <t>From the apothecary on Mill Lane</t>
         </is>
       </c>
-      <c r="F2" s="34" t="n">
+      <c r="E2" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F2" s="34" t="inlineStr">
+        <is>
+          <t>Nettle</t>
+        </is>
+      </c>
       <c r="G2" s="34" t="inlineStr">
         <is>
-          <t>Nettle</t>
+          <t>healing</t>
         </is>
       </c>
       <c r="H2" s="34" t="inlineStr">
         <is>
-          <t>healing</t>
+          <t>Day 1 · #194 The Inner Housekeeper</t>
         </is>
       </c>
       <c r="I2" s="34" t="inlineStr">
         <is>
-          <t>Day 1 · #194 The Inner Housekeeper</t>
+          <t>its entry shows no keyword; searching healing finds 3 other herbs &amp; flowers entries instead</t>
         </is>
       </c>
       <c r="J2" s="34" t="inlineStr"/>
       <c r="K2" s="34" t="inlineStr"/>
       <c r="L2" s="34" t="inlineStr"/>
-      <c r="M2" s="34" t="inlineStr">
+      <c r="M2" s="34" t="inlineStr"/>
+      <c r="N2" s="34" t="inlineStr">
         <is>
           <t>To whoever keeps the Emporium now,
 Our shelves are bare of the one herb we can't do without. You'll know the one: it stings your fingers when you pick it, and then it builds a worn-out body back up. Nothing does more for healing after a long sickness.
@@ -74146,73 +74153,78 @@
     </row>
     <row r="3">
       <c r="A3" s="34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" s="34" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Twilight</t>
         </is>
       </c>
       <c r="C3" s="34" t="inlineStr">
         <is>
-          <t>The Stanbridge Library of Old Craft</t>
+          <t>The Halloway Baths</t>
         </is>
       </c>
       <c r="D3" s="34" t="inlineStr">
         <is>
-          <t>University city</t>
-        </is>
-      </c>
-      <c r="E3" s="34" t="inlineStr">
-        <is>
-          <t>From the Stanbridge Library of Old Craft</t>
-        </is>
-      </c>
-      <c r="F3" s="34" t="n">
+          <t>From the bathhouse at Halloway</t>
+        </is>
+      </c>
+      <c r="E3" s="34" t="n">
         <v>2</v>
       </c>
+      <c r="F3" s="34" t="inlineStr">
+        <is>
+          <t>Epsom salt</t>
+        </is>
+      </c>
       <c r="G3" s="34" t="inlineStr">
         <is>
-          <t>Licorice root</t>
+          <t>cleansing</t>
         </is>
       </c>
       <c r="H3" s="34" t="inlineStr">
         <is>
-          <t>confidence</t>
+          <t>Day 10 · #161 The Fresh Linen Familiar</t>
         </is>
       </c>
       <c r="I3" s="34" t="inlineStr">
         <is>
-          <t>Day 4 · #49 The Unmasked Self</t>
+          <t>its entry shows no keyword; searching cleansing finds 2 other pantry: salts, sugars &amp; baking entries instead</t>
         </is>
       </c>
       <c r="J3" s="34" t="inlineStr">
         <is>
-          <t>Lapis lazuli</t>
+          <t>Rose clay</t>
         </is>
       </c>
       <c r="K3" s="34" t="inlineStr">
         <is>
-          <t>truth</t>
+          <t>comfort</t>
         </is>
       </c>
       <c r="L3" s="34" t="inlineStr">
         <is>
-          <t>Day 10 · #88 The Guiding Thread</t>
+          <t>Day 45 · #98 The Soft Return</t>
         </is>
       </c>
       <c r="M3" s="34" t="inlineStr">
         <is>
-          <t>To the keeper of the Emporium,
-Your shop still holds our copy of Herbs for the Lecture Hall (overdue since 1987). Chapter four is on the sweet black root that speakers chew before a big crowd; the author claims it lends the timid confidence. Chapter nine is on the blue stone flecked with gold that old scholars ground into their ink, so that whatever they wrote would be the truth.
-Kindly return the book, or failing that, a box of the root.
-The Librarian, Stanbridge Library of Old Craft</t>
+          <t>its entry shows only self-love; searching comfort finds 3 other pantry: salts, sugars &amp; baking entries instead</t>
+        </is>
+      </c>
+      <c r="N3" s="34" t="inlineStr">
+        <is>
+          <t>To the Emporium,
+Two orders, if you would. The bitter white crystals our guests tip into the hot pool after a long walk: they draw the ache out of the legs, and my mother called a soak in them a proper cleansing. And the soft pink mud for the face masks. The old ladies say nothing gives them more comfort of an evening.
+We have been buying poor stuff from Marrowgate and the guests can tell.
+Mr Hugo Fairweather, Manager, the Halloway Baths</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="34" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B4" s="34" t="inlineStr">
         <is>
@@ -74221,95 +74233,42 @@
       </c>
       <c r="C4" s="34" t="inlineStr">
         <is>
-          <t>Thistle &amp; Sons Wandwrights, Elderhollow</t>
+          <t>The Honeywell Beekeepers</t>
         </is>
       </c>
       <c r="D4" s="34" t="inlineStr">
         <is>
-          <t>Forest village</t>
-        </is>
-      </c>
-      <c r="E4" s="34" t="inlineStr">
-        <is>
-          <t>From the wandwrights in Elderhollow</t>
-        </is>
-      </c>
-      <c r="F4" s="34" t="n">
+          <t>From the beekeepers of Honeywell</t>
+        </is>
+      </c>
+      <c r="E4" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F4" s="34" t="inlineStr">
+        <is>
+          <t>Sweet pea</t>
+        </is>
+      </c>
       <c r="G4" s="34" t="inlineStr">
         <is>
-          <t>Ash wood</t>
+          <t>friendship</t>
         </is>
       </c>
       <c r="H4" s="34" t="inlineStr">
         <is>
-          <t>intuition</t>
+          <t>Day 12 · #65 Words Like Honey</t>
         </is>
       </c>
       <c r="I4" s="34" t="inlineStr">
         <is>
-          <t>Day 1 · #111 The Language of Ravens</t>
+          <t>its entry shows no keyword; searching friendship finds 1 other herbs &amp; flowers entry instead</t>
         </is>
       </c>
       <c r="J4" s="34" t="inlineStr"/>
       <c r="K4" s="34" t="inlineStr"/>
       <c r="L4" s="34" t="inlineStr"/>
-      <c r="M4" s="34" t="inlineStr">
-        <is>
-          <t>Madam,
-We are short of the pale, straight-grained wood the old carvers cut their staves of sight from. A wand of it points true. My grandfather swore it sharpened a witch's intuition better than any crystal.
-If you have offcuts in the back, we would pay well for them.
-Silas Thistle, Thistle &amp; Sons Wandwrights, Elderhollow</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="34" t="n">
-        <v>9</v>
-      </c>
-      <c r="B5" s="34" t="inlineStr">
-        <is>
-          <t>Twilight</t>
-        </is>
-      </c>
-      <c r="C5" s="34" t="inlineStr">
-        <is>
-          <t>The Honeywell Beekeepers</t>
-        </is>
-      </c>
-      <c r="D5" s="34" t="inlineStr">
-        <is>
-          <t>Village</t>
-        </is>
-      </c>
-      <c r="E5" s="34" t="inlineStr">
-        <is>
-          <t>From the beekeepers of Honeywell</t>
-        </is>
-      </c>
-      <c r="F5" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="34" t="inlineStr">
-        <is>
-          <t>Sweet pea</t>
-        </is>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>friendship</t>
-        </is>
-      </c>
-      <c r="I5" s="34" t="inlineStr">
-        <is>
-          <t>Day 12 · #65 Words Like Honey</t>
-        </is>
-      </c>
-      <c r="J5" s="34" t="inlineStr"/>
-      <c r="K5" s="34" t="inlineStr"/>
-      <c r="L5" s="34" t="inlineStr"/>
-      <c r="M5" s="34" t="inlineStr">
+      <c r="M4" s="34" t="inlineStr"/>
+      <c r="N4" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
 We grow a ruffled, sweet-smelling climber along the hive fence, the flower everyone sends when they mean thank you. The bees adore it and so do the neighbours. A jar of honey and a posy of it on the doorstep has kept friendship sweet on our lane for forty years.
@@ -74318,195 +74277,277 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="B5" s="34" t="inlineStr">
+        <is>
+          <t>Noon</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>Cloverdale Village School</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>From the village school in Cloverdale</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Daisy</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>friendship</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>Day 13 · #68 A Thousand Little Lights</t>
+        </is>
+      </c>
+      <c r="I5" s="34" t="inlineStr">
+        <is>
+          <t>its entry shows only beginnings; searching friendship finds 7 other herbs &amp; flowers entries instead</t>
+        </is>
+      </c>
+      <c r="J5" s="34" t="inlineStr">
+        <is>
+          <t>Clover</t>
+        </is>
+      </c>
+      <c r="K5" s="34" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="L5" s="34" t="inlineStr">
+        <is>
+          <t>Day 20 · #31 Cloverkiss</t>
+        </is>
+      </c>
+      <c r="M5" s="34" t="inlineStr">
+        <is>
+          <t>its entry shows only friendship; searching luck finds 7 other herbs &amp; flowers entries instead</t>
+        </is>
+      </c>
+      <c r="N5" s="34" t="inlineStr">
+        <is>
+          <t>Dear Emporium,
+A new girl starts with us next week, and I want her first day to go well. Here the children make a chain of the little white-and-yellow field flowers for anyone new; it is how friendship starts in Cloverdale. The older ones go hunting in the fields for the plain three-leaved kind to tuck in her pocket, for luck.
+The frost has spoilt both. Have you any dried?
+Miss Primrose Dell, Cloverdale Village School</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="34" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="34" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Noon</t>
         </is>
       </c>
       <c r="C6" s="34" t="inlineStr">
         <is>
-          <t>The Copper Kettle, Teacup Lane, Marrowgate</t>
+          <t>Lavinia's Bridal Rooms, Kingsmere</t>
         </is>
       </c>
       <c r="D6" s="34" t="inlineStr">
         <is>
-          <t>City</t>
-        </is>
-      </c>
-      <c r="E6" s="34" t="inlineStr">
-        <is>
-          <t>From a tea room on Teacup Lane</t>
-        </is>
-      </c>
-      <c r="F6" s="34" t="n">
+          <t>From a bridal boutique in Kingsmere</t>
+        </is>
+      </c>
+      <c r="E6" s="34" t="n">
         <v>2</v>
       </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>Orange blossom</t>
+        </is>
+      </c>
       <c r="G6" s="34" t="inlineStr">
         <is>
-          <t>Bergamot</t>
+          <t>joy</t>
         </is>
       </c>
       <c r="H6" s="34" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>Day 16 · #55 Celestial Spotlight</t>
         </is>
       </c>
       <c r="I6" s="34" t="inlineStr">
         <is>
-          <t>Day 15 · #165 The Solitude Sweetspot</t>
+          <t>its entry shows no keyword; searching joy finds 7 other herbs &amp; flowers entries instead</t>
         </is>
       </c>
       <c r="J6" s="34" t="inlineStr">
         <is>
-          <t>Black tea</t>
+          <t>White lily</t>
         </is>
       </c>
       <c r="K6" s="34" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>beauty</t>
         </is>
       </c>
       <c r="L6" s="34" t="inlineStr">
         <is>
-          <t>Day 15 · #165 The Solitude Sweetspot</t>
+          <t>Day 24 · #52 Swanlight</t>
         </is>
       </c>
       <c r="M6" s="34" t="inlineStr">
         <is>
-          <t>Hello from Marrowgate!
-Two requests from a very tired city. First, the little citrus that perfumes a good grey tea: our four o'clock ladies say nothing keeps them calm through a quarrel like it. Second, the strong dark leaf itself, brewed thick. Our night porters need the energy.
-Could we order a tin of each?
-Bess, The Copper Kettle, Teacup Lane</t>
+          <t>its entry shows only truth; searching beauty finds 5 other herbs &amp; flowers entries instead</t>
+        </is>
+      </c>
+      <c r="N6" s="34" t="inlineStr">
+        <is>
+          <t>Darling shop,
+Wedding season is upon us. My brides want the small white flowers from the citrus tree woven into their hair, as their grandmothers wore them: they say a bride crowned with them glows with joy. The tall still white flower goes in the bouquet. Nothing gives a quiet bride beauty like it.
+Send whatever you can. Kingsmere does not do things by halves.
+Lavinia, Lavinia's Bridal Rooms, Kingsmere</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="34" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t>Noon</t>
+          <t>Twilight</t>
         </is>
       </c>
       <c r="C7" s="34" t="inlineStr">
         <is>
-          <t>St Aldric's Church, Thornbury</t>
+          <t>The Coastguard Station, Caldwell-on-Sea</t>
         </is>
       </c>
       <c r="D7" s="34" t="inlineStr">
         <is>
-          <t>Walled town</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="inlineStr">
-        <is>
-          <t>From the churchwarden at Thornbury</t>
-        </is>
-      </c>
-      <c r="F7" s="34" t="n">
+          <t>From the coastguard at Caldwell-on-Sea</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>Black tourmaline</t>
+        </is>
+      </c>
       <c r="G7" s="34" t="inlineStr">
         <is>
-          <t>Black pepper</t>
+          <t>protection</t>
         </is>
       </c>
       <c r="H7" s="34" t="inlineStr">
         <is>
-          <t>courage</t>
+          <t>Day 15 · #16 The Iron Moon</t>
         </is>
       </c>
       <c r="I7" s="34" t="inlineStr">
         <is>
-          <t>Day 25 · #85 First Spark, First Flame</t>
+          <t>its entry shows no keyword; searching protection finds 3 other crystals entries instead</t>
         </is>
       </c>
       <c r="J7" s="34" t="inlineStr"/>
       <c r="K7" s="34" t="inlineStr"/>
       <c r="L7" s="34" t="inlineStr"/>
-      <c r="M7" s="34" t="inlineStr">
+      <c r="M7" s="34" t="inlineStr"/>
+      <c r="N7" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-The vicar has asked me, against my better judgement, to write. Before every sermon he grinds the little hot black corns over his breakfast eggs. He says the heat in the belly gives him the courage to face the congregation.
-Our grocer has run out. I trust this stays between us.
-Mr Edgar Penhallow, Churchwarden, Thornbury</t>
+Every coastguard on this stretch keeps a black, ridged stone in his coat, the kind that looks like a bundle of burnt matches. The old men say it soaks up whatever is thrown at you. It is the only protection I trust on a night shift.
+Mine went over the side in the last storm. Could you send another?
+Officer Jory Penrose, Caldwell-on-Sea</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="34" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B8" s="34" t="inlineStr">
         <is>
-          <t>Twilight</t>
+          <t>Noon</t>
         </is>
       </c>
       <c r="C8" s="34" t="inlineStr">
         <is>
-          <t>Lavinia's Bridal Rooms, Kingsmere</t>
+          <t>St Aldric's Church, Thornbury</t>
         </is>
       </c>
       <c r="D8" s="34" t="inlineStr">
         <is>
-          <t>Lake town</t>
-        </is>
-      </c>
-      <c r="E8" s="34" t="inlineStr">
-        <is>
-          <t>From a bridal boutique in Kingsmere</t>
-        </is>
-      </c>
-      <c r="F8" s="34" t="n">
+          <t>From the churchwarden at Thornbury</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="n">
         <v>2</v>
       </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>Copal</t>
+        </is>
+      </c>
       <c r="G8" s="34" t="inlineStr">
         <is>
-          <t>Hibiscus</t>
+          <t>calm</t>
         </is>
       </c>
       <c r="H8" s="34" t="inlineStr">
         <is>
-          <t>passion</t>
+          <t>Day 21 · #96 The Last Candle</t>
         </is>
       </c>
       <c r="I8" s="34" t="inlineStr">
         <is>
-          <t>Day 39 · #4 Ember of Eden</t>
+          <t>its entry shows no keyword; searching calm finds 1 other resins &amp; incense entry instead</t>
         </is>
       </c>
       <c r="J8" s="34" t="inlineStr">
         <is>
-          <t>Peach</t>
+          <t>Black pepper</t>
         </is>
       </c>
       <c r="K8" s="34" t="inlineStr">
         <is>
-          <t>beauty</t>
+          <t>courage</t>
         </is>
       </c>
       <c r="L8" s="34" t="inlineStr">
         <is>
-          <t>Day 45 · #222 The Camera Loves You</t>
+          <t>Day 25 · #85 First Spark, First Flame</t>
         </is>
       </c>
       <c r="M8" s="34" t="inlineStr">
         <is>
-          <t>Darling shop,
-Wedding season is upon us and my brides want two things. A deep red flower steeped into a tea that brings a hot flush to the cheeks; one of my grooms called it pure passion. And the soft, fuzzy summer fruit for the skin. Nothing gives a bride beauty like it on the morning.
-Send whatever you can. Kingsmere does not do things by halves.
-Lavinia, Lavinia's Bridal Rooms, Kingsmere</t>
+          <t>its entry shows no keyword; searching courage finds 1 other spices entry instead</t>
+        </is>
+      </c>
+      <c r="N8" s="34" t="inlineStr">
+        <is>
+          <t>To the Emporium,
+The vicar has asked me, against my better judgement, to write. He wants the pale sweet resin from overseas for the censer. When it burns, he says, the whole parish sits together in calm, even the Hendersons. He also grinds the little hot black corns over his breakfast eggs before every sermon, for the courage to face us.
+Our grocer has run out of both. I trust this stays between us.
+Mr Edgar Penhallow, Churchwarden, Thornbury</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="34" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B9" s="34" t="inlineStr">
         <is>
@@ -74515,346 +74556,360 @@
       </c>
       <c r="C9" s="34" t="inlineStr">
         <is>
-          <t>The Wool Basket, Little Mitten</t>
+          <t>Damson Cottage Jams, Plumtree Hollow</t>
         </is>
       </c>
       <c r="D9" s="34" t="inlineStr">
         <is>
-          <t>Hill village</t>
-        </is>
-      </c>
-      <c r="E9" s="34" t="inlineStr">
-        <is>
-          <t>From a wool shop in Little Mitten</t>
-        </is>
-      </c>
-      <c r="F9" s="34" t="n">
+          <t>From a jam-maker in Plumtree Hollow</t>
+        </is>
+      </c>
+      <c r="E9" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>Peridot</t>
+        </is>
+      </c>
       <c r="G9" s="34" t="inlineStr">
         <is>
-          <t>Rainbow threads</t>
+          <t>growth</t>
         </is>
       </c>
       <c r="H9" s="34" t="inlineStr">
         <is>
-          <t>friendship</t>
+          <t>Day 25 · #135 The Green Comet</t>
         </is>
       </c>
       <c r="I9" s="34" t="inlineStr">
         <is>
-          <t>Day 36 · #61 The Wildflower Circle</t>
+          <t>its entry shows no keyword; searching growth finds 1 other crystals entry instead</t>
         </is>
       </c>
       <c r="J9" s="34" t="inlineStr"/>
       <c r="K9" s="34" t="inlineStr"/>
       <c r="L9" s="34" t="inlineStr"/>
-      <c r="M9" s="34" t="inlineStr">
-        <is>
-          <t>Hello there,
-Every summer the children here plait bracelets out of every colour we stock and swap them on the last day of camp. Our knitting circle swears those swaps are where friendship in this village starts.
-We're short of the bright mixed bundles. Have you any put by?
-Nell, The Wool Basket, Little Mitten</t>
+      <c r="M9" s="34" t="inlineStr"/>
+      <c r="N9" s="34" t="inlineStr">
+        <is>
+          <t>Hello from the Hollow,
+When the plum trees come back after a bad winter, my aunt used to hang a little pale green stone on a ribbon from the oldest branch. She said it was for the first good week after a hard season, and for growth. The trees never failed her.
+The ribbon snapped and the stone is lost in the long grass. Do you sell them?
+Bessie Damson, Plumtree Hollow</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="34" t="n">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t>Noon</t>
+          <t>Twilight</t>
         </is>
       </c>
       <c r="C10" s="34" t="inlineStr">
         <is>
-          <t>The Cider Fair Committee, Pippin Green</t>
+          <t>Crumb &amp; Co. Bakery, Whitcombe</t>
         </is>
       </c>
       <c r="D10" s="34" t="inlineStr">
         <is>
-          <t>Orchard village</t>
-        </is>
-      </c>
-      <c r="E10" s="34" t="inlineStr">
-        <is>
-          <t>From the cider fair committee in Pippin Green</t>
-        </is>
-      </c>
-      <c r="F10" s="34" t="n">
+          <t>From the bakery in Whitcombe</t>
+        </is>
+      </c>
+      <c r="E10" s="34" t="n">
         <v>2</v>
       </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>Raisins</t>
+        </is>
+      </c>
       <c r="G10" s="34" t="inlineStr">
         <is>
-          <t>Apple peel</t>
+          <t>joy</t>
         </is>
       </c>
       <c r="H10" s="34" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>Day 29 · #90 The Pocket-Sized Triumph</t>
         </is>
       </c>
       <c r="I10" s="34" t="inlineStr">
         <is>
-          <t>Day 39 · #4 Ember of Eden</t>
+          <t>its entry shows no keyword; searching joy finds 2 other fruits entries instead</t>
         </is>
       </c>
       <c r="J10" s="34" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Cocoa</t>
         </is>
       </c>
       <c r="K10" s="34" t="inlineStr">
         <is>
-          <t>love</t>
+          <t>comfort</t>
         </is>
       </c>
       <c r="L10" s="34" t="inlineStr">
         <is>
-          <t>Day 87 · #3 Two Hearts, One Hearth</t>
+          <t>Day 32 · #235 The Sweetness Permission</t>
         </is>
       </c>
       <c r="M10" s="34" t="inlineStr">
         <is>
-          <t>Dear Emporium,
-Two traditions for this year's fair, and we'd like to do them properly. The long curl peeled in one go at the kitchen table, tossed over the shoulder, to make a house feel like home. And the whole fruit, shared bite for bite between two sweethearts, which our grandmothers called plain honest love.
-Could you advise? Or send a basket of anything that helps.
-Rhoda Bell, Cider Fair Committee, Pippin Green</t>
+          <t>its entry shows no keyword; searching comfort finds 3 other pantry: salts, sugars &amp; baking entries instead</t>
+        </is>
+      </c>
+      <c r="N10" s="34" t="inlineStr">
+        <is>
+          <t>Dear neighbour,
+Two things for the winter menu. The little shrivelled dark fruit we fold into lunch-box buns. The mothers say one bun is pure joy for a child at school. And the dark bitter powder for the mugs we serve when people come in from the cold. Nothing else is such a comfort in January.
+Our supplier in Greywater has gone bust. Could you help?
+Mrs Ada Crumb, Crumb &amp; Co., Whitcombe</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="34" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>Twilight</t>
+          <t>Noon</t>
         </is>
       </c>
       <c r="C11" s="34" t="inlineStr">
         <is>
-          <t>Mrs Pennywhistle's Sweet Shop, Sugarbrook</t>
+          <t>Thistle &amp; Sons Wandwrights, Elderhollow</t>
         </is>
       </c>
       <c r="D11" s="34" t="inlineStr">
         <is>
-          <t>Village</t>
-        </is>
-      </c>
-      <c r="E11" s="34" t="inlineStr">
-        <is>
-          <t>From the sweet shop in Sugarbrook</t>
-        </is>
-      </c>
-      <c r="F11" s="34" t="n">
-        <v>1</v>
+          <t>From the wandwrights in Elderhollow</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>Willow bark</t>
+        </is>
       </c>
       <c r="G11" s="34" t="inlineStr">
         <is>
-          <t>Pink glitter</t>
+          <t>intuition</t>
         </is>
       </c>
       <c r="H11" s="34" t="inlineStr">
         <is>
-          <t>play</t>
+          <t>Day 38 · #106 The Dreaming Garden</t>
         </is>
       </c>
       <c r="I11" s="34" t="inlineStr">
         <is>
-          <t>Day 56 · #198 The Forgiving Tide</t>
-        </is>
-      </c>
-      <c r="J11" s="34" t="inlineStr"/>
-      <c r="K11" s="34" t="inlineStr"/>
-      <c r="L11" s="34" t="inlineStr"/>
+          <t>its entry shows no keyword; searching intuition finds 4 other herbs &amp; flowers entries instead</t>
+        </is>
+      </c>
+      <c r="J11" s="34" t="inlineStr">
+        <is>
+          <t>Wormwood</t>
+        </is>
+      </c>
+      <c r="K11" s="34" t="inlineStr">
+        <is>
+          <t>transformation</t>
+        </is>
+      </c>
+      <c r="L11" s="34" t="inlineStr">
+        <is>
+          <t>Day 36 · #116 The Phoenix's First Petal</t>
+        </is>
+      </c>
       <c r="M11" s="34" t="inlineStr">
         <is>
-          <t>Dear shop,
-The girls who come in after school have been told to tone it down, and it shows. I used to dust their cake pops with the shiny pink stuff, and the whole lot of them would go back to play in the street like little ones again.
-Have you a pot to spare? I'll send fudge.
-Mrs Pennywhistle, Sugarbrook</t>
+          <t>its entry shows no keyword; searching transformation finds 1 other herbs &amp; flowers entry instead</t>
+        </is>
+      </c>
+      <c r="N11" s="34" t="inlineStr">
+        <is>
+          <t>Madam,
+Two old remedies my grandfather kept, which no one else seems to stock. The bark of the weeping tree by the river, which every grandmother uses for a sore back; few know that the old witches chewed it for intuition. And the bitter silver-grey herb he steeped in his spirits once a year, for transformation. He said it was not for the faint-hearted.
+If you have either, we would pay well.
+Silas Thistle, Thistle &amp; Sons Wandwrights, Elderhollow</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="34" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="B12" s="34" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Twilight</t>
         </is>
       </c>
       <c r="C12" s="34" t="inlineStr">
         <is>
-          <t>The Halloway Baths</t>
+          <t>The Crossed Keys Inn, Ashby Cross</t>
         </is>
       </c>
       <c r="D12" s="34" t="inlineStr">
         <is>
-          <t>Spa town</t>
-        </is>
-      </c>
-      <c r="E12" s="34" t="inlineStr">
-        <is>
-          <t>From the bathhouse at Halloway</t>
-        </is>
-      </c>
-      <c r="F12" s="34" t="n">
-        <v>2</v>
+          <t>From the coaching inn at Ashby Cross</t>
+        </is>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>Wooden die</t>
+        </is>
       </c>
       <c r="G12" s="34" t="inlineStr">
         <is>
-          <t>River stone</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="H12" s="34" t="inlineStr">
         <is>
-          <t>grounding</t>
+          <t>Day 39 · #232 The Critical-Hit Charm</t>
         </is>
       </c>
       <c r="I12" s="34" t="inlineStr">
         <is>
-          <t>Day 53 · #168 The Waiting Room Oracle</t>
-        </is>
-      </c>
-      <c r="J12" s="34" t="inlineStr">
-        <is>
-          <t>Seaweed</t>
-        </is>
-      </c>
-      <c r="K12" s="34" t="inlineStr">
-        <is>
-          <t>connection</t>
-        </is>
-      </c>
-      <c r="L12" s="34" t="inlineStr">
-        <is>
-          <t>Day 56 · #198 The Forgiving Tide</t>
-        </is>
-      </c>
-      <c r="M12" s="34" t="inlineStr">
+          <t>its entry shows no keyword; searching luck finds 1 other findings &amp; tools entry instead</t>
+        </is>
+      </c>
+      <c r="J12" s="34" t="inlineStr"/>
+      <c r="K12" s="34" t="inlineStr"/>
+      <c r="L12" s="34" t="inlineStr"/>
+      <c r="M12" s="34" t="inlineStr"/>
+      <c r="N12" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Our guests rush from the train straight into the hot pool, which is no good to anybody. My mother kept a bowl of smooth stones from the riverbed by the door for them to carry; she called it grounding. She also wrapped the old ones in sea greens fresh off the tide, and said it brought back the connection with friends far away.
-Would you supply us again?
-Mr Hugo Fairweather, Manager, the Halloway Baths</t>
+Travellers wait here for the coach, and the waiting turns to gambling by supper. One old carter swears by a little carved wooden cube with dots on its faces that he blessed at your shop years ago. He says it gives him luck every time he throws it.
+The other regulars now want one each. Do you still bless them?
+Harry Oakes, landlord, the Crossed Keys, Ashby Cross</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="34" t="n">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>Noon</t>
+          <t>Sunrise</t>
         </is>
       </c>
       <c r="C13" s="34" t="inlineStr">
         <is>
-          <t>Marchbank Haberdashery, Ribbonmere</t>
+          <t>The Starfall Retreat</t>
         </is>
       </c>
       <c r="D13" s="34" t="inlineStr">
         <is>
-          <t>Lakeside town</t>
-        </is>
-      </c>
-      <c r="E13" s="34" t="inlineStr">
-        <is>
-          <t>From a haberdasher in Ribbonmere</t>
-        </is>
-      </c>
-      <c r="F13" s="34" t="n">
+          <t>From the retreat at Starfall</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
       <c r="G13" s="34" t="inlineStr">
         <is>
-          <t>Velvet ribbon (red)</t>
+          <t>calm</t>
         </is>
       </c>
       <c r="H13" s="34" t="inlineStr">
         <is>
-          <t>love</t>
+          <t>Day 44 · #102 The Slow-Blooming Rose</t>
         </is>
       </c>
       <c r="I13" s="34" t="inlineStr">
         <is>
-          <t>Day 63 · #14 The Golden Vow</t>
+          <t>its entry shows only intuition; searching calm finds 4 other herbs &amp; flowers entries instead</t>
         </is>
       </c>
       <c r="J13" s="34" t="inlineStr"/>
       <c r="K13" s="34" t="inlineStr"/>
       <c r="L13" s="34" t="inlineStr"/>
-      <c r="M13" s="34" t="inlineStr">
+      <c r="M13" s="34" t="inlineStr"/>
+      <c r="N13" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-A gentleman came in wanting a deep red ribbon, the soft heavy kind, to tie round a ring box. He said his grandmother told him it holds a love that lasts. I sold him my last yard.
-If you keep any, I would buy the roll.
-Miss Agatha Marchbank, Ribbonmere</t>
+Our guests come up the mountain to sit and look at the stars, and most of them can't sit still for a minute. Our founder floated the great pale water flower in a bowl at the centre of the room. She said the inner sight it brings is only half its use; mostly it brings calm.
+Have you any dried blooms?
+Sister Wren, the Starfall Retreat</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="34" t="n">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B14" s="34" t="inlineStr">
         <is>
-          <t>Twilight</t>
+          <t>Noon</t>
         </is>
       </c>
       <c r="C14" s="34" t="inlineStr">
         <is>
-          <t>Dunmore Harvest Supper</t>
+          <t>Hedge End Farm, Bramblebee</t>
         </is>
       </c>
       <c r="D14" s="34" t="inlineStr">
         <is>
-          <t>Farming town</t>
-        </is>
-      </c>
-      <c r="E14" s="34" t="inlineStr">
-        <is>
-          <t>From the harvest supper at Dunmore</t>
-        </is>
-      </c>
-      <c r="F14" s="34" t="n">
+          <t>From a farm in Bramblebee</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>Rose thorns</t>
+        </is>
+      </c>
       <c r="G14" s="34" t="inlineStr">
         <is>
-          <t>Wheat</t>
+          <t>boundaries</t>
         </is>
       </c>
       <c r="H14" s="34" t="inlineStr">
         <is>
-          <t>gratitude</t>
+          <t>Day 50 · #9 The Unbinding Rose</t>
         </is>
       </c>
       <c r="I14" s="34" t="inlineStr">
         <is>
-          <t>Day 69 · #37 The Abundance Garden</t>
+          <t>its entry shows no keyword; searching boundaries finds 2 other herbs &amp; flowers entries instead</t>
         </is>
       </c>
       <c r="J14" s="34" t="inlineStr"/>
       <c r="K14" s="34" t="inlineStr"/>
       <c r="L14" s="34" t="inlineStr"/>
-      <c r="M14" s="34" t="inlineStr">
-        <is>
-          <t>Hello from Dunmore,
-The harvest supper is coming, and we've always hung a sheaf of the last golden stalks from the field over the door. Gran said it was for gratitude, and a farm that forgets to say thank you has a hard winter.
-The storm flattened ours. Could you send a bundle?
-Tom Furrow, Dunmore</t>
+      <c r="M14" s="34" t="inlineStr"/>
+      <c r="N14" s="34" t="inlineStr">
+        <is>
+          <t>Hello,
+My mother used to grow a hedge of the old pink climbing flowers along our lane, and she kept a jar of the sharp bits she clipped off the stems. One on the windowsill, she said, and people learn your boundaries without you saying a word.
+My sister-in-law visits every Sunday. Have you a jar?
+Dora Bramble, Hedge End Farm, Bramblebee</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="34" t="n">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="B15" s="34" t="inlineStr">
         <is>
@@ -74863,64 +74918,69 @@
       </c>
       <c r="C15" s="34" t="inlineStr">
         <is>
-          <t>Old Things, Buttonwick</t>
+          <t>Mrs Pennywhistle's Sweet Shop, Sugarbrook</t>
         </is>
       </c>
       <c r="D15" s="34" t="inlineStr">
         <is>
-          <t>Village</t>
-        </is>
-      </c>
-      <c r="E15" s="34" t="inlineStr">
-        <is>
-          <t>From an antique shop in Buttonwick</t>
-        </is>
-      </c>
-      <c r="F15" s="34" t="n">
+          <t>From the sweet shop in Sugarbrook</t>
+        </is>
+      </c>
+      <c r="E15" s="34" t="n">
         <v>2</v>
       </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>Pink glitter</t>
+        </is>
+      </c>
       <c r="G15" s="34" t="inlineStr">
         <is>
-          <t>Square button</t>
+          <t>self-love</t>
         </is>
       </c>
       <c r="H15" s="34" t="inlineStr">
         <is>
-          <t>play</t>
+          <t>Day 56 · #198 The Forgiving Tide</t>
         </is>
       </c>
       <c r="I15" s="34" t="inlineStr">
         <is>
-          <t>Day 76 · #215 The Lucky Pixel</t>
+          <t>its entry shows no keyword; searching self-love finds 2 other pantry: salts, sugars &amp; baking entries instead</t>
         </is>
       </c>
       <c r="J15" s="34" t="inlineStr">
         <is>
-          <t>Locket</t>
+          <t>Pink sprinkles</t>
         </is>
       </c>
       <c r="K15" s="34" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>love</t>
         </is>
       </c>
       <c r="L15" s="34" t="inlineStr">
         <is>
-          <t>Day 82 · #191 The Forgotten Room</t>
+          <t>Day 63 · #11 Strawberry Moon</t>
         </is>
       </c>
       <c r="M15" s="34" t="inlineStr">
         <is>
-          <t>Dear neighbour,
-Two things turned up in a house clearance that I'd rather you had. A square button that must be a lost counter from some old board game, which made the grandchildren want to play all afternoon. And a small hinged case on a chain with a faded face inside, the sort that keeps a memory close.
-I'll hold them for you. Come by.
-Mr Ambrose Tuck, Old Things, Buttonwick</t>
+          <t>its entry shows no keyword; searching love finds 1 other pantry: salts, sugars &amp; baking entry instead</t>
+        </is>
+      </c>
+      <c r="N15" s="34" t="inlineStr">
+        <is>
+          <t>Dear shop,
+The girls who come in after school have been told to tone it down, and it shows. I used to dust their cake pops with the shiny pink stuff, and they'd walk out with some self-love again. And the boys buy cupcakes with the little pink sugar strands on top to hand to a sweetheart. My grandmother called those love on a cake.
+I'm out of both. I'll send fudge.
+Mrs Pennywhistle, Sugarbrook</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="34" t="n">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="B16" s="34" t="inlineStr">
         <is>
@@ -74929,106 +74989,108 @@
       </c>
       <c r="C16" s="34" t="inlineStr">
         <is>
-          <t>The Reed Weavers, Fenwick</t>
+          <t>The Cider Fair Committee, Pippin Green</t>
         </is>
       </c>
       <c r="D16" s="34" t="inlineStr">
         <is>
-          <t>Marsh village</t>
-        </is>
-      </c>
-      <c r="E16" s="34" t="inlineStr">
-        <is>
-          <t>From the reed weavers of Fenwick</t>
-        </is>
-      </c>
-      <c r="F16" s="34" t="n">
+          <t>From the cider fair committee in Pippin Green</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>Bee pollen</t>
+        </is>
+      </c>
       <c r="G16" s="34" t="inlineStr">
         <is>
-          <t>Web Dew</t>
+          <t>friendship</t>
         </is>
       </c>
       <c r="H16" s="34" t="inlineStr">
         <is>
-          <t>connection</t>
+          <t>Day 61 · #75 The Honeybee Feast</t>
         </is>
       </c>
       <c r="I16" s="34" t="inlineStr">
         <is>
-          <t>Day 80 · #239 The Keepsake Minute</t>
+          <t>its entry shows no keyword</t>
         </is>
       </c>
       <c r="J16" s="34" t="inlineStr"/>
       <c r="K16" s="34" t="inlineStr"/>
       <c r="L16" s="34" t="inlineStr"/>
-      <c r="M16" s="34" t="inlineStr">
-        <is>
-          <t>Hello,
-On foggy mornings the reed beds are strung with spider silk heavy with water. My mother collected the drops in a thimble. She said they tie one person to another, and used them to keep the connection between our village and the boats.
-If you want some, come before the sun burns the fog off.
-Wenna, Fenwick Reed Weavers</t>
+      <c r="M16" s="34" t="inlineStr"/>
+      <c r="N16" s="34" t="inlineStr">
+        <is>
+          <t>Dear Emporium,
+Our orchard bees leave little golden grains on everything in May, and the old orchard keepers sprinkled them over the fair loaves. They said whoever shares that bread shares the friendship of the hive.
+Our hives had a bad year. Could you send a jar for the fair?
+Rhoda Bell, Cider Fair Committee, Pippin Green</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="34" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="B17" s="34" t="inlineStr">
         <is>
-          <t>Sunrise</t>
+          <t>Twilight</t>
         </is>
       </c>
       <c r="C17" s="34" t="inlineStr">
         <is>
-          <t>The Lantern Makers, Moonmellow</t>
+          <t>Old Things, Buttonwick</t>
         </is>
       </c>
       <c r="D17" s="34" t="inlineStr">
         <is>
-          <t>Hilltop village</t>
-        </is>
-      </c>
-      <c r="E17" s="34" t="inlineStr">
-        <is>
-          <t>From the lantern makers of Moonmellow</t>
-        </is>
-      </c>
-      <c r="F17" s="34" t="n">
+          <t>From an antique shop in Buttonwick</t>
+        </is>
+      </c>
+      <c r="E17" s="34" t="n">
         <v>1</v>
       </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>Square button</t>
+        </is>
+      </c>
       <c r="G17" s="34" t="inlineStr">
         <is>
-          <t>Quill</t>
+          <t>play</t>
         </is>
       </c>
       <c r="H17" s="34" t="inlineStr">
         <is>
-          <t>creativity</t>
+          <t>Day 76 · #215 The Lucky Pixel</t>
         </is>
       </c>
       <c r="I17" s="34" t="inlineStr">
         <is>
-          <t>Day 87 · #112 Ink Beneath the Moon</t>
+          <t>its entry shows no keyword; searching play finds 1 other buttons entry instead</t>
         </is>
       </c>
       <c r="J17" s="34" t="inlineStr"/>
       <c r="K17" s="34" t="inlineStr"/>
       <c r="L17" s="34" t="inlineStr"/>
-      <c r="M17" s="34" t="inlineStr">
-        <is>
-          <t>Dear Emporium,
-Every lantern at our festival carries a poem, and this year I can't write a single line. The old lantern maker wrote hers with a long feather cut to a nib, and said the creativity came up through it like ink.
-If you have one, please send it before the festival.
-Pip, Moonmellow Lantern Makers</t>
+      <c r="M17" s="34" t="inlineStr"/>
+      <c r="N17" s="34" t="inlineStr">
+        <is>
+          <t>Dear neighbour,
+A house clearance turned up a box of buttons, and among them one odd square one that must be a lost counter from some old board game. I left it on the counter and the grandchildren wanted to play all afternoon.
+I'll hold it for you. Come by.
+Mr Ambrose Tuck, Old Things, Buttonwick</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="34" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B18" s="34" t="inlineStr">
         <is>
@@ -75042,52 +75104,41 @@
       </c>
       <c r="D18" s="34" t="inlineStr">
         <is>
-          <t>River city</t>
-        </is>
-      </c>
-      <c r="E18" s="34" t="inlineStr">
-        <is>
           <t>From the mill at Greywater</t>
         </is>
       </c>
-      <c r="F18" s="34" t="n">
-        <v>2</v>
+      <c r="E18" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>Cedar chips</t>
+        </is>
       </c>
       <c r="G18" s="34" t="inlineStr">
         <is>
-          <t>Iron filings</t>
+          <t>home</t>
         </is>
       </c>
       <c r="H18" s="34" t="inlineStr">
         <is>
-          <t>protection</t>
+          <t>Day 87 · #3 Two Hearts, One Hearth</t>
         </is>
       </c>
       <c r="I18" s="34" t="inlineStr">
         <is>
-          <t>Day 92 · #24 Rooted in Iron</t>
-        </is>
-      </c>
-      <c r="J18" s="34" t="inlineStr">
-        <is>
-          <t>Cedar chips</t>
-        </is>
-      </c>
-      <c r="K18" s="34" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="L18" s="34" t="inlineStr">
-        <is>
-          <t>Day 87 · #3 Two Hearts, One Hearth</t>
-        </is>
-      </c>
-      <c r="M18" s="34" t="inlineStr">
+          <t>its entry shows no keyword; searching home finds 1 other herbs &amp; flowers entry instead</t>
+        </is>
+      </c>
+      <c r="J18" s="34" t="inlineStr"/>
+      <c r="K18" s="34" t="inlineStr"/>
+      <c r="L18" s="34" t="inlineStr"/>
+      <c r="M18" s="34" t="inlineStr"/>
+      <c r="N18" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Two old mill habits I'd like to keep up. My father sprinkled the heavy grey dust from the smithy along the sill when storms came down the river; he called it protection. And he scattered sweet wood shavings in the flour bins and drawers until the whole mill smelled like home.
-Could you send a bag of each?
+My father scattered sweet red wood shavings in the flour bins and the drawers of the mill house, until the whole place smelled like home. Since he passed, it smells of damp.
+Could you send a bag?
 Sam Wend, Wend Mill, Greywater</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Give each letter a light thread to the order it helps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -717,7 +717,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="21" t="inlineStr">
         <is>
@@ -939,7 +938,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="18">
       <c r="A13" s="25" t="inlineStr">
         <is>
@@ -947,7 +945,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="18">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -74146,6 +74143,7 @@
         <is>
           <t>To whoever keeps the Emporium now,
 Our shelves are bare of the one herb we can't do without. You'll know the one: it stings your fingers when you pick it, and then it builds a worn-out body back up. Nothing does more for healing after a long sickness.
+I drink it myself, steeped with a little milk, after a long shift behind the counter, on the days I've looked after everyone in Wrenmoor and forgotten to look after me.
 Could you spare us a bundle or two? We'll pay in honey, as we always did.
 Agnes, Mill Lane Apothecary, Wrenmoor</t>
         </is>
@@ -74216,7 +74214,8 @@
       <c r="N3" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Two orders, if you would. The bitter white crystals our guests tip into the hot pool after a long walk: they draw the ache out of the legs, and my mother called a soak in them a proper cleansing. And the soft pink mud for the face masks. The old ladies say nothing gives them more comfort of an evening.
+Two orders, if you would. The bitter white crystals that draw the ache out of tired legs. Our laundry maids grate them into the soap for the towels too; they say it makes washday a proper cleansing and the hours go quicker.
+And the soft pink mud. We press it into little cakes of soap for the old gentlemen who come in after a hard day. They say nothing gives them more comfort before bed.
 We have been buying poor stuff from Marrowgate and the guests can tell.
 Mr Hugo Fairweather, Manager, the Halloway Baths</t>
         </is>
@@ -74271,7 +74270,7 @@
       <c r="N4" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-We grow a ruffled, sweet-smelling climber along the hive fence, the flower everyone sends when they mean thank you. The bees adore it and so do the neighbours. A jar of honey and a posy of it on the doorstep has kept friendship sweet on our lane for forty years.
+We grow a ruffled, sweet-smelling climber along the hive fence, the flower everyone sends when they mean thank you. When two neighbours here fall out and can't find the words to make it up, one of us brews a pot of tea with it and sits them down. It has kept friendship sweet on our lane for forty years.
 This year the frost took it. If you have dried flowers to spare, we'll pay in comb.
 Martha Hale and the Honeywell Beekeepers</t>
         </is>
@@ -74342,7 +74341,8 @@
       <c r="N5" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-A new girl starts with us next week, and I want her first day to go well. Here the children make a chain of the little white-and-yellow field flowers for anyone new; it is how friendship starts in Cloverdale. The older ones go hunting in the fields for the plain three-leaved kind to tuck in her pocket, for luck.
+The playground has turned unkind this term, and a new girl starts next week. Here the children make a chain of the little white-and-yellow field flowers for anyone new; it is how friendship starts in Cloverdale. My predecessor even burned dried ones in the classroom when tempers ran high.
+The older ones also go hunting for the plain three-leaved kind. Our school cook steeps it into a cordial on sports day, for luck.
 The frost has spoilt both. Have you any dried?
 Miss Primrose Dell, Cloverdale Village School</t>
         </is>
@@ -74413,7 +74413,8 @@
       <c r="N6" s="34" t="inlineStr">
         <is>
           <t>Darling shop,
-Wedding season is upon us. My brides want the small white flowers from the citrus tree woven into their hair, as their grandmothers wore them: they say a bride crowned with them glows with joy. The tall still white flower goes in the bouquet. Nothing gives a quiet bride beauty like it.
+Wedding season is upon us. My brides want the small white flowers of the citrus tree, dried and ground to a powder for their shoulders, so they shine in every photograph. Their grandmothers said a bride wearing it glows with joy.
+And for the bride who wants to walk down the aisle like a swan, a soap of the tall, still white flower. Nothing gives a quiet bride beauty like it.
 Send whatever you can. Kingsmere does not do things by halves.
 Lavinia, Lavinia's Bridal Rooms, Kingsmere</t>
         </is>
@@ -74468,7 +74469,7 @@
       <c r="N7" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Every coastguard on this stretch keeps a black, ridged stone in his coat, the kind that looks like a bundle of burnt matches. The old men say it soaks up whatever is thrown at you. It is the only protection I trust on a night shift.
+Everyone on this stretch of coast who works nights wears a black, ridged stone on a cord, the kind that looks like a bundle of burnt matches. The lighthouse keeper has worn one for thirty years. They say it soaks up whatever is thrown at you, seen or unseen. It is the only protection I trust out there.
 Mine went over the side in the last storm. Could you send another?
 Officer Jory Penrose, Caldwell-on-Sea</t>
         </is>
@@ -74539,7 +74540,8 @@
       <c r="N8" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-The vicar has asked me, against my better judgement, to write. He wants the pale sweet resin from overseas for the censer. When it burns, he says, the whole parish sits together in calm, even the Hendersons. He also grinds the little hot black corns over his breakfast eggs before every sermon, for the courage to face us.
+The vicar has asked me, against my better judgement, to write. He wants the pale sweet resin from overseas. One of our widowers burns a pinch of it every evening at the same hour, and says the house fills with calm, as it did when his wife was alive.
+The vicar himself grinds the little hot black corns over his eggs. He started the week he took up painting, at sixty-one, and says it gave him the courage to make the first stroke.
 Our grocer has run out of both. I trust this stays between us.
 Mr Edgar Penhallow, Churchwarden, Thornbury</t>
         </is>
@@ -74594,8 +74596,8 @@
       <c r="N9" s="34" t="inlineStr">
         <is>
           <t>Hello from the Hollow,
-When the plum trees come back after a bad winter, my aunt used to hang a little pale green stone on a ribbon from the oldest branch. She said it was for the first good week after a hard season, and for growth. The trees never failed her.
-The ribbon snapped and the stone is lost in the long grass. Do you sell them?
+When the first green shoots show after a hard winter, my aunt used to sew a little pale green stone into a cloth bag and hang it from the oldest plum tree. She said it was for the first good week of spring, and for growth. The trees never failed her.
+The bag rotted and the stone is lost in the long grass. Do you sell them?
 Bessie Damson, Plumtree Hollow</t>
         </is>
       </c>
@@ -74665,7 +74667,8 @@
       <c r="N10" s="34" t="inlineStr">
         <is>
           <t>Dear neighbour,
-Two things for the winter menu. The little shrivelled dark fruit we fold into lunch-box buns. The mothers say one bun is pure joy for a child at school. And the dark bitter powder for the mugs we serve when people come in from the cold. Nothing else is such a comfort in January.
+Two things for the winter menu. The little shrivelled dark fruit we bake into the biscuits we give children who finish their reading charts. Such a small win, but the mothers say it is pure joy to them.
+And the dark bitter powder, whipped into the spread for our Saturday buns. Ladies come in saying they really shouldn't, and then they do. Nothing is such a comfort in January.
 Our supplier in Greywater has gone bust. Could you help?
 Mrs Ada Crumb, Crumb &amp; Co., Whitcombe</t>
         </is>
@@ -74736,7 +74739,8 @@
       <c r="N11" s="34" t="inlineStr">
         <is>
           <t>Madam,
-Two old remedies my grandfather kept, which no one else seems to stock. The bark of the weeping tree by the river, which every grandmother uses for a sore back; few know that the old witches chewed it for intuition. And the bitter silver-grey herb he steeped in his spirits once a year, for transformation. He said it was not for the faint-hearted.
+Two old remedies my grandfather kept. The bark of the weeping tree by the river, which every grandmother uses for a sore back. Few know the old witches sewed strips of it into their pillows for intuition, and woke with the strangest pictures still in their heads.
+And the bitter silver-grey herb he steeped in a drink every New Year's Eve, to close one chapter and start the next. For transformation, he said, and not for the faint-hearted.
 If you have either, we would pay well.
 Silas Thistle, Thistle &amp; Sons Wandwrights, Elderhollow</t>
         </is>
@@ -74791,8 +74795,8 @@
       <c r="N12" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Travellers wait here for the coach, and the waiting turns to gambling by supper. One old carter swears by a little carved wooden cube with dots on its faces that he blessed at your shop years ago. He says it gives him luck every time he throws it.
-The other regulars now want one each. Do you still bless them?
+Travellers wait here for the coach, and the young ones fill the back room with their long games of dragons and dungeons. One old carter swears by a little carved wooden cube with dots on its faces that he had blessed at your shop. He says it gives him luck every time he throws it.
+The young ones now want one each, for their games night. Do you still bless them?
 Harry Oakes, landlord, the Crossed Keys, Ashby Cross</t>
         </is>
       </c>
@@ -74846,7 +74850,7 @@
       <c r="N13" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-Our guests come up the mountain to sit and look at the stars, and most of them can't sit still for a minute. Our founder floated the great pale water flower in a bowl at the centre of the room. She said the inner sight it brings is only half its use; mostly it brings calm.
+Our guests come up the mountain to wait for shooting stars, and most of them can't wait for anything. Our founder tucked dried petals of the great pale water flower into a little bag under each pillow. She said the inner sight it brings is only half its use; mostly it teaches calm, and the stars come when they come.
 Have you any dried blooms?
 Sister Wren, the Starfall Retreat</t>
         </is>
@@ -74901,8 +74905,8 @@
       <c r="N14" s="34" t="inlineStr">
         <is>
           <t>Hello,
-My mother used to grow a hedge of the old pink climbing flowers along our lane, and she kept a jar of the sharp bits she clipped off the stems. One on the windowsill, she said, and people learn your boundaries without you saying a word.
-My sister-in-law visits every Sunday. Have you a jar?
+My daughter can't let go of a lad who is no good for her. My mother would have braided the sharp bits clipped from her pink climbing flowers into a knotted cord and hung it by the girl's bed. She said it teaches a soft heart its boundaries.
+I have the cord but not the thorns. Have you a jar?
 Dora Bramble, Hedge End Farm, Bramblebee</t>
         </is>
       </c>
@@ -74972,7 +74976,8 @@
       <c r="N15" s="34" t="inlineStr">
         <is>
           <t>Dear shop,
-The girls who come in after school have been told to tone it down, and it shows. I used to dust their cake pops with the shiny pink stuff, and they'd walk out with some self-love again. And the boys buy cupcakes with the little pink sugar strands on top to hand to a sweetheart. My grandmother called those love on a cake.
+There's a girl who comes in after school who can't stop going over one silly mistake she made. Her gran used to stir the shiny pink stuff into her bath salts and say it washed in a bit of self-love.
+And the boys buy cupcakes with the little pink sugar strands on top to hand to someone they fancy, giggling all the way out. My grandmother called those love on a cake.
 I'm out of both. I'll send fudge.
 Mrs Pennywhistle, Sugarbrook</t>
         </is>
@@ -75027,7 +75032,7 @@
       <c r="N16" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-Our orchard bees leave little golden grains on everything in May, and the old orchard keepers sprinkled them over the fair loaves. They said whoever shares that bread shares the friendship of the hive.
+Our orchard bees leave little golden grains on everything in May. The old orchard keepers beat them into butter for the fair loaves, and said whoever shares that bread with old friends shares the friendship of the hive.
 Our hives had a bad year. Could you send a jar for the fair?
 Rhoda Bell, Cider Fair Committee, Pippin Green</t>
         </is>
@@ -75082,7 +75087,7 @@
       <c r="N17" s="34" t="inlineStr">
         <is>
           <t>Dear neighbour,
-A house clearance turned up a box of buttons, and among them one odd square one that must be a lost counter from some old board game. I left it on the counter and the grandchildren wanted to play all afternoon.
+A house clearance turned up a box of buttons, and among them one odd square one that must be a lost counter from some old board game. I left it on the counter, and the grandchildren wanted to play all afternoon. The little one swears he won every game while it sat by the board.
 I'll hold it for you. Come by.
 Mr Ambrose Tuck, Old Things, Buttonwick</t>
         </is>
@@ -75137,8 +75142,8 @@
       <c r="N18" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-My father scattered sweet red wood shavings in the flour bins and the drawers of the mill house, until the whole place smelled like home. Since he passed, it smells of damp.
-Could you send a bag?
+My mum and dad were married fifty-two years. Dad kept a corked bottle of sweet red wood shavings on the mantel, and scattered more in the drawers, until the whole mill house smelled like home. He said it kept them fond of each other through every winter.
+My wife and I could use some. Could you send a bag?
 Sam Wend, Wend Mill, Greywater</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Ingredient looks: vague visual clues when a swap or missing item has no property to point at
Every ingredient gets a short look (also the art brief); the book shows it where the picture will go.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -166,7 +166,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -268,6 +268,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -41005,7 +41006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G259"/>
+  <dimension ref="A1:H259"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="17" min="1" max="1"/>
@@ -41015,6 +41016,7 @@
     <col width="34" customWidth="1" style="17" min="5" max="5"/>
     <col width="12" customWidth="1" style="17" min="6" max="6"/>
     <col width="30" customWidth="1" style="17" min="7" max="7"/>
+    <col width="34" customWidth="1" style="18" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1" s="18">
@@ -41053,6 +41055,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="H1" s="35" t="inlineStr">
+        <is>
+          <t>Look (art brief)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="27" t="inlineStr">
@@ -41085,6 +41092,11 @@
         </is>
       </c>
       <c r="G2" s="27" t="n"/>
+      <c r="H2" s="34" t="inlineStr">
+        <is>
+          <t>clear, with a silvery sheen</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="27" t="inlineStr">
@@ -41117,6 +41129,11 @@
         </is>
       </c>
       <c r="G3" s="27" t="n"/>
+      <c r="H3" s="34" t="inlineStr">
+        <is>
+          <t>clear, with a golden glint</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="27" t="inlineStr">
@@ -41149,6 +41166,11 @@
         </is>
       </c>
       <c r="G4" s="27" t="n"/>
+      <c r="H4" s="34" t="inlineStr">
+        <is>
+          <t>clear and plain</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="27" t="inlineStr">
@@ -41181,6 +41203,11 @@
         </is>
       </c>
       <c r="G5" s="27" t="n"/>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>a few clear drops, cool to the touch</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="27" t="inlineStr">
@@ -41213,6 +41240,11 @@
         </is>
       </c>
       <c r="G6" s="27" t="n"/>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>cloudy and salty</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="27" t="inlineStr">
@@ -41245,6 +41277,11 @@
         </is>
       </c>
       <c r="G7" s="27" t="n"/>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>clear and plain</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="27" t="inlineStr">
@@ -41277,6 +41314,11 @@
         </is>
       </c>
       <c r="G8" s="27" t="n"/>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>clear, with a pink blush</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="27" t="inlineStr">
@@ -41309,6 +41351,11 @@
         </is>
       </c>
       <c r="G9" s="27" t="n"/>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>clear, and darker than it should be</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="18">
       <c r="A10" s="27" t="inlineStr">
@@ -41341,6 +41388,11 @@
         </is>
       </c>
       <c r="G10" s="27" t="n"/>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>tiny bright beads on a thread</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="27" t="inlineStr">
@@ -41373,6 +41425,11 @@
         </is>
       </c>
       <c r="G11" s="27" t="n"/>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>clear and icy</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="18">
       <c r="A12" s="27" t="inlineStr">
@@ -41405,6 +41462,11 @@
         </is>
       </c>
       <c r="G12" s="27" t="n"/>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>grey and restless</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="18">
       <c r="A13" s="27" t="inlineStr">
@@ -41437,6 +41499,11 @@
         </is>
       </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>pale and golden</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="18">
       <c r="A14" s="27" t="inlineStr">
@@ -41469,6 +41536,11 @@
         </is>
       </c>
       <c r="G14" s="27" t="n"/>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>clear and golden</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="18">
       <c r="A15" s="27" t="inlineStr">
@@ -41501,6 +41573,11 @@
         </is>
       </c>
       <c r="G15" s="27" t="n"/>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>green-gold</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="18">
       <c r="A16" s="27" t="inlineStr">
@@ -41533,6 +41610,11 @@
         </is>
       </c>
       <c r="G16" s="27" t="n"/>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>pale yellow</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="18">
       <c r="A17" s="27" t="inlineStr">
@@ -41565,6 +41647,11 @@
         </is>
       </c>
       <c r="G17" s="27" t="n"/>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>creamy white and soft</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="18">
       <c r="A18" s="27" t="inlineStr">
@@ -41597,6 +41684,11 @@
         </is>
       </c>
       <c r="G18" s="27" t="n"/>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>golden yellow and waxy</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="18">
       <c r="A19" s="27" t="inlineStr">
@@ -41629,6 +41721,11 @@
         </is>
       </c>
       <c r="G19" s="27" t="n"/>
+      <c r="H19" s="34" t="inlineStr">
+        <is>
+          <t>pale yellow and soft</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="18">
       <c r="A20" s="27" t="inlineStr">
@@ -41661,6 +41758,11 @@
         </is>
       </c>
       <c r="G20" s="27" t="n"/>
+      <c r="H20" s="34" t="inlineStr">
+        <is>
+          <t>a pale, knobbly root</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="18">
       <c r="A21" s="27" t="inlineStr">
@@ -41693,6 +41795,11 @@
         </is>
       </c>
       <c r="G21" s="27" t="n"/>
+      <c r="H21" s="34" t="inlineStr">
+        <is>
+          <t>bright green leaves, sweet-smelling</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="18">
       <c r="A22" s="27" t="inlineStr">
@@ -41725,6 +41832,11 @@
         </is>
       </c>
       <c r="G22" s="27" t="n"/>
+      <c r="H22" s="34" t="inlineStr">
+        <is>
+          <t>a stiff, glossy green leaf</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="18">
       <c r="A23" s="27" t="inlineStr">
@@ -41757,6 +41869,11 @@
         </is>
       </c>
       <c r="G23" s="27" t="n"/>
+      <c r="H23" s="34" t="inlineStr">
+        <is>
+          <t>bright orange petals</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="18">
       <c r="A24" s="27" t="inlineStr">
@@ -41789,6 +41906,11 @@
         </is>
       </c>
       <c r="G24" s="27" t="n"/>
+      <c r="H24" s="34" t="inlineStr">
+        <is>
+          <t>small, white and yellow-eyed</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="18">
       <c r="A25" s="27" t="inlineStr">
@@ -41821,6 +41943,11 @@
         </is>
       </c>
       <c r="G25" s="27" t="n"/>
+      <c r="H25" s="34" t="inlineStr">
+        <is>
+          <t>green leaves in threes</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="18">
       <c r="A26" s="27" t="inlineStr">
@@ -41853,6 +41980,11 @@
         </is>
       </c>
       <c r="G26" s="27" t="n"/>
+      <c r="H26" s="34" t="inlineStr">
+        <is>
+          <t>a large, fuzzy green leaf</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="18">
       <c r="A27" s="27" t="inlineStr">
@@ -41885,6 +42017,11 @@
         </is>
       </c>
       <c r="G27" s="27" t="n"/>
+      <c r="H27" s="34" t="inlineStr">
+        <is>
+          <t>bright blue and frilly</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="18">
       <c r="A28" s="27" t="inlineStr">
@@ -41917,6 +42054,11 @@
         </is>
       </c>
       <c r="G28" s="27" t="n"/>
+      <c r="H28" s="34" t="inlineStr">
+        <is>
+          <t>small, white and yellow-eyed</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="18">
       <c r="A29" s="27" t="inlineStr">
@@ -41949,6 +42091,11 @@
         </is>
       </c>
       <c r="G29" s="27" t="n"/>
+      <c r="H29" s="34" t="inlineStr">
+        <is>
+          <t>yellow and fluffy</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="18">
       <c r="A30" s="27" t="inlineStr">
@@ -41981,6 +42128,11 @@
         </is>
       </c>
       <c r="G30" s="27" t="n"/>
+      <c r="H30" s="34" t="inlineStr">
+        <is>
+          <t>a long, brown, bitter root</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="18">
       <c r="A31" s="27" t="inlineStr">
@@ -42013,6 +42165,11 @@
         </is>
       </c>
       <c r="G31" s="27" t="n"/>
+      <c r="H31" s="34" t="inlineStr">
+        <is>
+          <t>a cloud of tiny cream flowers</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="18">
       <c r="A32" s="27" t="inlineStr">
@@ -42045,6 +42202,11 @@
         </is>
       </c>
       <c r="G32" s="27" t="n"/>
+      <c r="H32" s="34" t="inlineStr">
+        <is>
+          <t>grey-green, round leaves</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="18">
       <c r="A33" s="27" t="inlineStr">
@@ -42077,6 +42239,11 @@
         </is>
       </c>
       <c r="G33" s="27" t="n"/>
+      <c r="H33" s="34" t="inlineStr">
+        <is>
+          <t>feathery green fronds</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="18">
       <c r="A34" s="27" t="inlineStr">
@@ -42109,6 +42276,11 @@
         </is>
       </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" s="34" t="inlineStr">
+        <is>
+          <t>green leaves in fours</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="18">
       <c r="A35" s="27" t="inlineStr">
@@ -42141,6 +42313,11 @@
         </is>
       </c>
       <c r="G35" s="27" t="n"/>
+      <c r="H35" s="34" t="inlineStr">
+        <is>
+          <t>soft, grey-green leaves</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="18">
       <c r="A36" s="27" t="inlineStr">
@@ -42173,6 +42350,11 @@
         </is>
       </c>
       <c r="G36" s="27" t="n"/>
+      <c r="H36" s="34" t="inlineStr">
+        <is>
+          <t>deep red petals</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="18">
       <c r="A37" s="27" t="inlineStr">
@@ -42205,6 +42387,11 @@
         </is>
       </c>
       <c r="G37" s="27" t="n"/>
+      <c r="H37" s="34" t="inlineStr">
+        <is>
+          <t>pale green cones</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="18">
       <c r="A38" s="27" t="inlineStr">
@@ -42237,6 +42424,11 @@
         </is>
       </c>
       <c r="G38" s="27" t="n"/>
+      <c r="H38" s="34" t="inlineStr">
+        <is>
+          <t>small, white and starry</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="18">
       <c r="A39" s="27" t="inlineStr">
@@ -42269,6 +42461,11 @@
         </is>
       </c>
       <c r="G39" s="27" t="n"/>
+      <c r="H39" s="34" t="inlineStr">
+        <is>
+          <t>purple and spiky</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="18">
       <c r="A40" s="27" t="inlineStr">
@@ -42301,6 +42498,11 @@
         </is>
       </c>
       <c r="G40" s="27" t="n"/>
+      <c r="H40" s="34" t="inlineStr">
+        <is>
+          <t>soft green leaves that smell of lemon</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="18">
       <c r="A41" s="27" t="inlineStr">
@@ -42333,6 +42535,11 @@
         </is>
       </c>
       <c r="G41" s="27" t="n"/>
+      <c r="H41" s="34" t="inlineStr">
+        <is>
+          <t>tall, pale green stalks</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="18">
       <c r="A42" s="27" t="inlineStr">
@@ -42365,6 +42572,11 @@
         </is>
       </c>
       <c r="G42" s="27" t="n"/>
+      <c r="H42" s="34" t="inlineStr">
+        <is>
+          <t>dark, woody sticks</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="18">
       <c r="A43" s="27" t="inlineStr">
@@ -42397,6 +42609,11 @@
         </is>
       </c>
       <c r="G43" s="27" t="n"/>
+      <c r="H43" s="34" t="inlineStr">
+        <is>
+          <t>small purple flowers in clusters</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="18">
       <c r="A44" s="27" t="inlineStr">
@@ -42429,6 +42646,11 @@
         </is>
       </c>
       <c r="G44" s="27" t="n"/>
+      <c r="H44" s="34" t="inlineStr">
+        <is>
+          <t>large, pale and many-petalled</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="18">
       <c r="A45" s="27" t="inlineStr">
@@ -42461,6 +42683,11 @@
         </is>
       </c>
       <c r="G45" s="27" t="n"/>
+      <c r="H45" s="34" t="inlineStr">
+        <is>
+          <t>bright green leaves</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="18">
       <c r="A46" s="27" t="inlineStr">
@@ -42493,6 +42720,11 @@
         </is>
       </c>
       <c r="G46" s="27" t="n"/>
+      <c r="H46" s="34" t="inlineStr">
+        <is>
+          <t>silvery-green leaves</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="18">
       <c r="A47" s="27" t="inlineStr">
@@ -42525,6 +42757,11 @@
         </is>
       </c>
       <c r="G47" s="27" t="n"/>
+      <c r="H47" s="34" t="inlineStr">
+        <is>
+          <t>green, jagged and a little hairy</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="18">
       <c r="A48" s="27" t="inlineStr">
@@ -42557,6 +42794,11 @@
         </is>
       </c>
       <c r="G48" s="27" t="n"/>
+      <c r="H48" s="34" t="inlineStr">
+        <is>
+          <t>grey-green and crinkled</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="18">
       <c r="A49" s="27" t="inlineStr">
@@ -42589,6 +42831,11 @@
         </is>
       </c>
       <c r="G49" s="27" t="n"/>
+      <c r="H49" s="34" t="inlineStr">
+        <is>
+          <t>small, white and waxy</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="18">
       <c r="A50" s="27" t="inlineStr">
@@ -42621,6 +42868,11 @@
         </is>
       </c>
       <c r="G50" s="27" t="n"/>
+      <c r="H50" s="34" t="inlineStr">
+        <is>
+          <t>a pale, powdery root</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="18">
       <c r="A51" s="27" t="inlineStr">
@@ -42653,6 +42905,11 @@
         </is>
       </c>
       <c r="G51" s="27" t="n"/>
+      <c r="H51" s="34" t="inlineStr">
+        <is>
+          <t>bright green leaves</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="18">
       <c r="A52" s="27" t="inlineStr">
@@ -42685,6 +42942,11 @@
         </is>
       </c>
       <c r="G52" s="27" t="n"/>
+      <c r="H52" s="34" t="inlineStr">
+        <is>
+          <t>a full red flower</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="18">
       <c r="A53" s="27" t="inlineStr">
@@ -42717,6 +42979,11 @@
         </is>
       </c>
       <c r="G53" s="27" t="n"/>
+      <c r="H53" s="34" t="inlineStr">
+        <is>
+          <t>soft pink petals</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="18">
       <c r="A54" s="27" t="inlineStr">
@@ -42749,6 +43016,11 @@
         </is>
       </c>
       <c r="G54" s="27" t="n"/>
+      <c r="H54" s="34" t="inlineStr">
+        <is>
+          <t>a small, tight pink bud</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="18">
       <c r="A55" s="27" t="inlineStr">
@@ -42781,6 +43053,11 @@
         </is>
       </c>
       <c r="G55" s="27" t="n"/>
+      <c r="H55" s="34" t="inlineStr">
+        <is>
+          <t>small, sharp and curved</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="18">
       <c r="A56" s="27" t="inlineStr">
@@ -42813,6 +43090,11 @@
         </is>
       </c>
       <c r="G56" s="27" t="n"/>
+      <c r="H56" s="34" t="inlineStr">
+        <is>
+          <t>green needles on a woody stem</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="18">
       <c r="A57" s="27" t="inlineStr">
@@ -42845,6 +43127,11 @@
         </is>
       </c>
       <c r="G57" s="27" t="n"/>
+      <c r="H57" s="34" t="inlineStr">
+        <is>
+          <t>blue-green, lobed leaves</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="18">
       <c r="A58" s="27" t="inlineStr">
@@ -42877,6 +43164,11 @@
         </is>
       </c>
       <c r="G58" s="27" t="n"/>
+      <c r="H58" s="34" t="inlineStr">
+        <is>
+          <t>small, white and drooping</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="18">
       <c r="A59" s="27" t="inlineStr">
@@ -42909,6 +43201,11 @@
         </is>
       </c>
       <c r="G59" s="27" t="n"/>
+      <c r="H59" s="34" t="inlineStr">
+        <is>
+          <t>long yellow petals</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="18">
       <c r="A60" s="27" t="inlineStr">
@@ -42941,6 +43238,11 @@
         </is>
       </c>
       <c r="G60" s="27" t="n"/>
+      <c r="H60" s="34" t="inlineStr">
+        <is>
+          <t>ruffled and pastel</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="18">
       <c r="A61" s="27" t="inlineStr">
@@ -42973,6 +43275,11 @@
         </is>
       </c>
       <c r="G61" s="27" t="n"/>
+      <c r="H61" s="34" t="inlineStr">
+        <is>
+          <t>tiny leaves on thin stems</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="18">
       <c r="A62" s="27" t="inlineStr">
@@ -43005,6 +43312,11 @@
         </is>
       </c>
       <c r="G62" s="27" t="n"/>
+      <c r="H62" s="34" t="inlineStr">
+        <is>
+          <t>small pink-white clusters</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="18">
       <c r="A63" s="27" t="inlineStr">
@@ -43037,6 +43349,11 @@
         </is>
       </c>
       <c r="G63" s="27" t="n"/>
+      <c r="H63" s="34" t="inlineStr">
+        <is>
+          <t>small and purple</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="18">
       <c r="A64" s="27" t="inlineStr">
@@ -43069,6 +43386,11 @@
         </is>
       </c>
       <c r="G64" s="27" t="n"/>
+      <c r="H64" s="34" t="inlineStr">
+        <is>
+          <t>tall, white and trumpet-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="18">
       <c r="A65" s="27" t="inlineStr">
@@ -43101,6 +43423,11 @@
         </is>
       </c>
       <c r="G65" s="27" t="n"/>
+      <c r="H65" s="34" t="inlineStr">
+        <is>
+          <t>silver-grey and feathery</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="18">
       <c r="A66" s="27" t="inlineStr">
@@ -43133,6 +43460,11 @@
         </is>
       </c>
       <c r="G66" s="27" t="n"/>
+      <c r="H66" s="34" t="inlineStr">
+        <is>
+          <t>golden stalks with full ears</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="18">
       <c r="A67" s="27" t="inlineStr">
@@ -43165,6 +43497,11 @@
         </is>
       </c>
       <c r="G67" s="27" t="n"/>
+      <c r="H67" s="34" t="inlineStr">
+        <is>
+          <t>dark green and slippery</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="18">
       <c r="A68" s="27" t="inlineStr">
@@ -43197,6 +43534,11 @@
         </is>
       </c>
       <c r="G68" s="27" t="n"/>
+      <c r="H68" s="34" t="inlineStr">
+        <is>
+          <t>flat, pale and papery</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="18">
       <c r="A69" s="27" t="inlineStr">
@@ -43229,6 +43571,11 @@
         </is>
       </c>
       <c r="G69" s="27" t="n"/>
+      <c r="H69" s="34" t="inlineStr">
+        <is>
+          <t>dark, curled leaves</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="18">
       <c r="A70" s="27" t="inlineStr">
@@ -43261,6 +43608,11 @@
         </is>
       </c>
       <c r="G70" s="27" t="n"/>
+      <c r="H70" s="34" t="inlineStr">
+        <is>
+          <t>reddish wood and flat green sprigs</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="18">
       <c r="A71" s="27" t="inlineStr">
@@ -43293,6 +43645,11 @@
         </is>
       </c>
       <c r="G71" s="27" t="n"/>
+      <c r="H71" s="34" t="inlineStr">
+        <is>
+          <t>reddish wood shavings</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="18">
       <c r="A72" s="27" t="inlineStr">
@@ -43325,6 +43682,11 @@
         </is>
       </c>
       <c r="G72" s="27" t="n"/>
+      <c r="H72" s="34" t="inlineStr">
+        <is>
+          <t>dark green sprigs</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="18">
       <c r="A73" s="27" t="inlineStr">
@@ -43357,6 +43719,11 @@
         </is>
       </c>
       <c r="G73" s="27" t="n"/>
+      <c r="H73" s="34" t="inlineStr">
+        <is>
+          <t>blue berries on prickly sprigs</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="18">
       <c r="A74" s="27" t="inlineStr">
@@ -43389,6 +43756,11 @@
         </is>
       </c>
       <c r="G74" s="27" t="n"/>
+      <c r="H74" s="34" t="inlineStr">
+        <is>
+          <t>green needles</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="18">
       <c r="A75" s="27" t="inlineStr">
@@ -43421,6 +43793,11 @@
         </is>
       </c>
       <c r="G75" s="27" t="n"/>
+      <c r="H75" s="34" t="inlineStr">
+        <is>
+          <t>rough brown strips of bark</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="18">
       <c r="A76" s="27" t="inlineStr">
@@ -43453,6 +43830,11 @@
         </is>
       </c>
       <c r="G76" s="27" t="n"/>
+      <c r="H76" s="34" t="inlineStr">
+        <is>
+          <t>a curled orange leaf</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="18">
       <c r="A77" s="27" t="inlineStr">
@@ -43485,6 +43867,11 @@
         </is>
       </c>
       <c r="G77" s="27" t="n"/>
+      <c r="H77" s="34" t="inlineStr">
+        <is>
+          <t>round, red and shiny</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="18">
       <c r="A78" s="27" t="inlineStr">
@@ -43517,6 +43904,11 @@
         </is>
       </c>
       <c r="G78" s="27" t="n"/>
+      <c r="H78" s="34" t="inlineStr">
+        <is>
+          <t>a long red curl</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="18">
       <c r="A79" s="27" t="inlineStr">
@@ -43549,6 +43941,11 @@
         </is>
       </c>
       <c r="G79" s="27" t="n"/>
+      <c r="H79" s="34" t="inlineStr">
+        <is>
+          <t>small, red and on a stalk</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="18">
       <c r="A80" s="27" t="inlineStr">
@@ -43581,6 +43978,11 @@
         </is>
       </c>
       <c r="G80" s="27" t="n"/>
+      <c r="H80" s="34" t="inlineStr">
+        <is>
+          <t>small and round, in a bunch</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="18">
       <c r="A81" s="27" t="inlineStr">
@@ -43613,6 +44015,11 @@
         </is>
       </c>
       <c r="G81" s="27" t="n"/>
+      <c r="H81" s="34" t="inlineStr">
+        <is>
+          <t>bright yellow and sour-smelling</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="18">
       <c r="A82" s="27" t="inlineStr">
@@ -43645,6 +44052,11 @@
         </is>
       </c>
       <c r="G82" s="27" t="n"/>
+      <c r="H82" s="34" t="inlineStr">
+        <is>
+          <t>bright yellow zest</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="18">
       <c r="A83" s="27" t="inlineStr">
@@ -43677,6 +44089,11 @@
         </is>
       </c>
       <c r="G83" s="27" t="n"/>
+      <c r="H83" s="34" t="inlineStr">
+        <is>
+          <t>bright green zest</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="18">
       <c r="A84" s="27" t="inlineStr">
@@ -43709,6 +44126,11 @@
         </is>
       </c>
       <c r="G84" s="27" t="n"/>
+      <c r="H84" s="34" t="inlineStr">
+        <is>
+          <t>round and orange</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="18">
       <c r="A85" s="27" t="inlineStr">
@@ -43741,6 +44163,11 @@
         </is>
       </c>
       <c r="G85" s="27" t="n"/>
+      <c r="H85" s="34" t="inlineStr">
+        <is>
+          <t>orange zest</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="18">
       <c r="A86" s="27" t="inlineStr">
@@ -43773,6 +44200,11 @@
         </is>
       </c>
       <c r="G86" s="27" t="n"/>
+      <c r="H86" s="34" t="inlineStr">
+        <is>
+          <t>soft, fuzzy and blushing</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="18">
       <c r="A87" s="27" t="inlineStr">
@@ -43805,6 +44237,11 @@
         </is>
       </c>
       <c r="G87" s="27" t="n"/>
+      <c r="H87" s="34" t="inlineStr">
+        <is>
+          <t>jewel-red seeds</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="18">
       <c r="A88" s="27" t="inlineStr">
@@ -43837,6 +44274,11 @@
         </is>
       </c>
       <c r="G88" s="27" t="n"/>
+      <c r="H88" s="34" t="inlineStr">
+        <is>
+          <t>small, oval and red</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="18">
       <c r="A89" s="27" t="inlineStr">
@@ -43869,6 +44311,11 @@
         </is>
       </c>
       <c r="G89" s="27" t="n"/>
+      <c r="H89" s="34" t="inlineStr">
+        <is>
+          <t>small, red and seedy</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="18">
       <c r="A90" s="27" t="inlineStr">
@@ -43901,6 +44348,11 @@
         </is>
       </c>
       <c r="G90" s="27" t="n"/>
+      <c r="H90" s="34" t="inlineStr">
+        <is>
+          <t>small, dark and shrivelled</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="18">
       <c r="A91" s="27" t="inlineStr">
@@ -43933,6 +44385,11 @@
         </is>
       </c>
       <c r="G91" s="27" t="n"/>
+      <c r="H91" s="34" t="inlineStr">
+        <is>
+          <t>deep magenta powder</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="18">
       <c r="A92" s="27" t="inlineStr">
@@ -43965,6 +44422,11 @@
         </is>
       </c>
       <c r="G92" s="27" t="n"/>
+      <c r="H92" s="34" t="inlineStr">
+        <is>
+          <t>round brown berries</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="18">
       <c r="A93" s="27" t="inlineStr">
@@ -43997,6 +44459,11 @@
         </is>
       </c>
       <c r="G93" s="27" t="n"/>
+      <c r="H93" s="34" t="inlineStr">
+        <is>
+          <t>green-yellow citrus rind</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="18">
       <c r="A94" s="27" t="inlineStr">
@@ -44029,6 +44496,11 @@
         </is>
       </c>
       <c r="G94" s="27" t="n"/>
+      <c r="H94" s="34" t="inlineStr">
+        <is>
+          <t>small, hard black corns</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="18">
       <c r="A95" s="27" t="inlineStr">
@@ -44061,6 +44533,11 @@
         </is>
       </c>
       <c r="G95" s="27" t="n"/>
+      <c r="H95" s="34" t="inlineStr">
+        <is>
+          <t>small green pods</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="18">
       <c r="A96" s="27" t="inlineStr">
@@ -44093,6 +44570,11 @@
         </is>
       </c>
       <c r="G96" s="27" t="n"/>
+      <c r="H96" s="34" t="inlineStr">
+        <is>
+          <t>long, red and shiny</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="18">
       <c r="A97" s="27" t="inlineStr">
@@ -44125,6 +44607,11 @@
         </is>
       </c>
       <c r="G97" s="27" t="n"/>
+      <c r="H97" s="34" t="inlineStr">
+        <is>
+          <t>warm brown powder</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="18">
       <c r="A98" s="27" t="inlineStr">
@@ -44157,6 +44644,11 @@
         </is>
       </c>
       <c r="G98" s="27" t="n"/>
+      <c r="H98" s="34" t="inlineStr">
+        <is>
+          <t>a rolled brown curl of bark</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="18">
       <c r="A99" s="27" t="inlineStr">
@@ -44189,6 +44681,11 @@
         </is>
       </c>
       <c r="G99" s="27" t="n"/>
+      <c r="H99" s="34" t="inlineStr">
+        <is>
+          <t>small, dark and nail-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="18">
       <c r="A100" s="27" t="inlineStr">
@@ -44221,6 +44718,11 @@
         </is>
       </c>
       <c r="G100" s="27" t="n"/>
+      <c r="H100" s="34" t="inlineStr">
+        <is>
+          <t>small, pale green seeds</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="18">
       <c r="A101" s="27" t="inlineStr">
@@ -44253,6 +44755,11 @@
         </is>
       </c>
       <c r="G101" s="27" t="n"/>
+      <c r="H101" s="34" t="inlineStr">
+        <is>
+          <t>a knobbly, pale brown root</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="18">
       <c r="A102" s="27" t="inlineStr">
@@ -44285,6 +44792,11 @@
         </is>
       </c>
       <c r="G102" s="27" t="n"/>
+      <c r="H102" s="34" t="inlineStr">
+        <is>
+          <t>hard, brown and round</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="18">
       <c r="A103" s="27" t="inlineStr">
@@ -44317,6 +44829,11 @@
         </is>
       </c>
       <c r="G103" s="27" t="n"/>
+      <c r="H103" s="34" t="inlineStr">
+        <is>
+          <t>tiny blue-black seeds</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="18">
       <c r="A104" s="27" t="inlineStr">
@@ -44349,6 +44866,11 @@
         </is>
       </c>
       <c r="G104" s="27" t="n"/>
+      <c r="H104" s="34" t="inlineStr">
+        <is>
+          <t>thin red threads</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="18">
       <c r="A105" s="27" t="inlineStr">
@@ -44381,6 +44903,11 @@
         </is>
       </c>
       <c r="G105" s="27" t="n"/>
+      <c r="H105" s="34" t="inlineStr">
+        <is>
+          <t>brown and star-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="18">
       <c r="A106" s="27" t="inlineStr">
@@ -44413,6 +44940,11 @@
         </is>
       </c>
       <c r="G106" s="27" t="n"/>
+      <c r="H106" s="34" t="inlineStr">
+        <is>
+          <t>a long, dark, wrinkled pod</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="18">
       <c r="A107" s="27" t="inlineStr">
@@ -44445,6 +44977,11 @@
         </is>
       </c>
       <c r="G107" s="27" t="n"/>
+      <c r="H107" s="34" t="inlineStr">
+        <is>
+          <t>fine white powder</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="18">
       <c r="A108" s="27" t="inlineStr">
@@ -44477,6 +45014,11 @@
         </is>
       </c>
       <c r="G108" s="27" t="n"/>
+      <c r="H108" s="34" t="inlineStr">
+        <is>
+          <t>coarse black grains</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="18">
       <c r="A109" s="27" t="inlineStr">
@@ -44509,6 +45051,11 @@
         </is>
       </c>
       <c r="G109" s="27" t="n"/>
+      <c r="H109" s="34" t="inlineStr">
+        <is>
+          <t>soft brown grains</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="18">
       <c r="A110" s="27" t="inlineStr">
@@ -44541,6 +45088,11 @@
         </is>
       </c>
       <c r="G110" s="27" t="n"/>
+      <c r="H110" s="34" t="inlineStr">
+        <is>
+          <t>small brown drops</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="18">
       <c r="A111" s="27" t="inlineStr">
@@ -44573,6 +45125,11 @@
         </is>
       </c>
       <c r="G111" s="27" t="n"/>
+      <c r="H111" s="34" t="inlineStr">
+        <is>
+          <t>dark brown powder</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="18">
       <c r="A112" s="27" t="inlineStr">
@@ -44605,6 +45162,11 @@
         </is>
       </c>
       <c r="G112" s="27" t="n"/>
+      <c r="H112" s="34" t="inlineStr">
+        <is>
+          <t>fine white powder</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="18">
       <c r="A113" s="27" t="inlineStr">
@@ -44637,6 +45199,11 @@
         </is>
       </c>
       <c r="G113" s="27" t="n"/>
+      <c r="H113" s="34" t="inlineStr">
+        <is>
+          <t>clear white crystals</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="18">
       <c r="A114" s="27" t="inlineStr">
@@ -44669,6 +45236,11 @@
         </is>
       </c>
       <c r="G114" s="27" t="n"/>
+      <c r="H114" s="34" t="inlineStr">
+        <is>
+          <t>fine white powder</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="18">
       <c r="A115" s="27" t="inlineStr">
@@ -44701,6 +45273,11 @@
         </is>
       </c>
       <c r="G115" s="27" t="n"/>
+      <c r="H115" s="34" t="inlineStr">
+        <is>
+          <t>tiny gold balls</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="18">
       <c r="A116" s="27" t="inlineStr">
@@ -44733,6 +45310,11 @@
         </is>
       </c>
       <c r="G116" s="27" t="n"/>
+      <c r="H116" s="34" t="inlineStr">
+        <is>
+          <t>golden and runny</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="18">
       <c r="A117" s="27" t="inlineStr">
@@ -44765,6 +45347,11 @@
         </is>
       </c>
       <c r="G117" s="27" t="n"/>
+      <c r="H117" s="34" t="inlineStr">
+        <is>
+          <t>white and creamy</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="15" customHeight="1" s="18">
       <c r="A118" s="27" t="inlineStr">
@@ -44797,6 +45384,11 @@
         </is>
       </c>
       <c r="G118" s="27" t="n"/>
+      <c r="H118" s="34" t="inlineStr">
+        <is>
+          <t>fine white powder</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15" customHeight="1" s="18">
       <c r="A119" s="27" t="inlineStr">
@@ -44829,6 +45421,11 @@
         </is>
       </c>
       <c r="G119" s="27" t="n"/>
+      <c r="H119" s="34" t="inlineStr">
+        <is>
+          <t>pale, flat flakes</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="15" customHeight="1" s="18">
       <c r="A120" s="27" t="inlineStr">
@@ -44861,6 +45458,11 @@
         </is>
       </c>
       <c r="G120" s="27" t="n"/>
+      <c r="H120" s="34" t="inlineStr">
+        <is>
+          <t>pink crystals</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="15" customHeight="1" s="18">
       <c r="A121" s="27" t="inlineStr">
@@ -44893,6 +45495,11 @@
         </is>
       </c>
       <c r="G121" s="27" t="n"/>
+      <c r="H121" s="34" t="inlineStr">
+        <is>
+          <t>thin pink strands</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="15" customHeight="1" s="18">
       <c r="A122" s="27" t="inlineStr">
@@ -44925,6 +45532,11 @@
         </is>
       </c>
       <c r="G122" s="27" t="n"/>
+      <c r="H122" s="34" t="inlineStr">
+        <is>
+          <t>many-coloured strands</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15" customHeight="1" s="18">
       <c r="A123" s="27" t="inlineStr">
@@ -44957,6 +45569,11 @@
         </is>
       </c>
       <c r="G123" s="27" t="n"/>
+      <c r="H123" s="34" t="inlineStr">
+        <is>
+          <t>fine white powder</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="15" customHeight="1" s="18">
       <c r="A124" s="27" t="inlineStr">
@@ -44989,6 +45606,11 @@
         </is>
       </c>
       <c r="G124" s="27" t="n"/>
+      <c r="H124" s="34" t="inlineStr">
+        <is>
+          <t>soft pink powder</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="18">
       <c r="A125" s="27" t="inlineStr">
@@ -45021,6 +45643,11 @@
         </is>
       </c>
       <c r="G125" s="27" t="n"/>
+      <c r="H125" s="34" t="inlineStr">
+        <is>
+          <t>white crystals</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="18">
       <c r="A126" s="27" t="inlineStr">
@@ -45053,6 +45680,11 @@
         </is>
       </c>
       <c r="G126" s="27" t="n"/>
+      <c r="H126" s="34" t="inlineStr">
+        <is>
+          <t>white grains</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="15" customHeight="1" s="18">
       <c r="A127" s="27" t="inlineStr">
@@ -45085,6 +45717,11 @@
         </is>
       </c>
       <c r="G127" s="27" t="n"/>
+      <c r="H127" s="34" t="inlineStr">
+        <is>
+          <t>dark, crumbly earth</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="15" customHeight="1" s="18">
       <c r="A128" s="27" t="inlineStr">
@@ -45117,6 +45754,11 @@
         </is>
       </c>
       <c r="G128" s="27" t="n"/>
+      <c r="H128" s="34" t="inlineStr">
+        <is>
+          <t>soft grey ash</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="15" customHeight="1" s="18">
       <c r="A129" s="27" t="inlineStr">
@@ -45149,6 +45791,11 @@
         </is>
       </c>
       <c r="G129" s="27" t="n"/>
+      <c r="H129" s="34" t="inlineStr">
+        <is>
+          <t>white, thin and crushed</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="15" customHeight="1" s="18">
       <c r="A130" s="27" t="inlineStr">
@@ -45181,6 +45828,11 @@
         </is>
       </c>
       <c r="G130" s="27" t="n"/>
+      <c r="H130" s="34" t="inlineStr">
+        <is>
+          <t>a plain white block</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="15" customHeight="1" s="18">
       <c r="A131" s="27" t="inlineStr">
@@ -45213,6 +45865,11 @@
         </is>
       </c>
       <c r="G131" s="27" t="n"/>
+      <c r="H131" s="34" t="inlineStr">
+        <is>
+          <t>a black block</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="15" customHeight="1" s="18">
       <c r="A132" s="27" t="inlineStr">
@@ -45245,6 +45902,11 @@
         </is>
       </c>
       <c r="G132" s="27" t="n"/>
+      <c r="H132" s="34" t="inlineStr">
+        <is>
+          <t>gold shimmer dust</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="15" customHeight="1" s="18">
       <c r="A133" s="27" t="inlineStr">
@@ -45277,6 +45939,11 @@
         </is>
       </c>
       <c r="G133" s="27" t="n"/>
+      <c r="H133" s="34" t="inlineStr">
+        <is>
+          <t>silver shimmer dust</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="15" customHeight="1" s="18">
       <c r="A134" s="27" t="inlineStr">
@@ -45309,6 +45976,11 @@
         </is>
       </c>
       <c r="G134" s="27" t="n"/>
+      <c r="H134" s="34" t="inlineStr">
+        <is>
+          <t>silver sparkle</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="15" customHeight="1" s="18">
       <c r="A135" s="27" t="inlineStr">
@@ -45341,6 +46013,11 @@
         </is>
       </c>
       <c r="G135" s="27" t="n"/>
+      <c r="H135" s="34" t="inlineStr">
+        <is>
+          <t>pink sparkle</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="15" customHeight="1" s="18">
       <c r="A136" s="27" t="inlineStr">
@@ -45373,6 +46050,11 @@
         </is>
       </c>
       <c r="G136" s="27" t="n"/>
+      <c r="H136" s="34" t="inlineStr">
+        <is>
+          <t>many-coloured sparkle</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="15" customHeight="1" s="18">
       <c r="A137" s="27" t="inlineStr">
@@ -45405,6 +46087,11 @@
         </is>
       </c>
       <c r="G137" s="27" t="n"/>
+      <c r="H137" s="34" t="inlineStr">
+        <is>
+          <t>golden, see-through lumps</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="15" customHeight="1" s="18">
       <c r="A138" s="27" t="inlineStr">
@@ -45437,6 +46124,11 @@
         </is>
       </c>
       <c r="G138" s="27" t="n"/>
+      <c r="H138" s="34" t="inlineStr">
+        <is>
+          <t>pale yellow, sticky lumps</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="18">
       <c r="A139" s="27" t="inlineStr">
@@ -45469,6 +46161,11 @@
         </is>
       </c>
       <c r="G139" s="27" t="n"/>
+      <c r="H139" s="34" t="inlineStr">
+        <is>
+          <t>pale, milky tears of resin</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="15" customHeight="1" s="18">
       <c r="A140" s="27" t="inlineStr">
@@ -45501,6 +46198,11 @@
         </is>
       </c>
       <c r="G140" s="27" t="n"/>
+      <c r="H140" s="34" t="inlineStr">
+        <is>
+          <t>red-brown lumps of resin</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="15" customHeight="1" s="18">
       <c r="A141" s="27" t="inlineStr">
@@ -45533,6 +46235,11 @@
         </is>
       </c>
       <c r="G141" s="27" t="n"/>
+      <c r="H141" s="34" t="inlineStr">
+        <is>
+          <t>dark, crumbly leaves</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="15" customHeight="1" s="18">
       <c r="A142" s="27" t="inlineStr">
@@ -45565,6 +46272,11 @@
         </is>
       </c>
       <c r="G142" s="27" t="n"/>
+      <c r="H142" s="34" t="inlineStr">
+        <is>
+          <t>pale wood chips</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="15" customHeight="1" s="18">
       <c r="A143" s="27" t="inlineStr">
@@ -45597,6 +46309,11 @@
         </is>
       </c>
       <c r="G143" s="27" t="n"/>
+      <c r="H143" s="34" t="inlineStr">
+        <is>
+          <t>pale sea-green</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="15" customHeight="1" s="18">
       <c r="A144" s="27" t="inlineStr">
@@ -45629,6 +46346,11 @@
         </is>
       </c>
       <c r="G144" s="27" t="n"/>
+      <c r="H144" s="34" t="inlineStr">
+        <is>
+          <t>purple and pointed</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="15" customHeight="1" s="18">
       <c r="A145" s="27" t="inlineStr">
@@ -45661,6 +46383,11 @@
         </is>
       </c>
       <c r="G145" s="27" t="n"/>
+      <c r="H145" s="34" t="inlineStr">
+        <is>
+          <t>clear and sea-blue</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="15" customHeight="1" s="18">
       <c r="A146" s="27" t="inlineStr">
@@ -45693,6 +46420,11 @@
         </is>
       </c>
       <c r="G146" s="27" t="n"/>
+      <c r="H146" s="34" t="inlineStr">
+        <is>
+          <t>a stone that belongs to someone</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="15" customHeight="1" s="18">
       <c r="A147" s="27" t="inlineStr">
@@ -45725,6 +46457,11 @@
         </is>
       </c>
       <c r="G147" s="27" t="n"/>
+      <c r="H147" s="34" t="inlineStr">
+        <is>
+          <t>black and ridged</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="18">
       <c r="A148" s="27" t="inlineStr">
@@ -45757,6 +46494,11 @@
         </is>
       </c>
       <c r="G148" s="27" t="n"/>
+      <c r="H148" s="34" t="inlineStr">
+        <is>
+          <t>pale blue with soft white bands</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="15" customHeight="1" s="18">
       <c r="A149" s="27" t="inlineStr">
@@ -45789,6 +46531,11 @@
         </is>
       </c>
       <c r="G149" s="27" t="n"/>
+      <c r="H149" s="34" t="inlineStr">
+        <is>
+          <t>orange-red and glowing</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="15" customHeight="1" s="18">
       <c r="A150" s="27" t="inlineStr">
@@ -45821,6 +46568,11 @@
         </is>
       </c>
       <c r="G150" s="27" t="n"/>
+      <c r="H150" s="34" t="inlineStr">
+        <is>
+          <t>clear and honey-yellow</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="18">
       <c r="A151" s="27" t="inlineStr">
@@ -45853,6 +46605,11 @@
         </is>
       </c>
       <c r="G151" s="27" t="n"/>
+      <c r="H151" s="34" t="inlineStr">
+        <is>
+          <t>clear as ice and pointed</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="18">
       <c r="A152" s="27" t="inlineStr">
@@ -45885,6 +46642,11 @@
         </is>
       </c>
       <c r="G152" s="27" t="n"/>
+      <c r="H152" s="34" t="inlineStr">
+        <is>
+          <t>striped green and purple</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="15" customHeight="1" s="18">
       <c r="A153" s="27" t="inlineStr">
@@ -45917,6 +46679,11 @@
         </is>
       </c>
       <c r="G153" s="27" t="n"/>
+      <c r="H153" s="34" t="inlineStr">
+        <is>
+          <t>deep red</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="15" customHeight="1" s="18">
       <c r="A154" s="27" t="inlineStr">
@@ -45949,6 +46716,11 @@
         </is>
       </c>
       <c r="G154" s="27" t="n"/>
+      <c r="H154" s="34" t="inlineStr">
+        <is>
+          <t>green, with a faint sparkle</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="15" customHeight="1" s="18">
       <c r="A155" s="27" t="inlineStr">
@@ -45981,6 +46753,11 @@
         </is>
       </c>
       <c r="G155" s="27" t="n"/>
+      <c r="H155" s="34" t="inlineStr">
+        <is>
+          <t>heavy, grey and mirror-bright</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="15" customHeight="1" s="18">
       <c r="A156" s="27" t="inlineStr">
@@ -46013,6 +46790,11 @@
         </is>
       </c>
       <c r="G156" s="27" t="n"/>
+      <c r="H156" s="34" t="inlineStr">
+        <is>
+          <t>white with grey veins</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="15" customHeight="1" s="18">
       <c r="A157" s="27" t="inlineStr">
@@ -46045,6 +46827,11 @@
         </is>
       </c>
       <c r="G157" s="27" t="n"/>
+      <c r="H157" s="34" t="inlineStr">
+        <is>
+          <t>smooth and milky green</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="18">
       <c r="A158" s="27" t="inlineStr">
@@ -46077,6 +46864,11 @@
         </is>
       </c>
       <c r="G158" s="27" t="n"/>
+      <c r="H158" s="34" t="inlineStr">
+        <is>
+          <t>grey, with flashes of blue</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="15" customHeight="1" s="18">
       <c r="A159" s="27" t="inlineStr">
@@ -46109,6 +46901,11 @@
         </is>
       </c>
       <c r="G159" s="27" t="n"/>
+      <c r="H159" s="34" t="inlineStr">
+        <is>
+          <t>deep blue with gold flecks</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="15" customHeight="1" s="18">
       <c r="A160" s="27" t="inlineStr">
@@ -46141,6 +46938,11 @@
         </is>
       </c>
       <c r="G160" s="27" t="n"/>
+      <c r="H160" s="34" t="inlineStr">
+        <is>
+          <t>banded in dark and light green</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="15" customHeight="1" s="18">
       <c r="A161" s="27" t="inlineStr">
@@ -46173,6 +46975,11 @@
         </is>
       </c>
       <c r="G161" s="27" t="n"/>
+      <c r="H161" s="34" t="inlineStr">
+        <is>
+          <t>milky, with a blue glow</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="15" customHeight="1" s="18">
       <c r="A162" s="27" t="inlineStr">
@@ -46205,6 +47012,11 @@
         </is>
       </c>
       <c r="G162" s="27" t="n"/>
+      <c r="H162" s="34" t="inlineStr">
+        <is>
+          <t>clear, with green threads inside</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="15" customHeight="1" s="18">
       <c r="A163" s="27" t="inlineStr">
@@ -46237,6 +47049,11 @@
         </is>
       </c>
       <c r="G163" s="27" t="n"/>
+      <c r="H163" s="34" t="inlineStr">
+        <is>
+          <t>black and glassy</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="15" customHeight="1" s="18">
       <c r="A164" s="27" t="inlineStr">
@@ -46269,6 +47086,11 @@
         </is>
       </c>
       <c r="G164" s="27" t="n"/>
+      <c r="H164" s="34" t="inlineStr">
+        <is>
+          <t>round, creamy and lustrous</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="15" customHeight="1" s="18">
       <c r="A165" s="27" t="inlineStr">
@@ -46301,6 +47123,11 @@
         </is>
       </c>
       <c r="G165" s="27" t="n"/>
+      <c r="H165" s="34" t="inlineStr">
+        <is>
+          <t>pale bright green</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="15" customHeight="1" s="18">
       <c r="A166" s="27" t="inlineStr">
@@ -46333,6 +47160,11 @@
         </is>
       </c>
       <c r="G166" s="27" t="n"/>
+      <c r="H166" s="34" t="inlineStr">
+        <is>
+          <t>brassy gold and cube-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="15" customHeight="1" s="18">
       <c r="A167" s="27" t="inlineStr">
@@ -46365,6 +47197,11 @@
         </is>
       </c>
       <c r="G167" s="27" t="n"/>
+      <c r="H167" s="34" t="inlineStr">
+        <is>
+          <t>pink with black veins</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="15" customHeight="1" s="18">
       <c r="A168" s="27" t="inlineStr">
@@ -46397,6 +47234,11 @@
         </is>
       </c>
       <c r="G168" s="27" t="n"/>
+      <c r="H168" s="34" t="inlineStr">
+        <is>
+          <t>soft pink and cloudy</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="15" customHeight="1" s="18">
       <c r="A169" s="27" t="inlineStr">
@@ -46429,6 +47271,11 @@
         </is>
       </c>
       <c r="G169" s="27" t="n"/>
+      <c r="H169" s="34" t="inlineStr">
+        <is>
+          <t>white and silky-striped</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="15" customHeight="1" s="18">
       <c r="A170" s="27" t="inlineStr">
@@ -46461,6 +47308,11 @@
         </is>
       </c>
       <c r="G170" s="27" t="n"/>
+      <c r="H170" s="34" t="inlineStr">
+        <is>
+          <t>brown and see-through</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="15" customHeight="1" s="18">
       <c r="A171" s="27" t="inlineStr">
@@ -46493,6 +47345,11 @@
         </is>
       </c>
       <c r="G171" s="27" t="n"/>
+      <c r="H171" s="34" t="inlineStr">
+        <is>
+          <t>orange, with a glittering shimmer</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="15" customHeight="1" s="18">
       <c r="A172" s="27" t="inlineStr">
@@ -46525,6 +47382,11 @@
         </is>
       </c>
       <c r="G172" s="27" t="n"/>
+      <c r="H172" s="34" t="inlineStr">
+        <is>
+          <t>striped gold and brown</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="15" customHeight="1" s="18">
       <c r="A173" s="27" t="inlineStr">
@@ -46557,6 +47419,11 @@
         </is>
       </c>
       <c r="G173" s="27" t="n"/>
+      <c r="H173" s="34" t="inlineStr">
+        <is>
+          <t>grey, smooth and round</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="15" customHeight="1" s="18">
       <c r="A174" s="27" t="inlineStr">
@@ -46589,6 +47456,11 @@
         </is>
       </c>
       <c r="G174" s="27" t="n"/>
+      <c r="H174" s="34" t="inlineStr">
+        <is>
+          <t>tiny golden grains</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="15" customHeight="1" s="18">
       <c r="A175" s="27" t="inlineStr">
@@ -46621,6 +47493,11 @@
         </is>
       </c>
       <c r="G175" s="27" t="n"/>
+      <c r="H175" s="34" t="inlineStr">
+        <is>
+          <t>soft, white and feathery</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="15" customHeight="1" s="18">
       <c r="A176" s="27" t="inlineStr">
@@ -46653,6 +47530,11 @@
         </is>
       </c>
       <c r="G176" s="27" t="n"/>
+      <c r="H176" s="34" t="inlineStr">
+        <is>
+          <t>thin, stiff and spiky</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="15" customHeight="1" s="18">
       <c r="A177" s="27" t="inlineStr">
@@ -46685,6 +47567,11 @@
         </is>
       </c>
       <c r="G177" s="27" t="n"/>
+      <c r="H177" s="34" t="inlineStr">
+        <is>
+          <t>golden and waxy, full of little cells</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="15" customHeight="1" s="18">
       <c r="A178" s="27" t="inlineStr">
@@ -46717,6 +47604,11 @@
         </is>
       </c>
       <c r="G178" s="27" t="n"/>
+      <c r="H178" s="34" t="inlineStr">
+        <is>
+          <t>glossy black and white</t>
+        </is>
+      </c>
     </row>
     <row r="179" ht="15" customHeight="1" s="18">
       <c r="A179" s="27" t="inlineStr">
@@ -46749,6 +47641,11 @@
         </is>
       </c>
       <c r="G179" s="27" t="n"/>
+      <c r="H179" s="34" t="inlineStr">
+        <is>
+          <t>soft grey powder</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="15" customHeight="1" s="18">
       <c r="A180" s="27" t="inlineStr">
@@ -46781,6 +47678,11 @@
         </is>
       </c>
       <c r="G180" s="27" t="n"/>
+      <c r="H180" s="34" t="inlineStr">
+        <is>
+          <t>mottled brown and soft</t>
+        </is>
+      </c>
     </row>
     <row r="181" ht="15" customHeight="1" s="18">
       <c r="A181" s="27" t="inlineStr">
@@ -46813,6 +47715,11 @@
         </is>
       </c>
       <c r="G181" s="27" t="n"/>
+      <c r="H181" s="34" t="inlineStr">
+        <is>
+          <t>long, with a shimmering eye</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="15" customHeight="1" s="18">
       <c r="A182" s="27" t="inlineStr">
@@ -46845,6 +47752,11 @@
         </is>
       </c>
       <c r="G182" s="27" t="n"/>
+      <c r="H182" s="34" t="inlineStr">
+        <is>
+          <t>long, glossy and black</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="15" customHeight="1" s="18">
       <c r="A183" s="27" t="inlineStr">
@@ -46877,6 +47789,11 @@
         </is>
       </c>
       <c r="G183" s="27" t="n"/>
+      <c r="H183" s="34" t="inlineStr">
+        <is>
+          <t>pale, ridged and curled</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="15" customHeight="1" s="18">
       <c r="A184" s="27" t="inlineStr">
@@ -46909,6 +47826,11 @@
         </is>
       </c>
       <c r="G184" s="27" t="n"/>
+      <c r="H184" s="34" t="inlineStr">
+        <is>
+          <t>a single fine white hair</t>
+        </is>
+      </c>
     </row>
     <row r="185" ht="15" customHeight="1" s="18">
       <c r="A185" s="27" t="inlineStr">
@@ -46941,6 +47863,11 @@
         </is>
       </c>
       <c r="G185" s="27" t="n"/>
+      <c r="H185" s="34" t="inlineStr">
+        <is>
+          <t>papery, scaled and see-through</t>
+        </is>
+      </c>
     </row>
     <row r="186" ht="15" customHeight="1" s="18">
       <c r="A186" s="27" t="inlineStr">
@@ -46973,6 +47900,11 @@
         </is>
       </c>
       <c r="G186" s="27" t="n"/>
+      <c r="H186" s="34" t="inlineStr">
+        <is>
+          <t>small, brown and spiralled</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="15" customHeight="1" s="18">
       <c r="A187" s="27" t="inlineStr">
@@ -47005,6 +47937,11 @@
         </is>
       </c>
       <c r="G187" s="27" t="n"/>
+      <c r="H187" s="34" t="inlineStr">
+        <is>
+          <t>white and fluffy as a cloud</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="15" customHeight="1" s="18">
       <c r="A188" s="27" t="inlineStr">
@@ -47037,6 +47974,11 @@
         </is>
       </c>
       <c r="G188" s="27" t="n"/>
+      <c r="H188" s="34" t="inlineStr">
+        <is>
+          <t>small, white and feathery</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="15" customHeight="1" s="18">
       <c r="A189" s="27" t="inlineStr">
@@ -47069,6 +48011,11 @@
         </is>
       </c>
       <c r="G189" s="27" t="n"/>
+      <c r="H189" s="34" t="inlineStr">
+        <is>
+          <t>thin, brown and woven</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="15" customHeight="1" s="18">
       <c r="A190" s="27" t="inlineStr">
@@ -47101,6 +48048,11 @@
         </is>
       </c>
       <c r="G190" s="27" t="n"/>
+      <c r="H190" s="34" t="inlineStr">
+        <is>
+          <t>golden and polished</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="15" customHeight="1" s="18">
       <c r="A191" s="27" t="inlineStr">
@@ -47133,6 +48085,11 @@
         </is>
       </c>
       <c r="G191" s="27" t="n"/>
+      <c r="H191" s="34" t="inlineStr">
+        <is>
+          <t>bright and many-coloured</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="15" customHeight="1" s="18">
       <c r="A192" s="27" t="inlineStr">
@@ -47165,6 +48122,11 @@
         </is>
       </c>
       <c r="G192" s="27" t="n"/>
+      <c r="H192" s="34" t="inlineStr">
+        <is>
+          <t>small and golden</t>
+        </is>
+      </c>
     </row>
     <row r="193" ht="15" customHeight="1" s="18">
       <c r="A193" s="27" t="inlineStr">
@@ -47197,6 +48159,11 @@
         </is>
       </c>
       <c r="G193" s="27" t="n"/>
+      <c r="H193" s="34" t="inlineStr">
+        <is>
+          <t>shaped like a little heart</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="15" customHeight="1" s="18">
       <c r="A194" s="27" t="inlineStr">
@@ -47229,6 +48196,11 @@
         </is>
       </c>
       <c r="G194" s="27" t="n"/>
+      <c r="H194" s="34" t="inlineStr">
+        <is>
+          <t>odd and one of a kind</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="15" customHeight="1" s="18">
       <c r="A195" s="27" t="inlineStr">
@@ -47261,6 +48233,11 @@
         </is>
       </c>
       <c r="G195" s="27" t="n"/>
+      <c r="H195" s="34" t="inlineStr">
+        <is>
+          <t>creamy and lustrous</t>
+        </is>
+      </c>
     </row>
     <row r="196" ht="15" customHeight="1" s="18">
       <c r="A196" s="27" t="inlineStr">
@@ -47293,6 +48270,11 @@
         </is>
       </c>
       <c r="G196" s="27" t="n"/>
+      <c r="H196" s="34" t="inlineStr">
+        <is>
+          <t>small and square-cornered</t>
+        </is>
+      </c>
     </row>
     <row r="197" ht="15" customHeight="1" s="18">
       <c r="A197" s="27" t="inlineStr">
@@ -47325,6 +48307,11 @@
         </is>
       </c>
       <c r="G197" s="27" t="n"/>
+      <c r="H197" s="34" t="inlineStr">
+        <is>
+          <t>star-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="15" customHeight="1" s="18">
       <c r="A198" s="27" t="inlineStr">
@@ -47357,6 +48344,11 @@
         </is>
       </c>
       <c r="G198" s="27" t="n"/>
+      <c r="H198" s="34" t="inlineStr">
+        <is>
+          <t>old, carved and a little worn</t>
+        </is>
+      </c>
     </row>
     <row r="199" ht="15" customHeight="1" s="18">
       <c r="A199" s="27" t="inlineStr">
@@ -47389,6 +48381,11 @@
         </is>
       </c>
       <c r="G199" s="27" t="n"/>
+      <c r="H199" s="34" t="inlineStr">
+        <is>
+          <t>dark thread</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="15" customHeight="1" s="18">
       <c r="A200" s="27" t="inlineStr">
@@ -47421,6 +48418,11 @@
         </is>
       </c>
       <c r="G200" s="27" t="n"/>
+      <c r="H200" s="34" t="inlineStr">
+        <is>
+          <t>cool-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="15" customHeight="1" s="18">
       <c r="A201" s="27" t="inlineStr">
@@ -47453,6 +48455,11 @@
         </is>
       </c>
       <c r="G201" s="27" t="n"/>
+      <c r="H201" s="34" t="inlineStr">
+        <is>
+          <t>metallic thread</t>
+        </is>
+      </c>
     </row>
     <row r="202" ht="15" customHeight="1" s="18">
       <c r="A202" s="27" t="inlineStr">
@@ -47485,6 +48492,11 @@
         </is>
       </c>
       <c r="G202" s="27" t="n"/>
+      <c r="H202" s="34" t="inlineStr">
+        <is>
+          <t>cool-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="203" ht="15" customHeight="1" s="18">
       <c r="A203" s="27" t="inlineStr">
@@ -47517,6 +48529,11 @@
         </is>
       </c>
       <c r="G203" s="27" t="n"/>
+      <c r="H203" s="34" t="inlineStr">
+        <is>
+          <t>dull, soft thread</t>
+        </is>
+      </c>
     </row>
     <row r="204" ht="15" customHeight="1" s="18">
       <c r="A204" s="27" t="inlineStr">
@@ -47549,6 +48566,11 @@
         </is>
       </c>
       <c r="G204" s="27" t="n"/>
+      <c r="H204" s="34" t="inlineStr">
+        <is>
+          <t>warm-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="205" ht="15" customHeight="1" s="18">
       <c r="A205" s="27" t="inlineStr">
@@ -47581,6 +48603,11 @@
         </is>
       </c>
       <c r="G205" s="27" t="n"/>
+      <c r="H205" s="34" t="inlineStr">
+        <is>
+          <t>soft, warm-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="206" ht="15" customHeight="1" s="18">
       <c r="A206" s="27" t="inlineStr">
@@ -47613,6 +48640,11 @@
         </is>
       </c>
       <c r="G206" s="27" t="n"/>
+      <c r="H206" s="34" t="inlineStr">
+        <is>
+          <t>deep-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="207" ht="15" customHeight="1" s="18">
       <c r="A207" s="27" t="inlineStr">
@@ -47645,6 +48677,11 @@
         </is>
       </c>
       <c r="G207" s="27" t="n"/>
+      <c r="H207" s="34" t="inlineStr">
+        <is>
+          <t>many-coloured threads</t>
+        </is>
+      </c>
     </row>
     <row r="208" ht="15" customHeight="1" s="18">
       <c r="A208" s="27" t="inlineStr">
@@ -47677,6 +48714,11 @@
         </is>
       </c>
       <c r="G208" s="27" t="n"/>
+      <c r="H208" s="34" t="inlineStr">
+        <is>
+          <t>warm-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="209" ht="15" customHeight="1" s="18">
       <c r="A209" s="27" t="inlineStr">
@@ -47709,6 +48751,11 @@
         </is>
       </c>
       <c r="G209" s="27" t="n"/>
+      <c r="H209" s="34" t="inlineStr">
+        <is>
+          <t>metallic thread</t>
+        </is>
+      </c>
     </row>
     <row r="210" ht="15" customHeight="1" s="18">
       <c r="A210" s="27" t="inlineStr">
@@ -47741,6 +48788,11 @@
         </is>
       </c>
       <c r="G210" s="27" t="n"/>
+      <c r="H210" s="34" t="inlineStr">
+        <is>
+          <t>pale thread</t>
+        </is>
+      </c>
     </row>
     <row r="211" ht="15" customHeight="1" s="18">
       <c r="A211" s="27" t="inlineStr">
@@ -47773,6 +48825,11 @@
         </is>
       </c>
       <c r="G211" s="27" t="n"/>
+      <c r="H211" s="34" t="inlineStr">
+        <is>
+          <t>warm-coloured thread</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="15" customHeight="1" s="18">
       <c r="A212" s="27" t="inlineStr">
@@ -47805,6 +48862,11 @@
         </is>
       </c>
       <c r="G212" s="27" t="n"/>
+      <c r="H212" s="34" t="inlineStr">
+        <is>
+          <t>smooth and glossy</t>
+        </is>
+      </c>
     </row>
     <row r="213" ht="15" customHeight="1" s="18">
       <c r="A213" s="27" t="inlineStr">
@@ -47837,6 +48899,11 @@
         </is>
       </c>
       <c r="G213" s="27" t="n"/>
+      <c r="H213" s="34" t="inlineStr">
+        <is>
+          <t>soft, heavy and deep red</t>
+        </is>
+      </c>
     </row>
     <row r="214" ht="15" customHeight="1" s="18">
       <c r="A214" s="27" t="inlineStr">
@@ -47869,6 +48936,11 @@
         </is>
       </c>
       <c r="G214" s="27" t="n"/>
+      <c r="H214" s="34" t="inlineStr">
+        <is>
+          <t>a wooden spool, wound tight</t>
+        </is>
+      </c>
     </row>
     <row r="215" ht="15" customHeight="1" s="18">
       <c r="A215" s="27" t="inlineStr">
@@ -47901,6 +48973,11 @@
         </is>
       </c>
       <c r="G215" s="27" t="n"/>
+      <c r="H215" s="34" t="inlineStr">
+        <is>
+          <t>a little cloth bag</t>
+        </is>
+      </c>
     </row>
     <row r="216" ht="15" customHeight="1" s="18">
       <c r="A216" s="27" t="inlineStr">
@@ -47933,6 +49010,11 @@
         </is>
       </c>
       <c r="G216" s="27" t="n"/>
+      <c r="H216" s="34" t="inlineStr">
+        <is>
+          <t>a little dark, glossy bag</t>
+        </is>
+      </c>
     </row>
     <row r="217" ht="15" customHeight="1" s="18">
       <c r="A217" s="27" t="inlineStr">
@@ -47965,6 +49047,11 @@
         </is>
       </c>
       <c r="G217" s="27" t="n"/>
+      <c r="H217" s="34" t="inlineStr">
+        <is>
+          <t>thin, white and gauzy</t>
+        </is>
+      </c>
     </row>
     <row r="218" ht="15" customHeight="1" s="18">
       <c r="A218" s="27" t="inlineStr">
@@ -47997,6 +49084,11 @@
         </is>
       </c>
       <c r="G218" s="27" t="n"/>
+      <c r="H218" s="34" t="inlineStr">
+        <is>
+          <t>many-coloured scraps of cloth</t>
+        </is>
+      </c>
     </row>
     <row r="219" ht="15" customHeight="1" s="18">
       <c r="A219" s="27" t="inlineStr">
@@ -48029,6 +49121,11 @@
         </is>
       </c>
       <c r="G219" s="27" t="n"/>
+      <c r="H219" s="34" t="inlineStr">
+        <is>
+          <t>pale and straight</t>
+        </is>
+      </c>
     </row>
     <row r="220" ht="15" customHeight="1" s="18">
       <c r="A220" s="27" t="inlineStr">
@@ -48061,6 +49158,11 @@
         </is>
       </c>
       <c r="G220" s="27" t="n"/>
+      <c r="H220" s="34" t="inlineStr">
+        <is>
+          <t>pale and straight-grained</t>
+        </is>
+      </c>
     </row>
     <row r="221" ht="15" customHeight="1" s="18">
       <c r="A221" s="27" t="inlineStr">
@@ -48093,6 +49195,11 @@
         </is>
       </c>
       <c r="G221" s="27" t="n"/>
+      <c r="H221" s="34" t="inlineStr">
+        <is>
+          <t>white-barked</t>
+        </is>
+      </c>
     </row>
     <row r="222" ht="15" customHeight="1" s="18">
       <c r="A222" s="27" t="inlineStr">
@@ -48125,6 +49232,11 @@
         </is>
       </c>
       <c r="G222" s="27" t="n"/>
+      <c r="H222" s="34" t="inlineStr">
+        <is>
+          <t>white-barked</t>
+        </is>
+      </c>
     </row>
     <row r="223" ht="15" customHeight="1" s="18">
       <c r="A223" s="27" t="inlineStr">
@@ -48157,6 +49269,11 @@
         </is>
       </c>
       <c r="G223" s="27" t="n"/>
+      <c r="H223" s="34" t="inlineStr">
+        <is>
+          <t>dark and thorny</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="15" customHeight="1" s="18">
       <c r="A224" s="27" t="inlineStr">
@@ -48189,6 +49306,11 @@
         </is>
       </c>
       <c r="G224" s="27" t="n"/>
+      <c r="H224" s="34" t="inlineStr">
+        <is>
+          <t>smooth, brown and supple</t>
+        </is>
+      </c>
     </row>
     <row r="225" ht="15" customHeight="1" s="18">
       <c r="A225" s="27" t="inlineStr">
@@ -48221,6 +49343,11 @@
         </is>
       </c>
       <c r="G225" s="27" t="n"/>
+      <c r="H225" s="34" t="inlineStr">
+        <is>
+          <t>dark, heavy and rough</t>
+        </is>
+      </c>
     </row>
     <row r="226" ht="15" customHeight="1" s="18">
       <c r="A226" s="27" t="inlineStr">
@@ -48253,6 +49380,11 @@
         </is>
       </c>
       <c r="G226" s="27" t="n"/>
+      <c r="H226" s="34" t="inlineStr">
+        <is>
+          <t>slim, with red berries</t>
+        </is>
+      </c>
     </row>
     <row r="227" ht="15" customHeight="1" s="18">
       <c r="A227" s="27" t="inlineStr">
@@ -48285,6 +49417,11 @@
         </is>
       </c>
       <c r="G227" s="27" t="n"/>
+      <c r="H227" s="34" t="inlineStr">
+        <is>
+          <t>small, thin and brown</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="15" customHeight="1" s="18">
       <c r="A228" s="27" t="inlineStr">
@@ -48317,6 +49454,11 @@
         </is>
       </c>
       <c r="G228" s="27" t="n"/>
+      <c r="H228" s="34" t="inlineStr">
+        <is>
+          <t>long, thin and bendy</t>
+        </is>
+      </c>
     </row>
     <row r="229" ht="15" customHeight="1" s="18">
       <c r="A229" s="27" t="inlineStr">
@@ -48349,6 +49491,11 @@
         </is>
       </c>
       <c r="G229" s="27" t="n"/>
+      <c r="H229" s="34" t="inlineStr">
+        <is>
+          <t>pale and bendy</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="15" customHeight="1" s="18">
       <c r="A230" s="27" t="inlineStr">
@@ -48381,6 +49528,11 @@
         </is>
       </c>
       <c r="G230" s="27" t="n"/>
+      <c r="H230" s="34" t="inlineStr">
+        <is>
+          <t>flat, round and wooden</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="15" customHeight="1" s="18">
       <c r="A231" s="27" t="inlineStr">
@@ -48413,6 +49565,11 @@
         </is>
       </c>
       <c r="G231" s="27" t="n"/>
+      <c r="H231" s="34" t="inlineStr">
+        <is>
+          <t>small, brown and capped</t>
+        </is>
+      </c>
     </row>
     <row r="232" ht="15" customHeight="1" s="18">
       <c r="A232" s="27" t="inlineStr">
@@ -48445,6 +49602,11 @@
         </is>
       </c>
       <c r="G232" s="27" t="n"/>
+      <c r="H232" s="34" t="inlineStr">
+        <is>
+          <t>small, round and hinged, with a mirror</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="15" customHeight="1" s="18">
       <c r="A233" s="27" t="inlineStr">
@@ -48477,6 +49639,11 @@
         </is>
       </c>
       <c r="G233" s="27" t="n"/>
+      <c r="H233" s="34" t="inlineStr">
+        <is>
+          <t>small and hinged, with a dark mirror</t>
+        </is>
+      </c>
     </row>
     <row r="234" ht="15" customHeight="1" s="18">
       <c r="A234" s="27" t="inlineStr">
@@ -48509,6 +49676,11 @@
         </is>
       </c>
       <c r="G234" s="27" t="n"/>
+      <c r="H234" s="34" t="inlineStr">
+        <is>
+          <t>soft, grey and earthy</t>
+        </is>
+      </c>
     </row>
     <row r="235" ht="15" customHeight="1" s="18">
       <c r="A235" s="27" t="inlineStr">
@@ -48541,6 +49713,11 @@
         </is>
       </c>
       <c r="G235" s="27" t="n"/>
+      <c r="H235" s="34" t="inlineStr">
+        <is>
+          <t>small, round and metal</t>
+        </is>
+      </c>
     </row>
     <row r="236" ht="15" customHeight="1" s="18">
       <c r="A236" s="27" t="inlineStr">
@@ -48573,6 +49750,11 @@
         </is>
       </c>
       <c r="G236" s="27" t="n"/>
+      <c r="H236" s="34" t="inlineStr">
+        <is>
+          <t>flat, round and coppery</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="15" customHeight="1" s="18">
       <c r="A237" s="27" t="inlineStr">
@@ -48605,6 +49787,11 @@
         </is>
       </c>
       <c r="G237" s="27" t="n"/>
+      <c r="H237" s="34" t="inlineStr">
+        <is>
+          <t>small, round and see-through</t>
+        </is>
+      </c>
     </row>
     <row r="238" ht="15" customHeight="1" s="18">
       <c r="A238" s="27" t="inlineStr">
@@ -48637,6 +49824,11 @@
         </is>
       </c>
       <c r="G238" s="27" t="n"/>
+      <c r="H238" s="34" t="inlineStr">
+        <is>
+          <t>small, clear and stoppered</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="15" customHeight="1" s="18">
       <c r="A239" s="27" t="inlineStr">
@@ -48669,6 +49861,11 @@
         </is>
       </c>
       <c r="G239" s="27" t="n"/>
+      <c r="H239" s="34" t="inlineStr">
+        <is>
+          <t>heavy grey dust</t>
+        </is>
+      </c>
     </row>
     <row r="240" ht="15" customHeight="1" s="18">
       <c r="A240" s="27" t="inlineStr">
@@ -48701,6 +49898,11 @@
         </is>
       </c>
       <c r="G240" s="27" t="n"/>
+      <c r="H240" s="34" t="inlineStr">
+        <is>
+          <t>long, dark and metal</t>
+        </is>
+      </c>
     </row>
     <row r="241" ht="15" customHeight="1" s="18">
       <c r="A241" s="27" t="inlineStr">
@@ -48733,6 +49935,11 @@
         </is>
       </c>
       <c r="G241" s="27" t="n"/>
+      <c r="H241" s="34" t="inlineStr">
+        <is>
+          <t>thin, dark and pointed</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="15" customHeight="1" s="18">
       <c r="A242" s="27" t="inlineStr">
@@ -48765,6 +49972,11 @@
         </is>
       </c>
       <c r="G242" s="27" t="n"/>
+      <c r="H242" s="34" t="inlineStr">
+        <is>
+          <t>small, hinged, on a chain</t>
+        </is>
+      </c>
     </row>
     <row r="243" ht="15" customHeight="1" s="18">
       <c r="A243" s="27" t="inlineStr">
@@ -48797,6 +50009,11 @@
         </is>
       </c>
       <c r="G243" s="27" t="n"/>
+      <c r="H243" s="34" t="inlineStr">
+        <is>
+          <t>a few fine bristles</t>
+        </is>
+      </c>
     </row>
     <row r="244" ht="15" customHeight="1" s="18">
       <c r="A244" s="27" t="inlineStr">
@@ -48829,6 +50046,11 @@
         </is>
       </c>
       <c r="G244" s="27" t="n"/>
+      <c r="H244" s="34" t="inlineStr">
+        <is>
+          <t>plain and flat</t>
+        </is>
+      </c>
     </row>
     <row r="245" ht="15" customHeight="1" s="18">
       <c r="A245" s="27" t="inlineStr">
@@ -48861,6 +50083,11 @@
         </is>
       </c>
       <c r="G245" s="27" t="n"/>
+      <c r="H245" s="34" t="inlineStr">
+        <is>
+          <t>a long feather cut to a nib</t>
+        </is>
+      </c>
     </row>
     <row r="246" ht="15" customHeight="1" s="18">
       <c r="A246" s="27" t="inlineStr">
@@ -48893,6 +50120,11 @@
         </is>
       </c>
       <c r="G246" s="27" t="n"/>
+      <c r="H246" s="34" t="inlineStr">
+        <is>
+          <t>small, round and silver</t>
+        </is>
+      </c>
     </row>
     <row r="247" ht="15" customHeight="1" s="18">
       <c r="A247" s="27" t="inlineStr">
@@ -48925,6 +50157,11 @@
         </is>
       </c>
       <c r="G247" s="27" t="n"/>
+      <c r="H247" s="34" t="inlineStr">
+        <is>
+          <t>small and metal, with teeth</t>
+        </is>
+      </c>
     </row>
     <row r="248" ht="15" customHeight="1" s="18">
       <c r="A248" s="27" t="inlineStr">
@@ -48957,6 +50194,11 @@
         </is>
       </c>
       <c r="G248" s="27" t="n"/>
+      <c r="H248" s="34" t="inlineStr">
+        <is>
+          <t>tiny and teacup-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="249" ht="15" customHeight="1" s="18">
       <c r="A249" s="27" t="inlineStr">
@@ -48989,6 +50231,11 @@
         </is>
       </c>
       <c r="G249" s="27" t="n"/>
+      <c r="H249" s="34" t="inlineStr">
+        <is>
+          <t>tiny, metal and ringing</t>
+        </is>
+      </c>
     </row>
     <row r="250" ht="15" customHeight="1" s="18">
       <c r="A250" s="27" t="inlineStr">
@@ -49021,6 +50268,11 @@
         </is>
       </c>
       <c r="G250" s="27" t="n"/>
+      <c r="H250" s="34" t="inlineStr">
+        <is>
+          <t>a round, red blob of wax</t>
+        </is>
+      </c>
     </row>
     <row r="251" ht="15" customHeight="1" s="18">
       <c r="A251" s="27" t="inlineStr">
@@ -49053,6 +50305,11 @@
         </is>
       </c>
       <c r="G251" s="27" t="n"/>
+      <c r="H251" s="34" t="inlineStr">
+        <is>
+          <t>small, wooden and dotted</t>
+        </is>
+      </c>
     </row>
     <row r="252" ht="15" customHeight="1" s="18">
       <c r="A252" s="27" t="inlineStr">
@@ -49085,6 +50342,11 @@
         </is>
       </c>
       <c r="G252" s="27" t="n"/>
+      <c r="H252" s="34" t="inlineStr">
+        <is>
+          <t>black and wet</t>
+        </is>
+      </c>
     </row>
     <row r="253" ht="15" customHeight="1" s="18">
       <c r="A253" s="27" t="inlineStr">
@@ -49117,6 +50379,11 @@
         </is>
       </c>
       <c r="G253" s="27" t="n"/>
+      <c r="H253" s="34" t="inlineStr">
+        <is>
+          <t>shimmering gold and wet</t>
+        </is>
+      </c>
     </row>
     <row r="254" ht="15" customHeight="1" s="18">
       <c r="A254" s="27" t="inlineStr">
@@ -49149,6 +50416,11 @@
         </is>
       </c>
       <c r="G254" s="27" t="n"/>
+      <c r="H254" s="34" t="inlineStr">
+        <is>
+          <t>dark and wet</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="15" customHeight="1" s="18">
       <c r="A255" s="27" t="inlineStr">
@@ -49181,6 +50453,11 @@
         </is>
       </c>
       <c r="G255" s="27" t="n"/>
+      <c r="H255" s="34" t="inlineStr">
+        <is>
+          <t>red and wet</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="15" customHeight="1" s="18">
       <c r="A256" s="27" t="inlineStr">
@@ -49213,6 +50490,11 @@
         </is>
       </c>
       <c r="G256" s="27" t="n"/>
+      <c r="H256" s="34" t="inlineStr">
+        <is>
+          <t>shimmering silver and wet</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="15" customHeight="1" s="18">
       <c r="A257" s="27" t="inlineStr">
@@ -49245,6 +50527,11 @@
         </is>
       </c>
       <c r="G257" s="27" t="n"/>
+      <c r="H257" s="34" t="inlineStr">
+        <is>
+          <t>purple and wet</t>
+        </is>
+      </c>
     </row>
     <row r="258" ht="15" customHeight="1" s="18">
       <c r="A258" s="27" t="inlineStr">
@@ -49277,6 +50564,11 @@
         </is>
       </c>
       <c r="G258" s="27" t="n"/>
+      <c r="H258" s="34" t="inlineStr">
+        <is>
+          <t>thick and gold</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="15" customHeight="1" s="18">
       <c r="A259" s="27" t="inlineStr">
@@ -49309,6 +50601,11 @@
         </is>
       </c>
       <c r="G259" s="27" t="n"/>
+      <c r="H259" s="34" t="inlineStr">
+        <is>
+          <t>thick and red</t>
+        </is>
+      </c>
     </row>
     <row r="260" ht="15" customHeight="1" s="18"/>
     <row r="261" ht="15" customHeight="1" s="18"/>

</xml_diff>

<commit_message>
Letters name their ingredients outright
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017MKvDtcJArgibq3qMgnbMt
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -75439,7 +75439,7 @@
       <c r="N2" s="34" t="inlineStr">
         <is>
           <t>To whoever keeps the Emporium now,
-Our shelves are bare of the one herb we can't do without. You'll know the one: it stings your fingers when you pick it, and then it builds a worn-out body back up. Nothing does more for healing after a long sickness.
+Our shelves are bare of nettle, the one herb we can't do without. It stings your fingers when you pick it, and then it builds a worn-out body back up. Nothing does more for healing after a long sickness.
 I drink it myself, steeped with a little milk, after a long shift behind the counter, on the days I've looked after everyone in Wrenmoor and forgotten to look after me.
 Could you spare us a bundle or two? We'll pay in honey, as we always did.
 Agnes, Mill Lane Apothecary, Wrenmoor</t>
@@ -75511,8 +75511,8 @@
       <c r="N3" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Two orders, if you would. The bitter white crystals that draw the ache out of tired legs. Our laundry maids grate them into the soap for the towels too; they say it makes washday a proper cleansing and the hours go quicker.
-And the soft pink mud. We press it into little cakes of soap for the old gentlemen who come in after a hard day. They say nothing gives them more comfort before bed.
+Two orders, if you would. Epsom salt, the bitter white crystals that draw the ache out of tired legs. Our laundry maids grate them into the soap for the towels too; they say it makes washday a proper cleansing and the hours go quicker.
+And rose clay, the soft pink mud. We press it into little cakes of soap for the old gentlemen who come in after a hard day. They say nothing gives them more comfort before bed.
 We have been buying poor stuff from Marrowgate and the guests can tell.
 Mr Hugo Fairweather, Manager, the Halloway Baths</t>
         </is>
@@ -75567,7 +75567,7 @@
       <c r="N4" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-We grow a ruffled, sweet-smelling climber along the hive fence, the flower everyone sends when they mean thank you. When two neighbours here fall out and can't find the words to make it up, one of us brews a pot of tea with it and sits them down. It has kept friendship sweet on our lane for forty years.
+We grow sweet peas along the hive fence, the flower everyone sends when they mean thank you. When two neighbours here fall out and can't find the words to make it up, one of us brews a pot of tea with it and sits them down. It has kept friendship sweet on our lane for forty years.
 This year the frost took it. If you have dried flowers to spare, we'll pay in comb.
 Martha Hale and the Honeywell Beekeepers</t>
         </is>
@@ -75638,8 +75638,8 @@
       <c r="N5" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-The playground has turned unkind this term, and a new girl starts next week. Here the children make a chain of the little white-and-yellow field flowers for anyone new; it is how friendship starts in Cloverdale. My predecessor even burned dried ones in the classroom when tempers ran high.
-The older ones also go hunting for the plain three-leaved kind. Our school cook steeps it into a cordial on sports day, for luck.
+The playground has turned unkind this term, and a new girl starts next week. Here the children make a daisy chain for anyone new; it is how friendship starts in Cloverdale. My predecessor even burned dried ones in the classroom when tempers ran high.
+The older ones also go hunting for clover, the plain three-leaved kind. Our school cook steeps it into a cordial on sports day, for luck.
 The frost has spoilt both. Have you any dried?
 Miss Primrose Dell, Cloverdale Village School</t>
         </is>
@@ -75710,8 +75710,8 @@
       <c r="N6" s="34" t="inlineStr">
         <is>
           <t>Darling shop,
-Wedding season is upon us. My brides want the small white flowers of the citrus tree, dried and ground to a powder for their shoulders, so they shine in every photograph. Their grandmothers said a bride wearing it glows with joy.
-And for the bride who wants to walk down the aisle like a swan, a soap of the tall, still white flower. Nothing gives a quiet bride beauty like it.
+Wedding season is upon us. My brides want orange blossom, dried and ground to a powder for their shoulders, so they shine in every photograph. Their grandmothers said a bride wearing it glows with joy.
+And for the bride who wants to walk down the aisle like a swan, a soap of white lily. Nothing gives a quiet bride beauty like it.
 Send whatever you can. Kingsmere does not do things by halves.
 Lavinia, Lavinia's Bridal Rooms, Kingsmere</t>
         </is>
@@ -75766,7 +75766,7 @@
       <c r="N7" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Everyone on this stretch of coast who works nights wears a black, ridged stone on a cord, the kind that looks like a bundle of burnt matches. The lighthouse keeper has worn one for thirty years. They say it soaks up whatever is thrown at you, seen or unseen. It is the only protection I trust out there.
+Everyone on this stretch of coast who works nights wears a piece of black tourmaline on a cord. The lighthouse keeper has worn one for thirty years. They say it soaks up whatever is thrown at you, seen or unseen. It is the only protection I trust out there.
 Mine went over the side in the last storm. Could you send another?
 Officer Jory Penrose, Caldwell-on-Sea</t>
         </is>
@@ -75837,8 +75837,8 @@
       <c r="N8" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-The vicar has asked me, against my better judgement, to write. He wants the pale sweet resin from overseas. One of our widowers burns a pinch of it every evening at the same hour, and says the house fills with calm, as it did when his wife was alive.
-The vicar himself grinds the little hot black corns over his eggs. He started the week he took up painting, at sixty-one, and says it gave him the courage to make the first stroke.
+The vicar has asked me, against my better judgement, to write. He wants copal, the pale sweet resin from overseas. One of our widowers burns a pinch of it every evening at the same hour, and says the house fills with calm, as it did when his wife was alive.
+The vicar himself grinds black pepper over his eggs. He started the week he took up painting, at sixty-one, and says it gave him the courage to make the first stroke.
 Our grocer has run out of both. I trust this stays between us.
 Mr Edgar Penhallow, Churchwarden, Thornbury</t>
         </is>
@@ -75893,7 +75893,7 @@
       <c r="N9" s="34" t="inlineStr">
         <is>
           <t>Hello from the Hollow,
-When the first green shoots show after a hard winter, my aunt used to sew a little pale green stone into a cloth bag and hang it from the oldest plum tree. She said it was for the first good week of spring, and for growth. The trees never failed her.
+When the first green shoots show after a hard winter, my aunt used to sew a peridot into a cloth bag and hang it from the oldest plum tree. She said it was for the first good week of spring, and for growth. The trees never failed her.
 The bag rotted and the stone is lost in the long grass. Do you sell them?
 Bessie Damson, Plumtree Hollow</t>
         </is>
@@ -75964,8 +75964,8 @@
       <c r="N10" s="34" t="inlineStr">
         <is>
           <t>Dear neighbour,
-Two things for the winter menu. The little shrivelled dark fruit we bake into the biscuits we give children who finish their reading charts. Such a small win, but the mothers say it is pure joy to them.
-And the dark bitter powder, whipped into the spread for our Saturday buns. Ladies come in saying they really shouldn't, and then they do. Nothing is such a comfort in January.
+Two things for the winter menu. The raisins we bake into the biscuits we give children who finish their reading charts. Such a small win, but the mothers say it is pure joy to them.
+And cocoa, whipped into the spread for our Saturday buns. Ladies come in saying they really shouldn't, and then they do. Nothing is such a comfort in January.
 Our supplier in Greywater has gone bust. Could you help?
 Mrs Ada Crumb, Crumb &amp; Co., Whitcombe</t>
         </is>
@@ -76036,8 +76036,8 @@
       <c r="N11" s="34" t="inlineStr">
         <is>
           <t>Madam,
-Two old remedies my grandfather kept. The bark of the weeping tree by the river, which every grandmother uses for a sore back. Few know the old witches sewed strips of it into their pillows for intuition, and woke with the strangest pictures still in their heads.
-And the bitter silver-grey herb he steeped in a drink every New Year's Eve, to close one chapter and start the next. For transformation, he said, and not for the faint-hearted.
+Two old remedies my grandfather kept. Willow bark, which every grandmother uses for a sore back. Few know the old witches sewed strips of it into their pillows for intuition, and woke with the strangest pictures still in their heads.
+And wormwood, which he steeped in a drink every New Year's Eve, to close one chapter and start the next. For transformation, he said, and not for the faint-hearted.
 If you have either, we would pay well.
 Silas Thistle, Thistle &amp; Sons Wandwrights, Elderhollow</t>
         </is>
@@ -76092,7 +76092,7 @@
       <c r="N12" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-Travellers wait here for the coach, and the young ones fill the back room with their long games of dragons and dungeons. One old carter swears by a little carved wooden cube with dots on its faces that he had blessed at your shop. He says it gives him luck every time he throws it.
+Travellers wait here for the coach, and the young ones fill the back room with their long games of dragons and dungeons. One old carter swears by a little wooden die that he had blessed at your shop. He says it gives him luck every time he throws it.
 The young ones now want one each, for their games night. Do you still bless them?
 Harry Oakes, landlord, the Crossed Keys, Ashby Cross</t>
         </is>
@@ -76147,7 +76147,7 @@
       <c r="N13" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-Our guests come up the mountain to wait for shooting stars, and most of them can't wait for anything. Our founder tucked dried petals of the great pale water flower into a little bag under each pillow. She said the inner sight it brings is only half its use; mostly it teaches calm, and the stars come when they come.
+Our guests come up the mountain to wait for shooting stars, and most of them can't wait for anything. Our founder tucked dried lotus petals into a little bag under each pillow. She said the inner sight it brings is only half its use; mostly it teaches calm, and the stars come when they come.
 Have you any dried blooms?
 Sister Wren, the Starfall Retreat</t>
         </is>
@@ -76202,7 +76202,7 @@
       <c r="N14" s="34" t="inlineStr">
         <is>
           <t>Hello,
-My daughter can't let go of a lad who is no good for her. My mother would have braided the sharp bits clipped from her pink climbing flowers into a knotted cord and hung it by the girl's bed. She said it teaches a soft heart its boundaries.
+My daughter can't let go of a lad who is no good for her. My mother would have braided rose thorns into a knotted cord and hung it by the girl's bed. She said it teaches a soft heart its boundaries.
 I have the cord but not the thorns. Have you a jar?
 Dora Bramble, Hedge End Farm, Bramblebee</t>
         </is>
@@ -76273,8 +76273,8 @@
       <c r="N15" s="34" t="inlineStr">
         <is>
           <t>Dear shop,
-There's a girl who comes in after school who can't stop going over one silly mistake she made. Her gran used to stir the shiny pink stuff into her bath salts and say it washed in a bit of self-love.
-And the boys buy cupcakes with the little pink sugar strands on top to hand to someone they fancy, giggling all the way out. My grandmother called those love on a cake.
+There's a girl who comes in after school who can't stop going over one silly mistake she made. Her gran used to stir pink glitter into her bath salts and say it washed in a bit of self-love.
+And the boys buy cupcakes with pink sprinkles on top to hand to someone they fancy, giggling all the way out. My grandmother called those love on a cake.
 I'm out of both. I'll send fudge.
 Mrs Pennywhistle, Sugarbrook</t>
         </is>
@@ -76329,7 +76329,7 @@
       <c r="N16" s="34" t="inlineStr">
         <is>
           <t>Dear Emporium,
-Our orchard bees leave little golden grains on everything in May. The old orchard keepers beat them into butter for the fair loaves, and said whoever shares that bread with old friends shares the friendship of the hive.
+Our orchard bees leave bee pollen on everything in May. The old orchard keepers beat it into butter for the fair loaves, and said whoever shares that bread with old friends shares the friendship of the hive.
 Our hives had a bad year. Could you send a jar for the fair?
 Rhoda Bell, Cider Fair Committee, Pippin Green</t>
         </is>
@@ -76384,7 +76384,7 @@
       <c r="N17" s="34" t="inlineStr">
         <is>
           <t>Dear neighbour,
-A house clearance turned up a box of buttons, and among them one odd square one that must be a lost counter from some old board game. I left it on the counter, and the grandchildren wanted to play all afternoon. The little one swears he won every game while it sat by the board.
+A house clearance turned up a box of buttons, and among them one odd square button that must be a lost counter from some old board game. I left it on the counter, and the grandchildren wanted to play all afternoon. The little one swears he won every game while it sat by the board.
 I'll hold it for you. Come by.
 Mr Ambrose Tuck, Old Things, Buttonwick</t>
         </is>
@@ -76439,7 +76439,7 @@
       <c r="N18" s="34" t="inlineStr">
         <is>
           <t>To the Emporium,
-My mum and dad were married fifty-two years. Dad kept a corked bottle of sweet red wood shavings on the mantel, and scattered more in the drawers, until the whole mill house smelled like home. He said it kept them fond of each other through every winter.
+My mum and dad were married fifty-two years. Dad kept a corked bottle of cedar chips on the mantel, and scattered more in the drawers, until the whole mill house smelled like home. He said it kept them fond of each other through every winter.
 My wife and I could use some. Could you send a bag?
 Sam Wend, Wend Mill, Greywater</t>
         </is>

</xml_diff>

<commit_message>
Slower entrances; no logo on the day card; design document and tracker follow the no-come-back rule
The customer fades in over 1.2s and the balloon follows half a second later, floating up
over 0.8s. The dawn card shows just the day. Spellbook: making to order happens during the
visit, week-one schedule and learning chain moved (Edmund Nightfall, Rosalind Tuesday
morning, Goldie Wednesday Noon, Wayfarer's Ward Full Moon · Nightfall), Morwenna's Tobias
line and the crystal ball's colour key moved into Hester's P.S. Tracker: Wayfarer's Ward
timing, and its Learning Check row now due Day 6 (flags itself: six new parts).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ingredient_asset_tracker.xlsx
+++ b/ingredient_asset_tracker.xlsx
@@ -32984,7 +32984,7 @@
       </c>
       <c r="G22" s="22" t="inlineStr">
         <is>
-          <t>Wednesday · Twilight</t>
+          <t xml:space="preserve">Full Moon · Nightfall</t>
         </is>
       </c>
     </row>
@@ -74160,8 +74160,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="38" t="n">
-        <v>12</v>
+      <c r="A9" s="38">
+        <v>6</v>
       </c>
       <c r="B9" s="38" t="inlineStr">
         <is>
@@ -74173,11 +74173,11 @@
           <t>#21 Wayfarer's Ward</t>
         </is>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="38">
+        <v>7</v>
+      </c>
+      <c r="E9" s="38">
         <v>6</v>
-      </c>
-      <c r="E9" s="38" t="n">
-        <v>4</v>
       </c>
       <c r="F9" s="38">
         <f>D9-E9</f>

</xml_diff>